<commit_message>
Publish dashboard snapshot 2026-05-12 10:59
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>예천 감천면, 아삭하고 달콤한 '돌 토마토 ' 본격 출하</t>
+          <t>충주시, 본격 영농철 맞아 적기 모내기 돌입, 지역 특화 '중원진미' 재배...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>징글징글한 진딧물...'점 7개' 효과가 탁월합니다</t>
+          <t>횡성군, 토마토 세균병 예방 및 관리 강화</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>농우바이오 ５월 추천 품종 ‘수호 배추 ’</t>
+          <t>중동전쟁 장기화에도 영농 차질 없다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>임실군, 고추 병해충 공동방제 본격화</t>
+          <t>비료액 다시 쓰는 ‘순환식 수경재배’ 주목</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.kukinews.com</t>
+          <t>www.foodnews.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>산청군, 데이터 기반 꿀벌 월동 실험 성공…양봉산업 돌파구</t>
+          <t>농업과학원-농생명 5개 학회, 농생명 특화 거대언어모델 개발 협력</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>곡성군, '유럽채소의 기준 곡성몰 X 지티팜 기획전' 운영</t>
+          <t>오로지 '물가'뿐인 농식품부, 결국 농산물 품목별 '폐기'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>연암대 '로메인 상추 ' 도매시장 출하</t>
+          <t>아시아 종묘 "여름무 최강자 '동하무' 추천"</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.lawissue.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>논산시, 토마토뿔나방 방제사업 추진</t>
+          <t>농산물 가격 대부분 지난해보다 낮아…수급안정 대책 지속 추진</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>srn.hcn.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>소나무재선충병 매개충만 골라 잡는다… 친환경 RNAi 방제 기술 도입</t>
+          <t>군위군·경북대, 고추 탄저병 친환경 드론 방제 실증 착수</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>srn.hcn.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>과수화상병 집중관리 돌입 ‘명품 사과 재배 안정 총력’</t>
+          <t>고령 '우곡 수박 '…2026 전국 수박 품평회 금상 수상 쾌거</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[프리즘] 사우디 수출길 열었다, 날아오르는 K벌꿀</t>
+          <t>[단독]고령 우곡 수박 상표 도용한 수박 , 포항과 영덕 등 전국 유통</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>04월30일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.jibs.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>상주시, 올해 첫 모내기 시작에 풍년농사 기대감 고조</t>
+          <t>기후변화 적응...만감류 품종 개발 추진</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>cooknchefnews.com</t>
+          <t>www.breaknews.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>[서진영의 한식탐구] 봄에 먼저 만나는 마늘, 풋마늘의 계절</t>
+          <t>홍천군, 외래 해충 '토마토 뿔나방' 차단 총력… 재배 농가 방제자재 무...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>고창군, 무? 배추 뿌리혹병 및 돌발해충 방제 지원</t>
+          <t>"우수한 우리 농산물 만나보세요"…한유원, 기획전</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.sisacast.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>하이트진로, 주향미 개발 성공…농진청 국립식량과학원과 '증류식 소주...</t>
+          <t>전북농기원, 전주정원박람회서 국산 나리 정원 만들어 눈길</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.aitimes.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>충남 논산시, 토마토뿔나방 피해 예방 방제물품 지원 추진</t>
+          <t>농촌진흥청, 국가표준식품성분 데이터베이스 10.4 공개...아시아 최고 수...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.fnnews.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>제주, 고온·잦은 비에 마늘·브로콜리 병해충 비상… 농가 예찰 강화</t>
+          <t>출하량 증가·소비둔화…지역 농수산물값 하락</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월10일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.job-post.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>경북도,"채소류(고추) 출하조절시설 지원사업"공모 선정</t>
+          <t>"정원 화훼로 제격"…전북농기원, 전주정원산업박람회서 '나리' 선봬</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월09일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>news.cpbc.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>갈 곳 잃은 제주 양배추 , 분홍빛 물김치로 피어나다</t>
+          <t>5월 수박, 4월 복숭아… 더위 먹어 ‘철없는 과일’</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월09일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>서산 해미면 농가, 봄 배추 '가격 폭락'에 시름... 산지 폐기까지 검토 중</t>
+          <t>[추천제품] 팜한농 '검객'·'태풍여름무'·광분해 한번에측조'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월08일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>제주, 겨울 채소 재배의향 조사..."'수급조절로 과잉생산 차단"</t>
+          <t>생산비 치솟는데 농산물값 바닥…농가경영 손실 ‘눈덩이’</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월08일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,22 +660,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>제주도, 월동채소 파종 앞두고 재배의향 조사…여름작물 면적조사도</t>
+          <t>사람 없이도 밭갈기 ‘척척’…‘인공지능 트랙터’ 체험해보니</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월08일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>단양군, 노지 수박 조기재배 지원 대폭 확대···시장 틈새 공략으로 농...</t>
+          <t>단감 탄저병 포자 비산 첫 확인…꼼꼼한 방제 '필수'</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월07일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.newsgn.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>서부지역 밭작물 병해충 확산 우려</t>
+          <t>통영시,'한산찰옥수수'드론방제로 더 안전하게!</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월07일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>news.bbsi.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>청주시, 스마트폰 앱으로 과수화상병·돌발해충 예찰 시스템 도입</t>
+          <t>(주)경농 , 논 잡초 초종별 체계처리 제안</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>04월29일</t>
+          <t>05월07일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>전국 농산물 물가 보합세 유지</t>
+          <t>축구장 19개 규모가 온통 꽃밭으로… ‘2만2000주 장미’ 뒤덮인 국내 축...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>04월28일</t>
+          <t>05월07일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>원예작물 바이러스 옮기는 총채벌레... "예찰과 방제로 선제적 대응해야...</t>
+          <t>“엄마 사랑해” 말하자 꽃이 답했다…태안 원예치유박람회 관람객 80만...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>04월28일</t>
+          <t>05월07일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.livebiz.today</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>과수화상병 10분 만에 진단… 현장 해결형 기술 협력 본격화</t>
+          <t>'미스킴라일락'을 아시나요...국립수목원, 5월의 정원식물에 '털개회나...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>04월28일</t>
+          <t>05월07일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -849,22 +849,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>오이 재배기술&lt;44&gt;균핵병·오이 점무늬병·세균시듦병</t>
+          <t>경농 , 응애 초기 방제 맞춤형 약제 선봬</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>04월28일</t>
+          <t>05월06일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>충남 화훼 육종 기술 국제무대서 '정상' 입증</t>
+          <t>미림원예종묘, 내곡동 신사옥에서 새 시대를 열다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>04월28일</t>
+          <t>05월06일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.newscj.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>비료가격 급등에 재배 포기…글로벌 식량 생산 위협</t>
+          <t>광주, 조명1호 모내기 시연… 명품 쌀 생산 본격화</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>04월27일</t>
+          <t>05월05일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.dnews.co.kr</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>꽃, 시간을 물들이는 17일의 여정…2026고양국제꽃박람회 개막</t>
+          <t>[주간농사메모]고구마 싹 튼 후 물 조절 잘해야</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>04월27일</t>
+          <t>05월04일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>고추 농사 '정식 시기'가 반 년 농사 결정</t>
+          <t>국내 최다 1004종 장미라니... 7만 5000㎡가 10일간 붉게 물드는 '이곳'</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>04월23일</t>
+          <t>05월04일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.joongang.tv</t>
+          <t>www.newsjeju.net</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>농사의 첫 단추는 '토양 건강검진', 과학영농이 고품질 수확을 만든다</t>
+          <t>제주 토종 씨 말라...'생태계 교란 식물 퇴치' 본격 시동</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>04월23일</t>
+          <t>05월04일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,47 +1011,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 노지고추, 모판 충분한 물 줘 빼내기 쉽게 해야</t>
+          <t>고온·건조 날씨에 응애 비상, 방제전략 달라져야</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>04월22일</t>
+          <t>05월04일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>www.newsam.co.kr</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr" s="1">
-        <is>
-          <t>작물에 치명적인 바이러스, 매개충 방제가 핵심</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>04월22일</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
         <is>
           <t>(주)경농</t>
         </is>
@@ -1094,7 +1067,6 @@
     <hyperlink ref="C34" r:id="rId33"/>
     <hyperlink ref="C35" r:id="rId34"/>
     <hyperlink ref="C36" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-05-12 17:54
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,12 +93,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>충주시, 본격 영농철 맞아 적기 모내기 돌입, 지역 특화 '중원진미' 재배...</t>
+          <t>양파값 25% 급락...정부, 가격 안정 나선다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -120,12 +120,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>횡성군, 토마토 세균병 예방 및 관리 강화</t>
+          <t>경북 ‘2026 성주 참외 &amp;생명문화축제’ 5월 14일 개최</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>srn.hcn.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>중동전쟁 장기화에도 영농 차질 없다</t>
+          <t>상주시 농업기술센터, 고추 바이러스 매개충 방제 당부</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.headlinejeju.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>비료액 다시 쓰는 ‘순환식 수경재배’ 주목</t>
+          <t>제주 마늘 비료 '표준시비', 사용량 53% '대폭 절감'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.foodnews.co.kr</t>
+          <t>m.skyedaily.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농업과학원-농생명 5개 학회, 농생명 특화 거대언어모델 개발 협력</t>
+          <t>성주 참외 미래 묻다… 영농현장 세대교체 딜레마</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.jnilbo.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>오로지 '물가'뿐인 농식품부, 결국 농산물 품목별 '폐기'</t>
+          <t>함평군, 신품종 국화 '나비샛별' 품종보호권 등록</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>아시아 종묘 "여름무 최강자 '동하무' 추천"</t>
+          <t>배추· 무 ·양파 출하량 증가에 가격 뚝…농식품부, 수매비축 한달 앞당...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.headlinejeju.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 대부분 지난해보다 낮아…수급안정 대책 지속 추진</t>
+          <t>이경철 대정읍 후보 "월동채소 과잉생산 방지 위해 '농업수급 예보시스...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>srn.hcn.co.kr</t>
+          <t>www.newsjeju.net</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>군위군·경북대, 고추 탄저병 친환경 드론 방제 실증 착수</t>
+          <t>제주 솔껍질깍지벌레 "초비상"...긴급방제 3억7000만원 국비 투입</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>srn.hcn.co.kr</t>
+          <t>www.metroseoul.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>고령 '우곡 수박 '…2026 전국 수박 품평회 금상 수상 쾌거</t>
+          <t>올해 도입 '농어촌 기본소득'...읍면 소비·창업촉진 기여 사례 다수</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.foodnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[단독]고령 우곡 수박 상표 도용한 수박 , 포항과 영덕 등 전국 유통</t>
+          <t>배추· 무 2만1000톤 정부비축, 양파 1만5000톤 출하 정지…가격안정 총력</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.jibs.co.kr</t>
+          <t>www.kookje.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>기후변화 적응...만감류 품종 개발 추진</t>
+          <t>농식품부, 주요 채소 수급 불안 대비 선제 대응 나서</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.breaknews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>홍천군, 외래 해충 '토마토 뿔나방' 차단 총력… 재배 농가 방제자재 무...</t>
+          <t>저항성 해충 복합 발생에 고기능성 살충제 필요성 확대</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>"우수한 우리 농산물 만나보세요"…한유원, 기획전</t>
+          <t>아시아종묘 5월 추천품종</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>전북농기원, 전주정원박람회서 국산 나리 정원 만들어 눈길</t>
+          <t>충주시, 본격 영농철 맞아 적기 모내기 돌입, 지역 특화 '중원진미' 재배...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.aitimes.kr</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 국가표준식품성분 데이터베이스 10.4 공개...아시아 최고 수...</t>
+          <t>횡성군, 토마토 세균병 예방 및 관리 강화</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>출하량 증가·소비둔화…지역 농수산물값 하락</t>
+          <t>중동전쟁 장기화에도 영농 차질 없다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월10일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>"정원 화훼로 제격"…전북농기원, 전주정원산업박람회서 '나리' 선봬</t>
+          <t>비료액 다시 쓰는 ‘순환식 수경재배’ 주목</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월09일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.foodnews.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>5월 수박, 4월 복숭아… 더위 먹어 ‘철없는 과일’</t>
+          <t>농업과학원-농생명 5개 학회, 농생명 특화 거대언어모델 개발 협력</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월09일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[추천제품] 팜한농 '검객'·'태풍여름무'·광분해 한번에측조'</t>
+          <t>오로지 '물가'뿐인 농식품부, 결국 농산물 품목별 '폐기'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월08일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>생산비 치솟는데 농산물값 바닥…농가경영 손실 ‘눈덩이’</t>
+          <t>아시아 종묘 "여름무 최강자 '동하무' 추천"</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05월08일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,22 +660,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>사람 없이도 밭갈기 ‘척척’…‘인공지능 트랙터’ 체험해보니</t>
+          <t>농산물 가격 대부분 지난해보다 낮아…수급안정 대책 지속 추진</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05월08일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>단감 탄저병 포자 비산 첫 확인…꼼꼼한 방제 '필수'</t>
+          <t>"병해충·생리장해·노동력 부담 줄인다"… 팜한농, 5월 맞춤형 농자재...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월07일</t>
+          <t>05월09일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsgn.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>통영시,'한산찰옥수수'드론방제로 더 안전하게!</t>
+          <t>“엄마 사랑해” 말하자 꽃이 답했다…태안 원예치유박람회 관람객 80만...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.livebiz.today</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>(주)경농 , 논 잡초 초종별 체계처리 제안</t>
+          <t>'미스킴라일락'을 아시나요...국립수목원, 5월의 정원식물에 '털개회나...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>jejumbc.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>축구장 19개 규모가 온통 꽃밭으로… ‘2만2000주 장미’ 뒤덮인 국내 축...</t>
+          <t>농업에 인공지능 접목‥농가 지원사업 본격</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월07일</t>
+          <t>05월06일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>“엄마 사랑해” 말하자 꽃이 답했다…태안 원예치유박람회 관람객 80만...</t>
+          <t>경농 , 응애 초기 방제 맞춤형 약제 선봬</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월07일</t>
+          <t>05월06일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.livebiz.today</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>'미스킴라일락'을 아시나요...국립수목원, 5월의 정원식물에 '털개회나...</t>
+          <t>미림원예종묘, 내곡동 신사옥에서 새 시대를 열다</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월07일</t>
+          <t>05월06일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,22 +849,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.newscj.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>경농 , 응애 초기 방제 맞춤형 약제 선봬</t>
+          <t>광주, 조명1호 모내기 시연… 명품 쌀 생산 본격화</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월06일</t>
+          <t>05월05일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>미림원예종묘, 내곡동 신사옥에서 새 시대를 열다</t>
+          <t>[주간농사메모]고구마 싹 튼 후 물 조절 잘해야</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05월06일</t>
+          <t>05월04일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.newscj.com</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>광주, 조명1호 모내기 시연… 명품 쌀 생산 본격화</t>
+          <t>국내 최다 1004종 장미라니... 7만 5000㎡가 10일간 붉게 물드는 '이곳'</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05월05일</t>
+          <t>05월04일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.newsjeju.net</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>[주간농사메모]고구마 싹 튼 후 물 조절 잘해야</t>
+          <t>제주 토종 씨 말라...'생태계 교란 식물 퇴치' 본격 시동</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>국내 최다 1004종 장미라니... 7만 5000㎡가 10일간 붉게 물드는 '이곳'</t>
+          <t>고온·건조 날씨에 응애 비상, 방제전략 달라져야</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -971,60 +971,6 @@
         </is>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.newsjeju.net</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>제주 토종 씨 말라...'생태계 교란 식물 퇴치' 본격 시동</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>05월04일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.newsam.co.kr</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>고온·건조 날씨에 응애 비상, 방제전략 달라져야</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>05월04일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
         <is>
           <t>(주)경농</t>
         </is>
@@ -1065,8 +1011,6 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-05-13 16:39
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>양파값 25% 급락...정부, 가격 안정 나선다</t>
+          <t>[주목! 이상품] 아시아종묘 ‘동하무’, 누보 ‘누보 올코팅31’</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월13일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>경북 ‘2026 성주 참외 &amp;생명문화축제’ 5월 14일 개최</t>
+          <t>경북 포항농협, 원예모종 무상공급 나서</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월13일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>srn.hcn.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>상주시 농업기술센터, 고추 바이러스 매개충 방제 당부</t>
+          <t>배추 기계 심기 완성도 높인다… '맞춤 육묘 기술' 개발</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>제주 마늘 비료 '표준시비', 사용량 53% '대폭 절감'</t>
+          <t>양파·마늘 우수 계통 평가, 미래 품종 개발 기반 다진다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>m.skyedaily.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>성주 참외 미래 묻다… 영농현장 세대교체 딜레마</t>
+          <t>전북농기원 육성 장미, 고양국제꽃박람회서 우수성 인정</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.jnilbo.com</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>함평군, 신품종 국화 '나비샛별' 품종보호권 등록</t>
+          <t>경상국립대 이원훈 교수팀, 외래 해충 조기탐지 길 열어</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,12 +255,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>배추· 무 ·양파 출하량 증가에 가격 뚝…농식품부, 수매비축 한달 앞당...</t>
+          <t>경농 , 과수 곰팡이병 대응에 체계적 방제 제안</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -270,7 +270,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>이경철 대정읍 후보 "월동채소 과잉생산 방지 위해 '농업수급 예보시스...</t>
+          <t>" 병해충 ·생리장해·비료 부담 줄인다"… 팜한농, 5월 영농 맞춤형 제품...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newsjeju.net</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>제주 솔껍질깍지벌레 "초비상"...긴급방제 3억7000만원 국비 투입</t>
+          <t>양파값 25% 급락...정부, 가격 안정 나선다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,12 +336,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.metroseoul.co.kr</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>올해 도입 '농어촌 기본소득'...읍면 소비·창업촉진 기여 사례 다수</t>
+          <t>경북 ‘2026 성주 참외 &amp;생명문화축제’ 5월 14일 개최</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.foodnews.co.kr</t>
+          <t>srn.hcn.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>배추· 무 2만1000톤 정부비축, 양파 1만5000톤 출하 정지…가격안정 총력</t>
+          <t>상주시 농업기술센터, 고추 바이러스 매개충 방제 당부</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,12 +390,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.kookje.co.kr</t>
+          <t>www.headlinejeju.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>농식품부, 주요 채소 수급 불안 대비 선제 대응 나서</t>
+          <t>제주 마늘 비료 '표준시비', 사용량 53% '대폭 절감'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -417,12 +417,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>m.skyedaily.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>저항성 해충 복합 발생에 고기능성 살충제 필요성 확대</t>
+          <t>성주 참외 미래 묻다… 영농현장 세대교체 딜레마</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -432,7 +432,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,12 +444,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.jnilbo.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘 5월 추천품종</t>
+          <t>함평군, 신품종 국화 '나비샛별' 품종보호권 등록</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>충주시, 본격 영농철 맞아 적기 모내기 돌입, 지역 특화 '중원진미' 재배...</t>
+          <t>배추· 무 ·양파 출하량 증가에 가격 뚝…농식품부, 수매비축 한달 앞당...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.headlinejeju.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>횡성군, 토마토 세균병 예방 및 관리 강화</t>
+          <t>이경철 대정읍 후보 "월동채소 과잉생산 방지 위해 '농업수급 예보시스...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.newsjeju.net</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>중동전쟁 장기화에도 영농 차질 없다</t>
+          <t>제주 솔껍질깍지벌레 "초비상"...긴급방제 3억7000만원 국비 투입</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.metroseoul.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>비료액 다시 쓰는 ‘순환식 수경재배’ 주목</t>
+          <t>올해 도입 '농어촌 기본소득'...읍면 소비·창업촉진 기여 사례 다수</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -584,12 +584,12 @@
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>농업과학원-농생명 5개 학회, 농생명 특화 거대언어모델 개발 협력</t>
+          <t>배추· 무 2만1000톤 정부비축, 양파 1만5000톤 출하 정지…가격안정 총력</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.kookje.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>오로지 '물가'뿐인 농식품부, 결국 농산물 품목별 '폐기'</t>
+          <t>농식품부, 주요 채소 수급 불안 대비 선제 대응 나서</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>아시아 종묘 "여름무 최강자 '동하무' 추천"</t>
+          <t>저항성 해충 복합 발생에 고기능성 살충제 필요성 확대</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 대부분 지난해보다 낮아…수급안정 대책 지속 추진</t>
+          <t>아시아종묘 5월 추천품종</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>"병해충·생리장해·노동력 부담 줄인다"… 팜한농, 5월 맞춤형 농자재...</t>
+          <t>충주시, 본격 영농철 맞아 적기 모내기 돌입, 지역 특화 '중원진미' 재배...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월09일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>“엄마 사랑해” 말하자 꽃이 답했다…태안 원예치유박람회 관람객 80만...</t>
+          <t>횡성군, 토마토 세균병 예방 및 관리 강화</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월07일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.livebiz.today</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>'미스킴라일락'을 아시나요...국립수목원, 5월의 정원식물에 '털개회나...</t>
+          <t>중동전쟁 장기화에도 영농 차질 없다</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월07일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>jejumbc.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>농업에 인공지능 접목‥농가 지원사업 본격</t>
+          <t>비료액 다시 쓰는 ‘순환식 수경재배’ 주목</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월06일</t>
+          <t>05월12일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.foodnews.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>경농 , 응애 초기 방제 맞춤형 약제 선봬</t>
+          <t>농업과학원-농생명 5개 학회, 농생명 특화 거대언어모델 개발 협력</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월06일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>미림원예종묘, 내곡동 신사옥에서 새 시대를 열다</t>
+          <t>오로지 '물가'뿐인 농식품부, 결국 농산물 품목별 '폐기'</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월06일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.newscj.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>광주, 조명1호 모내기 시연… 명품 쌀 생산 본격화</t>
+          <t>아시아 종묘 "여름무 최강자 '동하무' 추천"</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월05일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>[주간농사메모]고구마 싹 튼 후 물 조절 잘해야</t>
+          <t>농산물 가격 대부분 지난해보다 낮아…수급안정 대책 지속 추진</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05월04일</t>
+          <t>05월11일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>jejumbc.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>국내 최다 1004종 장미라니... 7만 5000㎡가 10일간 붉게 물드는 '이곳'</t>
+          <t>농업에 인공지능 접목‥농가 지원사업 본격</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05월04일</t>
+          <t>05월06일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.newsjeju.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>제주 토종 씨 말라...'생태계 교란 식물 퇴치' 본격 시동</t>
+          <t>고온·건조 날씨에 응애 비상, 방제전략 달라져야</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -944,33 +944,6 @@
         </is>
       </c>
       <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.newsam.co.kr</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>고온·건조 날씨에 응애 비상, 방제전략 달라져야</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>05월04일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
         <is>
           <t>(주)경농</t>
         </is>
@@ -1010,7 +983,6 @@
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-05-21 16:43
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[주목! 이상품] 아시아종묘 ‘동하무’, 누보 ‘누보 올코팅31’</t>
+          <t>영암군 계절근로자, 농가숨통 틔인다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>05월13일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kyeonggi.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>경북 포항농협, 원예모종 무상공급 나서</t>
+          <t>화성서 올해 첫 경기도 과수화상병 발생…도농기원 “확산 차단 총력”</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05월13일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.shinailbo.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>배추 기계 심기 완성도 높인다… '맞춤 육묘 기술' 개발</t>
+          <t>순창군, 벼· 고추 재배농가 현장 기술지도 나서</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,22 +174,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.kenews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>양파·마늘 우수 계통 평가, 미래 품종 개발 기반 다진다</t>
+          <t>아시아종묘, ‘과학의 날 기념’ 부총리표창 수상</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t/>
+          <t>아시아종묘(주), 한국종묘(주)</t>
         </is>
       </c>
     </row>
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.newswhoplus.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>전북농기원 육성 장미, 고양국제꽃박람회서 우수성 인정</t>
+          <t>아프리카 바꾸는 'K-라이스벨트'… 3년 만에 종자 1만톤 돌파</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.naeil.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>경상국립대 이원훈 교수팀, 외래 해충 조기탐지 길 열어</t>
+          <t>[늘어나는 중앙아시아 인구 | 위기의 식량문제, 해결사 나선 코피아] 우...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,22 +255,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>경농 , 과수 곰팡이병 대응에 체계적 방제 제안</t>
+          <t>농산물 가격 폭락에 '산지 폐기' 도미노… 팩트로 본 수급 위기의 실상</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.sisunnews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>" 병해충 ·생리장해·비료 부담 줄인다"… 팜한농, 5월 영농 맞춤형 제품...</t>
+          <t>농업회사법인코파(주), 'SIAL 상하이 2026'서 K-파프리카 알려… 중국 시...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.cstimes.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>양파값 25% 급락...정부, 가격 안정 나선다</t>
+          <t>고유가·환율 직격탄…4월 생산자물가 2.5% 급등</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -341,17 +341,17 @@
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>경북 ‘2026 성주 참외 &amp;생명문화축제’ 5월 14일 개최</t>
+          <t>농작업 근력 보조 웨어러블 장비 개발나선 군포산업 진흥원</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월20일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>srn.hcn.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>상주시 농업기술센터, 고추 바이러스 매개충 방제 당부</t>
+          <t>농산업 유망기업, 농협과 협업해 기술 ·서비스 현장 검증한다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월20일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>www.gnmaeil.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>제주 마늘 비료 '표준시비', 사용량 53% '대폭 절감'</t>
+          <t>사천시, 21.5ha 규모 콩 채종단지 조성</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>m.skyedaily.com</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>성주 참외 미래 묻다… 영농현장 세대교체 딜레마</t>
+          <t>원주에 반복되는 과수화상병…“농가 초긴장”</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.jnilbo.com</t>
+          <t>www.cnet.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>함평군, 신품종 국화 '나비샛별' 품종보호권 등록</t>
+          <t>시그니파이, 연암대 스마트팜 허브에 LED 솔루션 적용…에너지 효율 25%...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>monthly.chosun.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>배추· 무 ·양파 출하량 증가에 가격 뚝…농식품부, 수매비축 한달 앞당...</t>
+          <t>국회의원들의 ‘농지 보유’ 현황 살펴보니… | ‘축구장 30배’ 면적 2...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>이경철 대정읍 후보 "월동채소 과잉생산 방지 위해 '농업수급 예보시스...</t>
+          <t>[수출현장을 가다] "화훼류 일본 의존도 완화 위해 대만시장 공략"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newsjeju.net</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>제주 솔껍질깍지벌레 "초비상"...긴급방제 3억7000만원 국비 투입</t>
+          <t>[단독] 국산 '과수화상병 방제제' 연내 등록 길 열렸다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.metroseoul.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>올해 도입 '농어촌 기본소득'...읍면 소비·창업촉진 기여 사례 다수</t>
+          <t>이석형 농진원장 "종자박람회 활성화···온 국민 즐기는 자리로 만들...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.foodnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>배추· 무 2만1000톤 정부비축, 양파 1만5000톤 출하 정지…가격안정 총력</t>
+          <t>"감자도 식량안보 작물"…정부 주도 '중장기 육성 전략' 시급</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.kookje.co.kr</t>
+          <t>www.newsgn.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>농식품부, 주요 채소 수급 불안 대비 선제 대응 나서</t>
+          <t>"햇양파·배추 급락 막아라"…정부, 대규모 수매·할인 총력전</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>kr.people.com.cn</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>저항성 해충 복합 발생에 고기능성 살충제 필요성 확대</t>
+          <t>생육 기간 절반 가까이 단축…‘우주 종자’, 사막서 개화 성공</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘 5월 추천품종</t>
+          <t>'5월인데 36도' 이른 고온에 농가 비상…작물 피해·병충해 속출</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>충주시, 본격 영농철 맞아 적기 모내기 돌입, 지역 특화 '중원진미' 재배...</t>
+          <t>[인터뷰-서용일 (사)한국화훼자조금협의회장] "수입꽃 연 3억 송이…국...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>횡성군, 토마토 세균병 예방 및 관리 강화</t>
+          <t>고품질 다수확을 위한 올인원 솔루션, 약알칼리성 바이오황 '황킬’</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.breaknews.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>중동전쟁 장기화에도 영농 차질 없다</t>
+          <t>경북 육성 거베라·국화, 고양국제꽃박람회 ‘2관왕’ 쾌거</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,22 +768,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>비료액 다시 쓰는 ‘순환식 수경재배’ 주목</t>
+          <t>국산 신품종 '샛별토마토', 홍콩 프리미엄 시장 오른다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월12일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t/>
+          <t>아시아종묘(주), 세계종묘(주), 한국종묘(주), (주)부농종묘</t>
         </is>
       </c>
     </row>
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.foodnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>농업과학원-농생명 5개 학회, 농생명 특화 거대언어모델 개발 협력</t>
+          <t>‘고추 바이러스병’ 미리 알고 예방해요</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>오로지 '물가'뿐인 농식품부, 결국 농산물 품목별 '폐기'</t>
+          <t>수급대책 약발 안먹히는 ‘햇양파’…“수출로 값 안정 도모하자”</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>아시아 종묘 "여름무 최강자 '동하무' 추천"</t>
+          <t>멕시코와 FTA 협상 재개 추진…농업 피해 불가피</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월19일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>jtv.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 대부분 지난해보다 낮아…수급안정 대책 지속 추진</t>
+          <t>군산시, 드론 활용 공동 방제 작업 추진</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05월11일</t>
+          <t>05월14일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>jejumbc.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>농업에 인공지능 접목‥농가 지원사업 본격</t>
+          <t>국립식량과학원, 국산 식량작물 산업화 및 현장 소통 강화</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05월06일</t>
+          <t>05월14일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,22 +930,103 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>고온·건조 날씨에 응애 비상, 방제전략 달라져야</t>
+          <t>SG한국삼공의 새로운 진딧물약 '이피콘'</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>05월04일</t>
+          <t>05월14일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>www.agrinet.co.kr</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>팜한농·아시아종묘 추천 '5월 파종 무 품종'은</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>05월14일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>www.amnews.co.kr</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>과수 농가, 고온다습한 날씨 속 '곰팡이병' 비상</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>05월13일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
           <t>(주)경농</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>www.wonyesanup.co.kr</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="1">
+        <is>
+          <t>신기술 &amp; 새상품</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>05월13일</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -983,6 +1064,9 @@
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-05-22 15:19
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.m-i.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>영암군 계절근로자, 농가숨통 틔인다</t>
+          <t>태안 청년농업인들, 수경재배로 미래 농업 이끈다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.kyeonggi.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>화성서 올해 첫 경기도 과수화상병 발생…도농기원 “확산 차단 총력”</t>
+          <t>“스마트팜·신품종 보급…품목맞춤형 접근 필요”</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.shinailbo.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>순창군, 벼· 고추 재배농가 현장 기술지도 나서</t>
+          <t>‘종자·비료·농약’ 종합 관리 효과 검증</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,22 +174,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.kenews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, ‘과학의 날 기념’ 부총리표창 수상</t>
+          <t>[한눈에 보는 시세] 양배추 , 반입량 많고 소비는 침체…‘약세늪’서 허...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>아시아종묘(주), 한국종묘(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.newswhoplus.com</t>
+          <t>www.gnmaeil.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>아프리카 바꾸는 'K-라이스벨트'… 3년 만에 종자 1만톤 돌파</t>
+          <t>이른 고온, 농가 피해 없도록 예방해야</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.naeil.com</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[늘어나는 중앙아시아 인구 | 위기의 식량문제, 해결사 나선 코피아] 우...</t>
+          <t>농산물값 안정세…배추·양파 내리고 참외·수박 강세</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,12 +255,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 폭락에 '산지 폐기' 도미노… 팩트로 본 수급 위기의 실상</t>
+          <t>호르무즈 막히자 비료값 폭등…글로벌 식량위기 “눈앞”</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.sisunnews.co.kr</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>농업회사법인코파(주), 'SIAL 상하이 2026'서 K-파프리카 알려… 중국 시...</t>
+          <t>영암군 계절근로자, 농가숨통 틔인다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.cstimes.com</t>
+          <t>www.kyeonggi.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>고유가·환율 직격탄…4월 생산자물가 2.5% 급등</t>
+          <t>화성서 올해 첫 경기도 과수화상병 발생…도농기원 “확산 차단 총력”</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,22 +336,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.shinailbo.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>농작업 근력 보조 웨어러블 장비 개발나선 군포산업 진흥원</t>
+          <t>순창군, 벼· 고추 재배농가 현장 기술지도 나서</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월20일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.kenews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>농산업 유망기업, 농협과 협업해 기술 ·서비스 현장 검증한다</t>
+          <t>아시아종묘, ‘과학의 날 기념’ 부총리표창 수상</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월20일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t>아시아종묘(주), 한국종묘(주)</t>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.gnmaeil.com</t>
+          <t>www.newswhoplus.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>사천시, 21.5ha 규모 콩 채종단지 조성</t>
+          <t>아프리카 바꾸는 'K-라이스벨트'… 3년 만에 종자 1만톤 돌파</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.naeil.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>원주에 반복되는 과수화상병…“농가 초긴장”</t>
+          <t>[늘어나는 중앙아시아 인구 | 위기의 식량문제, 해결사 나선 코피아] 우...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.cnet.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>시그니파이, 연암대 스마트팜 허브에 LED 솔루션 적용…에너지 효율 25%...</t>
+          <t>농산물 가격 폭락에 '산지 폐기' 도미노… 팩트로 본 수급 위기의 실상</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>monthly.chosun.com</t>
+          <t>www.sisunnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>국회의원들의 ‘농지 보유’ 현황 살펴보니… | ‘축구장 30배’ 면적 2...</t>
+          <t>농업회사법인코파(주), 'SIAL 상하이 2026'서 K-파프리카 알려… 중국 시...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.cstimes.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>[수출현장을 가다] "화훼류 일본 의존도 완화 위해 대만시장 공략"</t>
+          <t>고유가·환율 직격탄…4월 생산자물가 2.5% 급등</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월21일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,22 +525,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[단독] 국산 '과수화상병 방제제' 연내 등록 길 열렸다</t>
+          <t>농작업 근력 보조 웨어러블 장비 개발나선 군포산업 진흥원</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월20일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>이석형 농진원장 "종자박람회 활성화···온 국민 즐기는 자리로 만들...</t>
+          <t>농산업 유망기업, 농협과 협업해 기술 ·서비스 현장 검증한다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월20일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.cnet.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>"감자도 식량안보 작물"…정부 주도 '중장기 육성 전략' 시급</t>
+          <t>시그니파이, 연암대 스마트팜 허브에 LED 솔루션 적용…에너지 효율 25%...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>아시아종묘(주), 세계종묘(주), 한국종묘(주), (주)부농종묘</t>
+          <t>아시아종묘(주), 한국종묘(주), (주)부농종묘, 세계종묘(주)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-05-27 20:36
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.m-i.kr</t>
+          <t>www.cctimes.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>태안 청년농업인들, 수경재배로 미래 농업 이끈다</t>
+          <t>수경재배 현장활용 기술교육 추진</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.nocutnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>“스마트팜·신품종 보급…품목맞춤형 접근 필요”</t>
+          <t>증평군, 고추 양액재배 기반 구축…농가 2곳 시범 운영</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newstomato.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>‘종자·비료·농약’ 종합 관리 효과 검증</t>
+          <t>비료↓·수확↑ '스마트 이양기'…K-농기계 영토 확장도 '타진'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>[한눈에 보는 시세] 양배추 , 반입량 많고 소비는 침체…‘약세늪’서 허...</t>
+          <t>"환경제어·영농데이터·양분관리까지"…경농, 통합형 스마트농업 솔루...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.gnmaeil.com</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>이른 고온, 농가 피해 없도록 예방해야</t>
+          <t>[빨라진 폭염 시계] "금(金)추 되기 전에..." 식품·식자재 업계, 벌써 '...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>농산물값 안정세…배추·양파 내리고 참외·수박 강세</t>
+          <t>충남 공주서 과수화상병 신규 확인…농진청, 위기 단계 '주의'→'경계' ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>호르무즈 막히자 비료값 폭등…글로벌 식량위기 “눈앞”</t>
+          <t>'청정지대' 공주서 과수화상병 발생…농진청, 위기경보 '경계' 격상</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>영암군 계절근로자, 농가숨통 틔인다</t>
+          <t>성주 참외 , 일본 국민 입맛 잡는다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.kyeonggi.com</t>
+          <t>www.ekoreanews.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>화성서 올해 첫 경기도 과수화상병 발생…도농기원 “확산 차단 총력”</t>
+          <t>소나무재선충병 확산 막으려면 숲관리 방식의 전환이 필요하다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.shinailbo.co.kr</t>
+          <t>www.ziksir.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>순창군, 벼· 고추 재배농가 현장 기술지도 나서</t>
+          <t>농식품부, 농축산물 수급 점검회의 개최···"6월 이후 대파 ·수박 안정...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.kenews.co.kr</t>
+          <t>www.wowtv.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, ‘과학의 날 기념’ 부총리표창 수상</t>
+          <t>알아서 비료 뿌리고 모내기도 한번에…똑똑한 '스마트 이앙기' 개발</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>아시아종묘(주), 한국종묘(주)</t>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.newswhoplus.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>아프리카 바꾸는 'K-라이스벨트'… 3년 만에 종자 1만톤 돌파</t>
+          <t>완주 삼례농협, 명품 흑피수박 ‘블랙위너’ 본격 출하</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.naeil.com</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>[늘어나는 중앙아시아 인구 | 위기의 식량문제, 해결사 나선 코피아] 우...</t>
+          <t>성주 참외 , 일본 도쿄서 판촉전…현지 소비자 공략</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 폭락에 '산지 폐기' 도미노… 팩트로 본 수급 위기의 실상</t>
+          <t>"산업 플랫폼으로서의 엑스포, 논산 딸기의 기준을 세계로"</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.sisunnews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>농업회사법인코파(주), 'SIAL 상하이 2026'서 K-파프리카 알려… 중국 시...</t>
+          <t>아산시, 과수화상병 차단 총력… 생육기 방제약제 전 농가 무상 지원</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.cstimes.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>고유가·환율 직격탄…4월 생산자물가 2.5% 급등</t>
+          <t>충남도농기원, 딸기 우량묘 생산 현장 점검… "육묘기 관리 중요"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월21일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,22 +525,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>농작업 근력 보조 웨어러블 장비 개발나선 군포산업 진흥원</t>
+          <t>충남도농기원, 바이러스 강한 방울토마토 신품종 선보여</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월20일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>농산업 유망기업, 농협과 협업해 기술 ·서비스 현장 검증한다</t>
+          <t>충북 증평군, 시설고추 스마트 양액재배 본격 추진</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월20일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.cnet.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>시그니파이, 연암대 스마트팜 허브에 LED 솔루션 적용…에너지 효율 25%...</t>
+          <t>증평군, 고추 농사도 스마트하게... 양액재배 기반 구축 완료</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsgn.com</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>"햇양파·배추 급락 막아라"…정부, 대규모 수매·할인 총력전</t>
+          <t>양파·배추값 급락, 축산물 강세…" 수급 관리·할인지원 강화"</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>kr.people.com.cn</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>생육 기간 절반 가까이 단축…‘우주 종자’, 사막서 개화 성공</t>
+          <t>아산시, 치명적 병해 '과수화상병' 예방 총력전. 농가 부담 덜어</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>'5월인데 36도' 이른 고온에 농가 비상…작물 피해·병충해 속출</t>
+          <t>네덜란드 농업부 장관 “한국의 농업 AI 탐난다”</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>[인터뷰-서용일 (사)한국화훼자조금협의회장] "수입꽃 연 3억 송이…국...</t>
+          <t>고성군 지역 특성화 작물로 농업경쟁력 키운다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>고품질 다수확을 위한 올인원 솔루션, 약알칼리성 바이오황 '황킬’</t>
+          <t>밭농업 맞춤형 농기계 현장에 보급한다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.breaknews.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>경북 육성 거베라·국화, 고양국제꽃박람회 ‘2관왕’ 쾌거</t>
+          <t>팜한농 ‘관동여름무’ 주목</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,22 +768,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.goodkyung.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>국산 신품종 '샛별토마토', 홍콩 프리미엄 시장 오른다</t>
+          <t>리만코리아, '자이언트 병풀' 유전자 판별기술 특허…K뷰티 대표원료로...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>아시아종묘(주), 한국종묘(주), (주)부농종묘, 세계종묘(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>‘고추 바이러스병’ 미리 알고 예방해요</t>
+          <t>국립종자원, AI디지털 육종 협약…"품종개발 8년에서 3.8년으로"</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>수급대책 약발 안먹히는 ‘햇양파’…“수출로 값 안정 도모하자”</t>
+          <t>팜한농 6월 추천제품</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.handmk.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>멕시코와 FTA 협상 재개 추진…농업 피해 불가피</t>
+          <t>희소 식물로 화훼 유행을 만들어 온 30년 농장 - 농업회사법인 용오름농...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월19일</t>
+          <t>05월25일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>jtv.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>군산시, 드론 활용 공동 방제 작업 추진</t>
+          <t>포도 도둑 막으려다 발견한 살균제, 농사에 이렇게 씁니다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05월14일</t>
+          <t>05월24일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>국립식량과학원, 국산 식량작물 산업화 및 현장 소통 강화</t>
+          <t>아시아종묘, 국산 청경채 품종 '임펙트' 개발 공로 표창</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05월14일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>SG한국삼공의 새로운 진딧물약 '이피콘'</t>
+          <t>NH농우바이오, 6월 추천품종</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>05월14일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,74 +957,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>팜한농·아시아종묘 추천 '5월 파종 무 품종'은</t>
+          <t>주요 채소 낮은 시세 '여전'…전망 역시 밝지 않아</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>05월14일</t>
+          <t>05월22일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.amnews.co.kr</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>과수 농가, 고온다습한 날씨 속 '곰팡이병' 비상</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>05월13일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>(주)경농</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.wonyesanup.co.kr</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>신기술 &amp; 새상품</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>05월13일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1065,8 +1011,6 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-05-29 09:48
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.cctimes.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>수경재배 현장활용 기술교육 추진</t>
+          <t>[업체 소식] 삼례농협-NH농우바이오, '완주 삼례 수박 ' 출하 기념 행사 개...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nocutnews.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>증평군, 고추 양액재배 기반 구축…농가 2곳 시범 운영</t>
+          <t>[업체 소식] 경농, 스마트팜코리아서 통합 스마트농업 솔루션 선보여</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newstomato.com</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>비료↓·수확↑ '스마트 이양기'…K-농기계 영토 확장도 '타진'</t>
+          <t>[업체 소식] 팜한농 6월 추천 제품</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>"환경제어·영농데이터·양분관리까지"…경농, 통합형 스마트농업 솔루...</t>
+          <t>세계 곳곳서 모은 정보, 대한민국 식량안보 지킨다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>[빨라진 폭염 시계] "금(金)추 되기 전에..." 식품·식자재 업계, 벌써 '...</t>
+          <t>[AI로 읽는 경제] ④ 하나로마트엔 왜 수입농산물 논란이 끊이지 않나…...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>충남 공주서 과수화상병 신규 확인…농진청, 위기 단계 '주의'→'경계' ...</t>
+          <t>소나무재선충병 부실방제 잔혹사 끊는다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,22 +255,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>'청정지대' 공주서 과수화상병 발생…농진청, 위기경보 '경계' 격상</t>
+          <t>무측지 ‘부여뜨래’ 수박 품평회 개최</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -287,12 +287,12 @@
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>성주 참외 , 일본 국민 입맛 잡는다</t>
+          <t>노란 참외 물결 서울 도심 물들였다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ekoreanews.co.kr</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>소나무재선충병 확산 막으려면 숲관리 방식의 전환이 필요하다</t>
+          <t>깍지벌레 가득… 포항 띠녹지 병충해 의심 '비상'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.ziksir.com</t>
+          <t>www.fnnews.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>농식품부, 농축산물 수급 점검회의 개최···"6월 이후 대파 ·수박 안정...</t>
+          <t>한국산 파프리카·피망 중남미 식탁 오른다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.wowtv.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>알아서 비료 뿌리고 모내기도 한번에…똑똑한 '스마트 이앙기' 개발</t>
+          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>완주 삼례농협, 명품 흑피수박 ‘블랙위너’ 본격 출하</t>
+          <t>경제</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>성주 참외 , 일본 도쿄서 판촉전…현지 소비자 공략</t>
+          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>"산업 플랫폼으로서의 엑스포, 논산 딸기의 기준을 세계로"</t>
+          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>아산시, 과수화상병 차단 총력… 생육기 방제약제 전 농가 무상 지원</t>
+          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>충남도농기원, 딸기 우량묘 생산 현장 점검… "육묘기 관리 중요"</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>충남도농기원, 바이러스 강한 방울토마토 신품종 선보여</t>
+          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>충북 증평군, 시설고추 스마트 양액재배 본격 추진</t>
+          <t>5월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>증평군, 고추 농사도 스마트하게... 양액재배 기반 구축 완료</t>
+          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>news.knn.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>양파·배추값 급락, 축산물 강세…" 수급 관리·할인지원 강화"</t>
+          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>아산시, 치명적 병해 '과수화상병' 예방 총력전. 농가 부담 덜어</t>
+          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>네덜란드 농업부 장관 “한국의 농업 AI 탐난다”</t>
+          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.korea.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>고성군 지역 특성화 작물로 농업경쟁력 키운다</t>
+          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>밭농업 맞춤형 농기계 현장에 보급한다</t>
+          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>팜한농 ‘관동여름무’ 주목</t>
+          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.goodkyung.com</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>리만코리아, '자이언트 병풀' 유전자 판별기술 특허…K뷰티 대표원료로...</t>
+          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,12 +795,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>국립종자원, AI디지털 육종 협약…"품종개발 8년에서 3.8년으로"</t>
+          <t>고성군 지역 특성화 작물로 농업경쟁력 키운다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>팜한농 6월 추천제품</t>
+          <t>밭농업 맞춤형 농기계 현장에 보급한다</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.handmk.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>희소 식물로 화훼 유행을 만들어 온 30년 농장 - 농업회사법인 용오름농...</t>
+          <t>팜한농 ‘관동여름무’ 주목</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월25일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.goodkyung.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>포도 도둑 막으려다 발견한 살균제, 농사에 이렇게 씁니다</t>
+          <t>리만코리아, '자이언트 병풀' 유전자 판별기술 특허…K뷰티 대표원료로...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05월24일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 국산 청경채 품종 '임펙트' 개발 공로 표창</t>
+          <t>국립종자원, AI디지털 육종 협약…"품종개발 8년에서 3.8년으로"</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월26일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.handmk.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 6월 추천품종</t>
+          <t>희소 식물로 화훼 유행을 만들어 온 30년 농장 - 농업회사법인 용오름농...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월25일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,20 +957,74 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>www.ohmynews.com</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>포도 도둑 막으려다 발견한 살균제, 농사에 이렇게 씁니다</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>05월24일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>www.agrinet.co.kr</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>아시아종묘, 국산 청경채 품종 '임펙트' 개발 공로 표창</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>05월22일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>www.ikpnews.net</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr" s="1">
+      <c r="C36" t="inlineStr" s="1">
         <is>
           <t>주요 채소 낮은 시세 '여전'…전망 역시 밝지 않아</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>05월22일</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1011,6 +1065,8 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-01 10:41
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>kjmbc.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[업체 소식] 삼례농협-NH농우바이오, '완주 삼례 수박 ' 출하 기념 행사 개...</t>
+          <t>[경남] 비룟값 고공행진...재활용 농업 대안</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[업체 소식] 경농, 스마트팜코리아서 통합 스마트농업 솔루션 선보여</t>
+          <t>중동전쟁발 비료 위기…순환식 수경재배 기술로 뚫는다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[업체 소식] 팜한농 6월 추천 제품</t>
+          <t>농촌진흥청, ‘잠자던 농업기술’ 깨워 현장 실용화 추진한다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>세계 곳곳서 모은 정보, 대한민국 식량안보 지킨다</t>
+          <t>농협 종묘 ·NH농우바이오 합병 추진…종자산업계 지각변동 예고</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 하나로마트엔 왜 수입농산물 논란이 끊이지 않나…...</t>
+          <t>농사의 꽃 수확을 좌우하는 ‘탄저병’</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>소나무재선충병 부실방제 잔혹사 끊는다</t>
+          <t>한국 농정 70년사, 농민들은 어떻게 보는가</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,22 +255,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>무측지 ‘부여뜨래’ 수박 품평회 개최</t>
+          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>노란 참외 물결 서울 도심 물들였다</t>
+          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>깍지벌레 가득… 포항 띠녹지 병충해 의심 '비상'</t>
+          <t>공주 의당면서 과수화상병 발생</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.fnnews.com</t>
+          <t>www.idomin.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>한국산 파프리카·피망 중남미 식탁 오른다</t>
+          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
+          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>경제</t>
+          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
+          <t>[업체 소식] 삼례농협-NH농우바이오, '완주 삼례 수박 ' 출하 기념 행사 개...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
+          <t>[업체 소식] 경농, 스마트팜코리아서 통합 스마트농업 솔루션 선보여</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
+          <t>[업체 소식] 팜한농 6월 추천 제품</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>세계 곳곳서 모은 정보, 대한민국 식량안보 지킨다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
+          <t>[AI로 읽는 경제] ④ 하나로마트엔 왜 수입농산물 논란이 끊이지 않나…...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>5월 채소류 농업관측</t>
+          <t>소나무재선충병 부실방제 잔혹사 끊는다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
+          <t>무측지 ‘부여뜨래’ 수박 품평회 개최</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>news.knn.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
+          <t>노란 참외 물결 서울 도심 물들였다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
+          <t>깍지벌레 가득… 포항 띠녹지 병충해 의심 '비상'</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.fnnews.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
+          <t>한국산 파프리카·피망 중남미 식탁 오른다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.korea.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
+          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
+          <t>경제</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
+          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
+          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월27일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>고성군 지역 특성화 작물로 농업경쟁력 키운다</t>
+          <t>5월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>밭농업 맞춤형 농기계 현장에 보급한다</t>
+          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>팜한농 ‘관동여름무’ 주목</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.goodkyung.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>리만코리아, '자이언트 병풀' 유전자 판별기술 특허…K뷰티 대표원료로...</t>
+          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>국립종자원, AI디지털 육종 협약…"품종개발 8년에서 3.8년으로"</t>
+          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>05월26일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.handmk.com</t>
+          <t>news.knn.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>희소 식물로 화훼 유행을 만들어 온 30년 농장 - 농업회사법인 용오름농...</t>
+          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>05월25일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>포도 도둑 막으려다 발견한 살균제, 농사에 이렇게 씁니다</t>
+          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>05월24일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 국산 청경채 품종 '임펙트' 개발 공로 표창</t>
+          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,20 +1011,101 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.korea.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>주요 채소 낮은 시세 '여전'…전망 역시 밝지 않아</t>
+          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>05월22일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>www.gukjenews.com</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="1">
+        <is>
+          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>05월27일</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>www.newsam.co.kr</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="1">
+        <is>
+          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>05월27일</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>www.enewstoday.co.kr</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="1">
+        <is>
+          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>05월27일</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1067,6 +1148,9 @@
     <hyperlink ref="C34" r:id="rId33"/>
     <hyperlink ref="C35" r:id="rId34"/>
     <hyperlink ref="C36" r:id="rId35"/>
+    <hyperlink ref="C37" r:id="rId36"/>
+    <hyperlink ref="C38" r:id="rId37"/>
+    <hyperlink ref="C39" r:id="rId38"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-01 15:55
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,12 +93,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>kjmbc.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[경남] 비룟값 고공행진...재활용 농업 대안</t>
+          <t>재생에너지 잠재량· 병해충 진단…AI 공공데이터 25종 개방</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -120,12 +120,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.dailian.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>중동전쟁발 비료 위기…순환식 수경재배 기술로 뚫는다</t>
+          <t>정부, 여름철 농·수산물 특별 안전관리…비브리오균·잔류농약 집중 점...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>kjmbc.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, ‘잠자던 농업기술’ 깨워 현장 실용화 추진한다</t>
+          <t>[경남] 비룟값 고공행진...재활용 농업 대안</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>농협 종묘 ·NH농우바이오 합병 추진…종자산업계 지각변동 예고</t>
+          <t>중동전쟁발 비료 위기…순환식 수경재배 기술로 뚫는다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -206,7 +206,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농사의 꽃 수확을 좌우하는 ‘탄저병’</t>
+          <t>농촌진흥청, ‘잠자던 농업기술’ 깨워 현장 실용화 추진한다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>한국 농정 70년사, 농민들은 어떻게 보는가</t>
+          <t>농협 종묘 ·NH농우바이오 합병 추진…종자산업계 지각변동 예고</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
+          <t>농사의 꽃 수확을 좌우하는 ‘탄저병’</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
+          <t>한국 농정 70년사, 농민들은 어떻게 보는가</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>공주 의당면서 과수화상병 발생</t>
+          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,12 +336,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.idomin.com</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
+          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
+          <t>공주 의당면서 과수화상병 발생</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.idomin.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
+          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>[업체 소식] 삼례농협-NH농우바이오, '완주 삼례 수박 ' 출하 기념 행사 개...</t>
+          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,12 +444,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>[업체 소식] 경농, 스마트팜코리아서 통합 스마트농업 솔루션 선보여</t>
+          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>[업체 소식] 팜한농 6월 추천 제품</t>
+          <t>세계 곳곳서 모은 정보, 대한민국 식량안보 지킨다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>세계 곳곳서 모은 정보, 대한민국 식량안보 지킨다</t>
+          <t>[AI로 읽는 경제] ④ 하나로마트엔 왜 수입농산물 논란이 끊이지 않나…...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 하나로마트엔 왜 수입농산물 논란이 끊이지 않나…...</t>
+          <t>소나무재선충병 부실방제 잔혹사 끊는다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>소나무재선충병 부실방제 잔혹사 끊는다</t>
+          <t>무측지 ‘부여뜨래’ 수박 품평회 개최</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>무측지 ‘부여뜨래’ 수박 품평회 개최</t>
+          <t>노란 참외 물결 서울 도심 물들였다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>노란 참외 물결 서울 도심 물들였다</t>
+          <t>깍지벌레 가득… 포항 띠녹지 병충해 의심 '비상'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월28일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.fnnews.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>깍지벌레 가득… 포항 띠녹지 병충해 의심 '비상'</t>
+          <t>한국산 파프리카·피망 중남미 식탁 오른다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.fnnews.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>한국산 파프리카·피망 중남미 식탁 오른다</t>
+          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
+          <t>경제</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>경제</t>
+          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
+          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -768,12 +768,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
+          <t>5월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>5월 채소류 농업관측</t>
+          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
+          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>news.knn.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
+          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>news.knn.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
+          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
+          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,12 +984,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.korea.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
+          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1011,12 +1011,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.korea.kr</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
+          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
+          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1065,12 +1065,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="1">
         <is>
-          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
+          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1079,33 +1079,6 @@
         </is>
       </c>
       <c r="E38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>www.enewstoday.co.kr</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr" s="1">
-        <is>
-          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1150,7 +1123,6 @@
     <hyperlink ref="C36" r:id="rId35"/>
     <hyperlink ref="C37" r:id="rId36"/>
     <hyperlink ref="C38" r:id="rId37"/>
-    <hyperlink ref="C39" r:id="rId38"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-02 12:56
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.metroseoul.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>재생에너지 잠재량· 병해충 진단…AI 공공데이터 25종 개방</t>
+          <t>청송군, 스마트 사과재배 핵심장비 검증…무인방제기 현장 시연 실시</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.dailian.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름철 농·수산물 특별 안전관리…비브리오균·잔류농약 집중 점...</t>
+          <t>기후변화 대응, 폭염·가뭄 강한 배추 자원 선발한다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>kjmbc.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[경남] 비룟값 고공행진...재활용 농업 대안</t>
+          <t>농촌진흥청, ‘벼멸구 유입 예측부터 약제 처방까지’ 선제 대응</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>중동전쟁발 비료 위기…순환식 수경재배 기술로 뚫는다</t>
+          <t>6월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, ‘잠자던 농업기술’ 깨워 현장 실용화 추진한다</t>
+          <t>보석처럼 단단하고 붉은 장미처럼 매혹적인 신품종 '강적'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>농협 종묘 ·NH농우바이오 합병 추진…종자산업계 지각변동 예고</t>
+          <t>‘감튀 원조’ 벨기에, 감자값 ‘0’원…유럽 500만t 남아 “밭에 버렸...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,12 +255,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>농사의 꽃 수확을 좌우하는 ‘탄저병’</t>
+          <t>재생에너지 잠재량· 병해충 진단…AI 공공데이터 25종 개방</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.dailian.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>한국 농정 70년사, 농민들은 어떻게 보는가</t>
+          <t>정부, 여름철 농·수산물 특별 안전관리…비브리오균·잔류농약 집중 점...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>kjmbc.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
+          <t>[경남] 비룟값 고공행진...재활용 농업 대안</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
+          <t>중동전쟁발 비료 위기…순환식 수경재배 기술로 뚫는다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>공주 의당면서 과수화상병 발생</t>
+          <t>농촌진흥청, ‘잠자던 농업기술’ 깨워 현장 실용화 추진한다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.idomin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
+          <t>농협 종묘 ·NH농우바이오 합병 추진…종자산업계 지각변동 예고</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
+          <t>농사의 꽃 수확을 좌우하는 ‘탄저병’</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
+          <t>한국 농정 70년사, 농민들은 어떻게 보는가</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>세계 곳곳서 모은 정보, 대한민국 식량안보 지킨다</t>
+          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 하나로마트엔 왜 수입농산물 논란이 끊이지 않나…...</t>
+          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>소나무재선충병 부실방제 잔혹사 끊는다</t>
+          <t>공주 의당면서 과수화상병 발생</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.idomin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>무측지 ‘부여뜨래’ 수박 품평회 개최</t>
+          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>노란 참외 물결 서울 도심 물들였다</t>
+          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>깍지벌레 가득… 포항 띠녹지 병충해 의심 '비상'</t>
+          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.fnnews.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>한국산 파프리카·피망 중남미 식탁 오른다</t>
+          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
+          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>경제</t>
+          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
+          <t>5월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
+          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>5월 채소류 농업관측</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
+          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>news.knn.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
+          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
+          <t>[AI로 읽는 경제] ③ 배추· 무 ·양파는 왜 유독 비쌀까…값이 뛰는 게 아...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>news.knn.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
+          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
+          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월27일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.korea.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
+          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -984,12 +984,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.korea.kr</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
+          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1011,12 +1011,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
+          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
+          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1052,33 +1052,6 @@
         </is>
       </c>
       <c r="E37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>www.enewstoday.co.kr</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr" s="1">
-        <is>
-          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1122,7 +1095,6 @@
     <hyperlink ref="C35" r:id="rId34"/>
     <hyperlink ref="C36" r:id="rId35"/>
     <hyperlink ref="C37" r:id="rId36"/>
-    <hyperlink ref="C38" r:id="rId37"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-04 14:48
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.metroseoul.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>청송군, 스마트 사과재배 핵심장비 검증…무인방제기 현장 시연 실시</t>
+          <t>농산물 선박 수출 늘린다 ‘시에이(CA) 수출·품질 관리 프로그램’ 공...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>기후변화 대응, 폭염·가뭄 강한 배추 자원 선발한다</t>
+          <t>[AI로 읽는 경제] ⑧ 도매시장은 꼭 거쳐야 하나…없애야 할 중간단계가...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.jnilbo.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, ‘벼멸구 유입 예측부터 약제 처방까지’ 선제 대응</t>
+          <t>곡성군, 장미축제서 농특산물 3억3천만원 판매</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>6월 이달의 추천품종</t>
+          <t>5월 농축산물 소비자물가 전년대비 1.8% 상승</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>보석처럼 단단하고 붉은 장미처럼 매혹적인 신품종 '강적'</t>
+          <t>정부, 중동전쟁 장기화 속 봄철 농자재 수급 안정 총력</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>‘감튀 원조’ 벨기에, 감자값 ‘0’원…유럽 500만t 남아 “밭에 버렸...</t>
+          <t>기능성 성분 높인 쌈배추 신품종 공개…농가 현장서 상용화 가능성 점검</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>아시아종묘(주), 한국종묘(주)</t>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.dkilbo.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>재생에너지 잠재량· 병해충 진단…AI 공공데이터 25종 개방</t>
+          <t>예천군, 나만의 작은 실내 텃밭 가꾸기 교육</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.dailian.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름철 농·수산물 특별 안전관리…비브리오균·잔류농약 집중 점...</t>
+          <t>수박값 14% 뛰었다… 식탁 물가 변수로 부상한 여름 날씨</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,22 +309,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>kjmbc.co.kr</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[경남] 비룟값 고공행진...재활용 농업 대안</t>
+          <t>장기화되는 폭염에 시설하우스 차광막 각광</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)코레곤</t>
         </is>
       </c>
     </row>
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>중동전쟁발 비료 위기…순환식 수경재배 기술로 뚫는다</t>
+          <t>사과 '평면형 수형' 재배 확대···기계화 접목 속도낸다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, ‘잠자던 농업기술’ 깨워 현장 실용화 추진한다</t>
+          <t>충북 청주·음성 수박 '본격 출하'</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.dnews.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>농협 종묘 ·NH농우바이오 합병 추진…종자산업계 지각변동 예고</t>
+          <t>청송군, 과수화상병 발생 대비 모의훈련 실시</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>news.tvchosun.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>농사의 꽃 수확을 좌우하는 ‘탄저병’</t>
+          <t>'폭염 견디는 채소'…서울시, 기후 위기 대응할 품종 연구</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>한국 농정 70년사, 농민들은 어떻게 보는가</t>
+          <t>[전문가칼럼] 수확 로봇 시대, 지금 필요한 것은 '기술'이 아닌 '신뢰'다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.metroseoul.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
+          <t>청송군, 스마트 사과재배 핵심장비 검증…무인방제기 현장 시연 실시</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>공주 의당면서 과수화상병 발생</t>
+          <t>기후변화 대응, 폭염·가뭄 강한 배추 자원 선발한다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.idomin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
+          <t>농촌진흥청, ‘벼멸구 유입 예측부터 약제 처방까지’ 선제 대응</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
+          <t>6월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
+          <t>보석처럼 단단하고 붉은 장미처럼 매혹적인 신품종 '강적'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>쌀·감자·과일값 오름세…수산물은 하락 지속</t>
+          <t>‘감튀 원조’ 벨기에, 감자값 ‘0’원…유럽 500만t 남아 “밭에 버렸...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>비트 재배 기술&lt;2&gt;주요특성과 생산현황</t>
+          <t>재생에너지 잠재량· 병해충 진단…AI 공공데이터 25종 개방</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.dailian.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>'양채류 연작지 뿌리혹병 구제' 작부체계 실증 추진</t>
+          <t>정부, 여름철 농·수산물 특별 안전관리…비브리오균·잔류농약 집중 점...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>06월01일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>5월 채소류 농업관측</t>
+          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>채소류 도미노 산지폐기에 농심 '폭발'</t>
+          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>공주 의당면서 과수화상병 발생</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.idomin.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 하우스 내부 온도 30~35℃ 넘기면 수정불량 발생</t>
+          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>청주 '청원생명 수박 ' 본격 출하…고당도·GAP 앞세워 시장 공략</t>
+          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월31일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,209 +849,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>news.knn.co.kr</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>AI기반 미래 스마트농업 ‘혁신에 혁신’으로 거듭난다</t>
+          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월28일</t>
+          <t>05월29일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>www.newspim.com</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>[AI로 읽는 경제] ③ 배추· 무 ·양파는 왜 유독 비쌀까…값이 뛰는 게 아...</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>05월28일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>www.khan.co.kr</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>‘치료제 없어 걸리면 답도 없다’···사과 과수원 덮친 ‘붉은 죽음...</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>05월28일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>www.youngnong.co.kr</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="1">
-        <is>
-          <t>AI가 신품종 개발한다…국립종자원, 디지털육종 인재양성 본격화</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.korea.kr</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>[사실은 이렇습니다] 큰 일교차로 일부 노지채소 도매가격 일시 상승하...</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.gukjenews.com</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>봉화군 장군봉 소나무재선충병 발생…드론 집중 예찰 실시</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.newsam.co.kr</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>충남 공주에서 과수화상병 신규 발생 확인</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>www.enewstoday.co.kr</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr" s="1">
-        <is>
-          <t>증평군, 고추 재배에 스마트 기술 접목···생산성 향상 기대</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>05월27일</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1088,13 +899,6 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-08 10:10
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -98,12 +98,12 @@
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>농산물 선박 수출 늘린다 ‘시에이(CA) 수출·품질 관리 프로그램’ 공...</t>
+          <t>미생물 기반 농업 바이오 소재 “이제 현장에서 효과 입증”</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑧ 도매시장은 꼭 거쳐야 하나…없애야 할 중간단계가...</t>
+          <t>[기고] 평년이 사라진 밭농업, 병해충 ·잡초관리도 달라져야</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.jnilbo.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>곡성군, 장미축제서 농특산물 3억3천만원 판매</t>
+          <t>[Issue+] 스마트팜의 현재와 미래를 보다 - 2026 스마트팜코리아</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.newstnt.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>5월 농축산물 소비자물가 전년대비 1.8% 상승</t>
+          <t>충남농업기술원, 국화 '백야' 베트남 진출...전용실시 계약 체결</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>정부, 중동전쟁 장기화 속 봄철 농자재 수급 안정 총력</t>
+          <t>‘괴산 배추 ’ 대만 수출 가속도 붙는다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>기능성 성분 높인 쌈배추 신품종 공개…농가 현장서 상용화 가능성 점검</t>
+          <t>가락 쉬자 전국 도매시장 들썩…휴업 도미노 오나</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>아시아종묘(주), 한국종묘(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.dkilbo.com</t>
+          <t>www.hani.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>예천군, 나만의 작은 실내 텃밭 가꾸기 교육</t>
+          <t>‘과수 괴질’ 과수 화상병 전국 확산…충북 등 전국 78농가 발병</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월07일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.jibs.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>수박값 14% 뛰었다… 식탁 물가 변수로 부상한 여름 날씨</t>
+          <t>여름철 고온에도 안정적 생산...쪽파 신 품종 개발</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월07일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,22 +309,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>장기화되는 폭염에 시설하우스 차광막 각광</t>
+          <t>도심 수직농장서 딸기 생산...베이커리 카페서 전부 소화</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월07일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(주)코레곤</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.joongboo.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>사과 '평면형 수형' 재배 확대···기계화 접목 속도낸다</t>
+          <t>이천대월농협, 이천쌀의 뿌리 '자채쌀' 복원 나섰다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월07일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.kmib.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>충북 청주·음성 수박 '본격 출하'</t>
+          <t>‘여름금파’ ‘해찬이’… 고온에 강한 신품종 선발 박차</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월07일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.dnews.co.kr</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>청송군, 과수화상병 발생 대비 모의훈련 실시</t>
+          <t>충남 육성 국화 ‘백야’, 베트남 등 글로벌 시장 공략 본격화</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월07일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>news.tvchosun.com</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>'폭염 견디는 채소'…서울시, 기후 위기 대응할 품종 연구</t>
+          <t>"상추 싸질 줄 알았는데"…밥상 채소값 다시 '꿈틀' [권 기자의 장바구...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월06일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>[전문가칼럼] 수확 로봇 시대, 지금 필요한 것은 '기술'이 아닌 '신뢰'다</t>
+          <t>NH농우바이오·팜한농 6월 추천 품종은</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월05일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,22 +471,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>아시아종묘, 항암·지방간억제 쌈채소 선보여</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월05일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t/>
+          <t>아시아종묘(주)</t>
         </is>
       </c>
     </row>
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.metroseoul.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>청송군, 스마트 사과재배 핵심장비 검증…무인방제기 현장 시연 실시</t>
+          <t>[AI로 읽는 경제] ⑨ 온라인도매시장은 진짜 유통거품을 빼고 있나…성...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월05일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.greened.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>기후변화 대응, 폭염·가뭄 강한 배추 자원 선발한다</t>
+          <t>고물가 속 빛난 토마토…제철 농산물에 쏠리는 소비자들</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, ‘벼멸구 유입 예측부터 약제 처방까지’ 선제 대응</t>
+          <t>농사포인트 - 노지고추, 쓰러지지 않도록 지주대 보강 단단히 묶어</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>6월 이달의 추천품종</t>
+          <t>"기후변화· 수입 증가 대응 서류 산업 정책 필요"</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>보석처럼 단단하고 붉은 장미처럼 매혹적인 신품종 '강적'</t>
+          <t>농산물 선박 수출 늘린다 ‘시에이(CA) 수출·품질 관리 프로그램’ 공...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>‘감튀 원조’ 벨기에, 감자값 ‘0’원…유럽 500만t 남아 “밭에 버렸...</t>
+          <t>[AI로 읽는 경제] ⑧ 도매시장은 꼭 거쳐야 하나…없애야 할 중간단계가...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.jnilbo.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>재생에너지 잠재량· 병해충 진단…AI 공공데이터 25종 개방</t>
+          <t>곡성군, 장미축제서 농특산물 3억3천만원 판매</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월04일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.dailian.co.kr</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름철 농·수산물 특별 안전관리…비브리오균·잔류농약 집중 점...</t>
+          <t>5월 농축산물 소비자물가 전년대비 1.8% 상승</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월01일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>음성군, 대표 농특산물 '다올찬 수박 ' 본격 출하</t>
+          <t>정부, 중동전쟁 장기화 속 봄철 농자재 수급 안정 총력</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>‘허락 없는 이삭줍기는 절도’ 현수막…감자·양파 등 수확기 농촌에 ...</t>
+          <t>기능성 성분 높인 쌈배추 신품종 공개…농가 현장서 상용화 가능성 점검</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t/>
+          <t>아시아종묘(주), 한국종묘(주)</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.dkilbo.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>공주 의당면서 과수화상병 발생</t>
+          <t>예천군, 나만의 작은 실내 텃밭 가꾸기 교육</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.idomin.com</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>봄철 출하 공백에 날씨 변덕까지…대파 등 채소류 가격 오름세</t>
+          <t>수박값 14% 뛰었다… 식탁 물가 변수로 부상한 여름 날씨</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월03일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>양채류 병해충 경감 재배 매뉴얼 제작 배포</t>
+          <t>장기화되는 폭염에 시설하우스 차광막 각광</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>05월31일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)코레곤</t>
         </is>
       </c>
     </row>
@@ -849,20 +849,155 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>'딸기 농사 성패 가르는 6월'... 충남도, 우량 자묘 생산 집중 관리</t>
+          <t>사과 '평면형 수형' 재배 확대···기계화 접목 속도낸다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>05월29일</t>
+          <t>06월02일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>www.agrinet.co.kr</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>충북 청주·음성 수박 '본격 출하'</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>06월02일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>www.dnews.co.kr</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="1">
+        <is>
+          <t>청송군, 과수화상병 발생 대비 모의훈련 실시</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>06월02일</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>news.tvchosun.com</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="1">
+        <is>
+          <t>'폭염 견디는 채소'…서울시, 기후 위기 대응할 품종 연구</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>06월02일</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>www.newsfarm.co.kr</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>[전문가칼럼] 수확 로봇 시대, 지금 필요한 것은 '기술'이 아닌 '신뢰'다</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>06월02일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>한국농업기술진흥원</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>www.dynews.co.kr</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>주간농사정보</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>06월02일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -899,6 +1034,11 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
+    <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-15 09:55
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.bzeronews.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>미생물 기반 농업 바이오 소재 “이제 현장에서 효과 입증”</t>
+          <t>'탄저병 비상·농지 전수조사 착수'…옥천군, 여름 농정 현장 점검 강화</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -125,12 +125,12 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[기고] 평년이 사라진 밭농업, 병해충 ·잡초관리도 달라져야</t>
+          <t>[afl Interview] 류재영 아시아종묘 부사장</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -152,17 +152,17 @@
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 스마트팜의 현재와 미래를 보다 - 2026 스마트팜코리아</t>
+          <t>[기획] 고온다습한 여름 예고에 탄저병 '비상'…단계적 방제 필요</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,22 +174,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.newstnt.com</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>충남농업기술원, 국화 '백야' 베트남 진출...전용실시 계약 체결</t>
+          <t>'2026 농업기술 박람회' 청주오스코서 18일 개막</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -206,12 +206,12 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>‘괴산 배추 ’ 대만 수출 가속도 붙는다</t>
+          <t>[일본 도매시장, 경계를 허물다] 저장·소분·가공·배송까지…무한 변...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>가락 쉬자 전국 도매시장 들썩…휴업 도미노 오나</t>
+          <t>희귀식물 불법으로 심고 파는 ‘식테크’ 기승</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>‘과수 괴질’ 과수 화상병 전국 확산…충북 등 전국 78농가 발병</t>
+          <t>배추 1포기 평균 3656원… 한 달 새 11% 올라</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월07일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.jibs.co.kr</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>여름철 고온에도 안정적 생산...쪽파 신 품종 개발</t>
+          <t>축구장 100개 면적 밭 초토화… 우박에 농심도 멍들었다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월07일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>도심 수직농장서 딸기 생산...베이커리 카페서 전부 소화</t>
+          <t>“ 배추 수확 앞두고 쑥대밭” 강원농가 덮친 우박 피해 속출</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월07일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.joongboo.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>이천대월농협, 이천쌀의 뿌리 '자채쌀' 복원 나섰다</t>
+          <t>'공동영농', 초고령화·지역소멸위기 농촌의 최적 대안일까?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월07일</t>
+          <t>06월14일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.kmib.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>‘여름금파’ ‘해찬이’… 고온에 강한 신품종 선발 박차</t>
+          <t>시금치 가격 18% 상승… 여름철 앞두고 ‘채소값 들썩’</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월07일</t>
+          <t>06월14일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>충남 육성 국화 ‘백야’, 베트남 등 글로벌 시장 공략 본격화</t>
+          <t>토양생태환경보전사업으로 제주 밭작물 휴경·작물전환 유도</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월07일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>"상추 싸질 줄 알았는데"…밥상 채소값 다시 '꿈틀' [권 기자의 장바구...</t>
+          <t>[풍경] 달콤한 여름 시작…영동 양산 수박 출하 한창</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월06일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오·팜한농 6월 추천 품종은</t>
+          <t>시설하우스 ‘천장 환기창’ 달아 폭염 극복</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월05일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,22 +471,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 항암·지방간억제 쌈채소 선보여</t>
+          <t>영월군, 솔잎혹파리 방제사업 착수... 건강한 산림자원 보호</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월05일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>아시아종묘(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑨ 온라인도매시장은 진짜 유통거품을 빼고 있나…성...</t>
+          <t>타 지역 참외 의 '성주 참외 ' 둔갑 정황 포착… 농민들 "박스갈이 의심" [...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월05일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.greened.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>고물가 속 빛난 토마토…제철 농산물에 쏠리는 소비자들</t>
+          <t>바이러스 병 확산 우려, 매개충 관리 중요성 확대</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.domin.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 노지고추, 쓰러지지 않도록 지주대 보강 단단히 묶어</t>
+          <t>올여름도 피할 수 없는 '히트플레이션' 식탁물가 또 들썩이나</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>"기후변화· 수입 증가 대응 서류 산업 정책 필요"</t>
+          <t>[포토] 롯데百, 초고당도 ‘춘천 하니원 메론 ’ 맛보세요</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>news.bbsi.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>농산물 선박 수출 늘린다 ‘시에이(CA) 수출·품질 관리 프로그램’ 공...</t>
+          <t>[경제 오딧세이]aT, 사계절 딸기 생산에 본격 나선다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑧ 도매시장은 꼭 거쳐야 하나…없애야 할 중간단계가...</t>
+          <t>2030년까지 민간정원 360곳·지방정원 48곳 더 조성한다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.jnilbo.com</t>
+          <t>www.sisaweek.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>곡성군, 장미축제서 농특산물 3억3천만원 판매</t>
+          <t>이상기후, 우리 식탁 물가도 '이상'해진다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월04일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>5월 농축산물 소비자물가 전년대비 1.8% 상승</t>
+          <t>경기도농업기술원, 장마철 고추·사과 탄저병 주의보 발령</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.etnews.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>정부, 중동전쟁 장기화 속 봄철 농자재 수급 안정 총력</t>
+          <t>권대규 전북대 교수팀, 농작업 근력보조 웨어러블 로봇 추진</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.gjdream.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>기능성 성분 높인 쌈배추 신품종 공개…농가 현장서 상용화 가능성 점검</t>
+          <t>곡성, 멜론 할인전ㆍ가루쌀 특허…농산물 경쟁력 강화</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>아시아종묘(주), 한국종묘(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.dkilbo.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>예천군, 나만의 작은 실내 텃밭 가꾸기 교육</t>
+          <t>농사포인트 - 양파, 망에 담아 통풍 잘되고 직사광선 피하는 곳 보관</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월10일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>수박값 14% 뛰었다… 식탁 물가 변수로 부상한 여름 날씨</t>
+          <t>“하나로 통한다!” 수출농산물 농약안전사용 지침 ‘정보무늬’ 고도...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월03일</t>
+          <t>06월09일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>장기화되는 폭염에 시설하우스 차광막 각광</t>
+          <t>중국 햇양파에 밀리는 국산 저장양파...“우수품종 보급·저장기술 고도...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월09일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>(주)코레곤</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>사과 '평면형 수형' 재배 확대···기계화 접목 속도낸다</t>
+          <t>홍성서 올해 첫 과수화상병 발생</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>충북 청주·음성 수박 '본격 출하'</t>
+          <t>영양, 2026년산 홍 고추 수매약정 체결</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.dnews.co.kr</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>청송군, 과수화상병 발생 대비 모의훈련 실시</t>
+          <t>[주간농사메모]노지고추 강풍·폭우 대비</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>news.tvchosun.com</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>'폭염 견디는 채소'…서울시, 기후 위기 대응할 품종 연구</t>
+          <t>경주시, 조사료 국산화 승부수...트리티케일 신계통 '화랑 1호' 발굴</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,47 +957,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>[전문가칼럼] 수확 로봇 시대, 지금 필요한 것은 '기술'이 아닌 '신뢰'다</t>
+          <t>포도 노균병 방제, 바이엘크롭사이언스 ‘시바나’로 초기부터 꽉</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월02일</t>
+          <t>06월08일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t>한국농업기술진흥원</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.dynews.co.kr</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>주간농사정보</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>06월02일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1038,7 +1011,6 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-16 14:39
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.bzeronews.com</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>'탄저병 비상·농지 전수조사 착수'…옥천군, 여름 농정 현장 점검 강화</t>
+          <t>강원도, 우박 피해 농가 지원 위해 보험 가입 촉진</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[afl Interview] 류재영 아시아종묘 부사장</t>
+          <t>장마철 노지 고추 '칼슘결핍·탄저병' 방제해야</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[기획] 고온다습한 여름 예고에 탄저병 '비상'…단계적 방제 필요</t>
+          <t>장마철 앞두고 고추·사과 탄저병 주의보… 포장 관리·방제 유의해야</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>'2026 농업기술 박람회' 청주오스코서 18일 개막</t>
+          <t>“7분 내내 쏟아졌어요”…때아닌 우박에 농가 ‘울상’</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -189,7 +189,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -206,7 +206,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>[일본 도매시장, 경계를 허물다] 저장·소분·가공·배송까지…무한 변...</t>
+          <t>제주, 남도마늘 약세에 재고까지 ‘답답’…“깐마늘 수급조절 가이드...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.ntoday.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>희귀식물 불법으로 심고 파는 ‘식테크’ 기승</t>
+          <t>[TN 현장] 멸종위기 식물의 마지막 보루, 알파인하우스·시드볼트에 가...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,12 +255,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.dailian.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>배추 1포기 평균 3656원… 한 달 새 11% 올라</t>
+          <t>농진청 “장마철 고추 칼슘결핍·탄저병 주의해야”</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.bokuennews.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>축구장 100개 면적 밭 초토화… 우박에 농심도 멍들었다</t>
+          <t>소량 씨앗도 식물검역증명서 필수</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.fsnews.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>“ 배추 수확 앞두고 쑥대밭” 강원농가 덮친 우박 피해 속출</t>
+          <t>여름 식탁 물가 엇갈려</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.bzeronews.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>'공동영농', 초고령화·지역소멸위기 농촌의 최적 대안일까?</t>
+          <t>'탄저병 비상·농지 전수조사 착수'…옥천군, 여름 농정 현장 점검 강화</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월14일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>시금치 가격 18% 상승… 여름철 앞두고 ‘채소값 들썩’</t>
+          <t>[afl Interview] 류재영 아시아종묘 부사장</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월14일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -395,12 +395,12 @@
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>토양생태환경보전사업으로 제주 밭작물 휴경·작물전환 유도</t>
+          <t>[기획] 고온다습한 여름 예고에 탄저병 '비상'…단계적 방제 필요</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>[풍경] 달콤한 여름 시작…영동 양산 수박 출하 한창</t>
+          <t>'2026 농업기술 박람회' 청주오스코서 18일 개막</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -449,12 +449,12 @@
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>시설하우스 ‘천장 환기창’ 달아 폭염 극복</t>
+          <t>[일본 도매시장, 경계를 허물다] 저장·소분·가공·배송까지…무한 변...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>영월군, 솔잎혹파리 방제사업 착수... 건강한 산림자원 보호</t>
+          <t>희귀식물 불법으로 심고 파는 ‘식테크’ 기승</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>타 지역 참외 의 '성주 참외 ' 둔갑 정황 포착… 농민들 "박스갈이 의심" [...</t>
+          <t>배추 1포기 평균 3656원… 한 달 새 11% 올라</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>바이러스 병 확산 우려, 매개충 관리 중요성 확대</t>
+          <t>축구장 100개 면적 밭 초토화… 우박에 농심도 멍들었다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.domin.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>올여름도 피할 수 없는 '히트플레이션' 식탁물가 또 들썩이나</t>
+          <t>“ 배추 수확 앞두고 쑥대밭” 강원농가 덮친 우박 피해 속출</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>[포토] 롯데百, 초고당도 ‘춘천 하니원 메론 ’ 맛보세요</t>
+          <t>'공동영농', 초고령화·지역소멸위기 농촌의 최적 대안일까?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월14일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>news.bbsi.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[경제 오딧세이]aT, 사계절 딸기 생산에 본격 나선다</t>
+          <t>시금치 가격 18% 상승… 여름철 앞두고 ‘채소값 들썩’</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월14일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>2030년까지 민간정원 360곳·지방정원 48곳 더 조성한다</t>
+          <t>토양생태환경보전사업으로 제주 밭작물 휴경·작물전환 유도</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.sisaweek.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>이상기후, 우리 식탁 물가도 '이상'해진다</t>
+          <t>[풍경] 달콤한 여름 시작…영동 양산 수박 출하 한창</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 장마철 고추·사과 탄저병 주의보 발령</t>
+          <t>시설하우스 ‘천장 환기창’ 달아 폭염 극복</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.etnews.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>권대규 전북대 교수팀, 농작업 근력보조 웨어러블 로봇 추진</t>
+          <t>영월군, 솔잎혹파리 방제사업 착수... 건강한 산림자원 보호</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월12일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.gjdream.com</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>곡성, 멜론 할인전ㆍ가루쌀 특허…농산물 경쟁력 강화</t>
+          <t>타 지역 참외 의 '성주 참외 ' 둔갑 정황 포착… 농민들 "박스갈이 의심" [...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 양파, 망에 담아 통풍 잘되고 직사광선 피하는 곳 보관</t>
+          <t>바이러스 병 확산 우려, 매개충 관리 중요성 확대</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월10일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.domin.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>“하나로 통한다!” 수출농산물 농약안전사용 지침 ‘정보무늬’ 고도...</t>
+          <t>올여름도 피할 수 없는 '히트플레이션' 식탁물가 또 들썩이나</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월09일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>중국 햇양파에 밀리는 국산 저장양파...“우수품종 보급·저장기술 고도...</t>
+          <t>[포토] 롯데百, 초고당도 ‘춘천 하니원 메론 ’ 맛보세요</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월09일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>홍성서 올해 첫 과수화상병 발생</t>
+          <t>영양, 2026년산 홍 고추 수매약정 체결</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>영양, 2026년산 홍 고추 수매약정 체결</t>
+          <t>[주간농사메모]노지고추 강풍·폭우 대비</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>[주간농사메모]노지고추 강풍·폭우 대비</t>
+          <t>경주시, 조사료 국산화 승부수...트리티케일 신계통 '화랑 1호' 발굴</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -917,60 +917,6 @@
         </is>
       </c>
       <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>www.hidomin.com</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="1">
-        <is>
-          <t>경주시, 조사료 국산화 승부수...트리티케일 신계통 '화랑 1호' 발굴</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>06월08일</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.newsam.co.kr</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>포도 노균병 방제, 바이엘크롭사이언스 ‘시바나’로 초기부터 꽉</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>06월08일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1009,8 +955,6 @@
     <hyperlink ref="C30" r:id="rId29"/>
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-18 14:55
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>강원도, 우박 피해 농가 지원 위해 보험 가입 촉진</t>
+          <t>진천군, 중소형 수박 브랜드 '소과담' 전시회 성료</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>장마철 노지 고추 '칼슘결핍·탄저병' 방제해야</t>
+          <t>안성시, 기후변화 대응 찰옥수수 품종 선발 연구 추진</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>장마철 앞두고 고추·사과 탄저병 주의보… 포장 관리·방제 유의해야</t>
+          <t>‘농지 전수조사’ 후폭풍…십여년 키워온 ‘친환경쌀 단지’ 와해되나</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>“7분 내내 쏟아졌어요”…때아닌 우박에 농가 ‘울상’</t>
+          <t>폭염에 채소도 녹는다…농산물 가격 '껑충'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.cctimes.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>제주, 남도마늘 약세에 재고까지 ‘답답’…“깐마늘 수급조절 가이드...</t>
+          <t>풍년에 가격 폭락 … 양파농가 시름</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.ntoday.co.kr</t>
+          <t>biz.heraldcorp.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[TN 현장] 멸종위기 식물의 마지막 보루, 알파인하우스·시드볼트에 가...</t>
+          <t>참외·딸기 키웠더니 농가소득 6.5배…지역특화작목 효과 입증</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.dailian.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>농진청 “장마철 고추 칼슘결핍·탄저병 주의해야”</t>
+          <t>‘국산 유기 풋거름 종자 ’ 생산, 보급 확대 첫걸음</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.bokuennews.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>소량 씨앗도 식물검역증명서 필수</t>
+          <t>정부, 배추· 무 3만 4천t 확보…신선란 3천만 개 수입 추진</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.fsnews.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>여름 식탁 물가 엇갈려</t>
+          <t>"폭 줄이고 통풍 극대화"... 신개념 시설하우스 농가 보급 시동</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.bzeronews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>'탄저병 비상·농지 전수조사 착수'…옥천군, 여름 농정 현장 점검 강화</t>
+          <t>농사포인트 - 바이러스 전염 차단 … 묘판 주위 방충망 촘촘히 피복</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[afl Interview] 류재영 아시아종묘 부사장</t>
+          <t>신젠타코리아 인시피오®, 주요 수출국 MRL 기준 충족</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>신젠타코리아(주)</t>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>[기획] 고온다습한 여름 예고에 탄저병 '비상'…단계적 방제 필요</t>
+          <t>6월 과채류 농업관측</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>'2026 농업기술 박람회' 청주오스코서 18일 개막</t>
+          <t>채소 병해충의 모든 것</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>[일본 도매시장, 경계를 허물다] 저장·소분·가공·배송까지…무한 변...</t>
+          <t>2026년 하반기 주목해야할 농기자재</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>희귀식물 불법으로 심고 파는 ‘식테크’ 기승</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>배추 1포기 평균 3656원… 한 달 새 11% 올라</t>
+          <t>장마철 고추농사 성패, 탄저병 예방에 달렸다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>축구장 100개 면적 밭 초토화… 우박에 농심도 멍들었다</t>
+          <t>강원도, 우박 피해 농가 지원 위해 보험 가입 촉진</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>“ 배추 수확 앞두고 쑥대밭” 강원농가 덮친 우박 피해 속출</t>
+          <t>장마철 노지 고추 '칼슘결핍·탄저병' 방제해야</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>'공동영농', 초고령화·지역소멸위기 농촌의 최적 대안일까?</t>
+          <t>고온다습한 장마철, 고추 칼슘결핍증·탄저병 예방 철저히</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월14일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>시금치 가격 18% 상승… 여름철 앞두고 ‘채소값 들썩’</t>
+          <t>장마철 앞두고 고추·사과 탄저병 주의보… 포장 관리·방제 유의해야</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월14일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>토양생태환경보전사업으로 제주 밭작물 휴경·작물전환 유도</t>
+          <t>“7분 내내 쏟아졌어요”…때아닌 우박에 농가 ‘울상’</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>[풍경] 달콤한 여름 시작…영동 양산 수박 출하 한창</t>
+          <t>제주, 남도마늘 약세에 재고까지 ‘답답’…“깐마늘 수급조절 가이드...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ntoday.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>시설하우스 ‘천장 환기창’ 달아 폭염 극복</t>
+          <t>[TN 현장] 멸종위기 식물의 마지막 보루, 알파인하우스·시드볼트에 가...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.bokuennews.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>영월군, 솔잎혹파리 방제사업 착수... 건강한 산림자원 보호</t>
+          <t>소량 씨앗도 식물검역증명서 필수</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월12일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.fsnews.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>타 지역 참외 의 '성주 참외 ' 둔갑 정황 포착… 농민들 "박스갈이 의심" [...</t>
+          <t>여름 식탁 물가 엇갈려</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월15일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,12 +768,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>바이러스 병 확산 우려, 매개충 관리 중요성 확대</t>
+          <t>타 지역 참외 의 '성주 참외 ' 둔갑 정황 포착… 농민들 "박스갈이 의심" [...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -795,12 +795,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.domin.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>올여름도 피할 수 없는 '히트플레이션' 식탁물가 또 들썩이나</t>
+          <t>바이러스 병 확산 우려, 매개충 관리 중요성 확대</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.domin.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>[포토] 롯데百, 초고당도 ‘춘천 하니원 메론 ’ 맛보세요</t>
+          <t>올여름도 피할 수 없는 '히트플레이션' 식탁물가 또 들썩이나</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,74 +849,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>영양, 2026년산 홍 고추 수매약정 체결</t>
+          <t>[포토] 롯데百, 초고당도 ‘춘천 하니원 메론 ’ 맛보세요</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월08일</t>
+          <t>06월11일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>www.gnnews.co.kr</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>[주간농사메모]노지고추 강풍·폭우 대비</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>06월08일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>www.hidomin.com</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>경주시, 조사료 국산화 승부수...트리티케일 신계통 '화랑 1호' 발굴</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>06월08일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -953,8 +899,6 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-22 10:29
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>진천군, 중소형 수박 브랜드 '소과담' 전시회 성료</t>
+          <t>[글로벌 특징주] 인플레 새 복병 '슈퍼 엘니뇨'…투자 대응법은</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>안성시, 기후변화 대응 찰옥수수 품종 선발 연구 추진</t>
+          <t>화사하고 재배 쉬운 ‘국산 나리’ 현장에서 경쟁력 살핀다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.goodkyung.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>‘농지 전수조사’ 후폭풍…십여년 키워온 ‘친환경쌀 단지’ 와해되나</t>
+          <t>유럽은 왜 유전자편집 작물의 문을 열었나</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>폭염에 채소도 녹는다…농산물 가격 '껑충'</t>
+          <t>[AFL칼럼] 농업기술박람회, 연구성과를 농업인의 기술로</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.cctimes.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>풍년에 가격 폭락 … 양파농가 시름</t>
+          <t>참외 수확하는 로봇 '참독'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>biz.heraldcorp.com</t>
+          <t>biz.chosun.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>참외·딸기 키웠더니 농가소득 6.5배…지역특화작목 효과 입증</t>
+          <t>[위성 관측 리포트] 한 포기 ‘2만원’ 고랭지 배추 가격 이면에는… 재...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>‘국산 유기 풋거름 종자 ’ 생산, 보급 확대 첫걸음</t>
+          <t>7~9월 ‘가락시장 배추 경매’ 22시 시작</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.jejunews.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>정부, 배추· 무 3만 4천t 확보…신선란 3천만 개 수입 추진</t>
+          <t>비료값 폭등 "농가 한숨 깊어진다"</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월21일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>"폭 줄이고 통풍 극대화"... 신개념 시설하우스 농가 보급 시동</t>
+          <t>이른 더위에…풋고추·토마토 가격 뛰어</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월21일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 바이러스 전염 차단 … 묘판 주위 방충망 촘촘히 피복</t>
+          <t>고랭지 여름배추 불청객 '반쪽시들음병'···미생물 퇴비로 고민 끝</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>신젠타코리아 인시피오®, 주요 수출국 MRL 기준 충족</t>
+          <t>日, 농산물 신 품종 보호 강화…韓中 '무단유출' 염두</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>신젠타코리아(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>6월 과채류 농업관측</t>
+          <t>고환율에 히트플레이션, 역대급 장마까지⋯빨간불 켜진 ‘여름 물가’[...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>채소 병해충의 모든 것</t>
+          <t>[요즘 이기술] 장마철 고추 병해 예방하려면…땅 적정 산성도 유지·통...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>2026년 하반기 주목해야할 농기자재</t>
+          <t>신젠타 인시피오Ⓡ, 미국·대만·일본에 등록 완료</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t>신젠타코리아(주)</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>진천군, 중소형 수박 브랜드 '소과담' 전시회 성료</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.viva100.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>장마철 고추농사 성패, 탄저병 예방에 달렸다</t>
+          <t>안성시, 기후변화 대응 찰옥수수 품종 선발 연구 추진</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>강원도, 우박 피해 농가 지원 위해 보험 가입 촉진</t>
+          <t>‘농지 전수조사’ 후폭풍…십여년 키워온 ‘친환경쌀 단지’ 와해되나</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>장마철 노지 고추 '칼슘결핍·탄저병' 방제해야</t>
+          <t>폭염에 채소도 녹는다…농산물 가격 '껑충'</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.cctimes.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>고온다습한 장마철, 고추 칼슘결핍증·탄저병 예방 철저히</t>
+          <t>풍년에 가격 폭락 … 양파농가 시름</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>biz.heraldcorp.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>장마철 앞두고 고추·사과 탄저병 주의보… 포장 관리·방제 유의해야</t>
+          <t>참외·딸기 키웠더니 농가소득 6.5배…지역특화작목 효과 입증</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>“7분 내내 쏟아졌어요”…때아닌 우박에 농가 ‘울상’</t>
+          <t>‘국산 유기 풋거름 종자 ’ 생산, 보급 확대 첫걸음</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>제주, 남도마늘 약세에 재고까지 ‘답답’…“깐마늘 수급조절 가이드...</t>
+          <t>정부, 배추· 무 3만 4천t 확보…신선란 3천만 개 수입 추진</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.ntoday.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>[TN 현장] 멸종위기 식물의 마지막 보루, 알파인하우스·시드볼트에 가...</t>
+          <t>"폭 줄이고 통풍 극대화"... 신개념 시설하우스 농가 보급 시동</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.bokuennews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>소량 씨앗도 식물검역증명서 필수</t>
+          <t>신젠타코리아 인시피오®, 주요 수출국 MRL 기준 충족</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t/>
+          <t>신젠타코리아(주)</t>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.fsnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>여름 식탁 물가 엇갈려</t>
+          <t>농사포인트 - 바이러스 전염 차단 … 묘판 주위 방충망 촘촘히 피복</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>타 지역 참외 의 '성주 참외 ' 둔갑 정황 포착… 농민들 "박스갈이 의심" [...</t>
+          <t>6월 과채류 농업관측</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>바이러스 병 확산 우려, 매개충 관리 중요성 확대</t>
+          <t>채소 병해충의 모든 것</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.domin.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>올여름도 피할 수 없는 '히트플레이션' 식탁물가 또 들썩이나</t>
+          <t>2026년 하반기 주목해야할 농기자재</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -849,20 +849,101 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>[포토] 롯데百, 초고당도 ‘춘천 하니원 메론 ’ 맛보세요</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월11일</t>
+          <t>06월16일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>www.farmnmarket.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>장마철 고추농사 성패, 탄저병 예방에 달렸다</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>06월16일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>www.bokuennews.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="1">
+        <is>
+          <t>소량 씨앗도 식물검역증명서 필수</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>06월15일</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>www.fsnews.co.kr</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="1">
+        <is>
+          <t>여름 식탁 물가 엇갈려</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>06월15일</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -899,6 +980,9 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
+    <hyperlink ref="C33" r:id="rId32"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-24 14:36
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -98,12 +98,12 @@
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[글로벌 특징주] 인플레 새 복병 '슈퍼 엘니뇨'…투자 대응법은</t>
+          <t>[AI로 읽는 경제] ③ 세계 2위 농식품 수출국의 비밀...네덜란드는 왜 바...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>화사하고 재배 쉬운 ‘국산 나리’ 현장에서 경쟁력 살핀다</t>
+          <t>군위군, 여름철 엽채류 실증재배 추진</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.goodkyung.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>유럽은 왜 유전자편집 작물의 문을 열었나</t>
+          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,22 +174,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>[AFL칼럼] 농업기술박람회, 연구성과를 농업인의 기술로</t>
+          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.queen.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>참외 수확하는 로봇 '참독'</t>
+          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>biz.chosun.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[위성 관측 리포트] 한 포기 ‘2만원’ 고랭지 배추 가격 이면에는… 재...</t>
+          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>7~9월 ‘가락시장 배추 경매’ 22시 시작</t>
+          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.jejunews.com</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>비료값 폭등 "농가 한숨 깊어진다"</t>
+          <t>부정농약 주의보… 농산물 안정성 우려</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월21일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>이른 더위에…풋고추·토마토 가격 뛰어</t>
+          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월21일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>고랭지 여름배추 불청객 '반쪽시들음병'···미생물 퇴비로 고민 끝</t>
+          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>日, 농산물 신 품종 보호 강화…韓中 '무단유출' 염두</t>
+          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>고환율에 히트플레이션, 역대급 장마까지⋯빨간불 켜진 ‘여름 물가’[...</t>
+          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>kr.aving.net</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>[요즘 이기술] 장마철 고추 병해 예방하려면…땅 적정 산성도 유지·통...</t>
+          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.hani.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>신젠타 인시피오Ⓡ, 미국·대만·일본에 등록 완료</t>
+          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>신젠타코리아(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>진천군, 중소형 수박 브랜드 '소과담' 전시회 성료</t>
+          <t>[글로벌 특징주] 인플레 새 복병 '슈퍼 엘니뇨'…투자 대응법은</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.viva100.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>안성시, 기후변화 대응 찰옥수수 품종 선발 연구 추진</t>
+          <t>화사하고 재배 쉬운 ‘국산 나리’ 현장에서 경쟁력 살핀다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.goodkyung.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>‘농지 전수조사’ 후폭풍…십여년 키워온 ‘친환경쌀 단지’ 와해되나</t>
+          <t>유럽은 왜 유전자편집 작물의 문을 열었나</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>폭염에 채소도 녹는다…농산물 가격 '껑충'</t>
+          <t>[AFL칼럼] 농업기술박람회, 연구성과를 농업인의 기술로</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.cctimes.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>풍년에 가격 폭락 … 양파농가 시름</t>
+          <t>참외 수확하는 로봇 '참독'</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>biz.heraldcorp.com</t>
+          <t>biz.chosun.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>참외·딸기 키웠더니 농가소득 6.5배…지역특화작목 효과 입증</t>
+          <t>[위성 관측 리포트] 한 포기 ‘2만원’ 고랭지 배추 가격 이면에는… 재...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>‘국산 유기 풋거름 종자 ’ 생산, 보급 확대 첫걸음</t>
+          <t>7~9월 ‘가락시장 배추 경매’ 22시 시작</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.jejunews.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>정부, 배추· 무 3만 4천t 확보…신선란 3천만 개 수입 추진</t>
+          <t>비료값 폭등 "농가 한숨 깊어진다"</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월21일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>"폭 줄이고 통풍 극대화"... 신개념 시설하우스 농가 보급 시동</t>
+          <t>이른 더위에…풋고추·토마토 가격 뛰어</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월21일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>신젠타코리아 인시피오®, 주요 수출국 MRL 기준 충족</t>
+          <t>고랭지 여름배추 불청객 '반쪽시들음병'···미생물 퇴비로 고민 끝</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>신젠타코리아(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 바이러스 전염 차단 … 묘판 주위 방충망 촘촘히 피복</t>
+          <t>日, 농산물 신 품종 보호 강화…韓中 '무단유출' 염두</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>6월 과채류 농업관측</t>
+          <t>고환율에 히트플레이션, 역대급 장마까지⋯빨간불 켜진 ‘여름 물가’[...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>채소 병해충의 모든 것</t>
+          <t>[요즘 이기술] 장마철 고추 병해 예방하려면…땅 적정 산성도 유지·통...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>2026년 하반기 주목해야할 농기자재</t>
+          <t>신젠타 인시피오Ⓡ, 미국·대만·일본에 등록 완료</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월18일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t>신젠타코리아(주)</t>
         </is>
       </c>
     </row>
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>농사포인트 - 바이러스 전염 차단 … 묘판 주위 방충망 촘촘히 피복</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>장마철 고추농사 성패, 탄저병 예방에 달렸다</t>
+          <t>신젠타코리아 인시피오®, 주요 수출국 MRL 기준 충족</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t/>
+          <t>신젠타코리아(주)</t>
         </is>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.bokuennews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>소량 씨앗도 식물검역증명서 필수</t>
+          <t>6월 과채류 농업관측</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,20 +930,101 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.fsnews.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>여름 식탁 물가 엇갈려</t>
+          <t>채소 병해충의 모든 것</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월15일</t>
+          <t>06월17일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>www.newsam.co.kr</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>2026년 하반기 주목해야할 농기자재</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>06월16일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>(주)팜한농</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>www.dynews.co.kr</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>주간농사정보</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>06월16일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>www.farmnmarket.com</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="1">
+        <is>
+          <t>장마철 고추농사 성패, 탄저병 예방에 달렸다</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>06월16일</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -983,6 +1064,9 @@
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-25 13:09
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.munhwa.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ③ 세계 2위 농식품 수출국의 비밀...네덜란드는 왜 바...</t>
+          <t>경기도농업기술원, ‘길어야 한 달’ 봄당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>군위군, 여름철 엽채류 실증재배 추진</t>
+          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
+          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,22 +174,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
+          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.queen.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
+          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
+          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -260,12 +260,12 @@
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
+          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>부정농약 주의보… 농산물 안정성 우려</t>
+          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
+          <t>충남 대표 백합 4종 소비자 만나다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
+          <t>우주농업, 지구를 위한 미래 기술</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
+          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.kihoilbo.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
+          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>kr.aving.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
+          <t>NH농우바이오 , 7월 추천품종</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)NH농우바이오</t>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
+          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -476,12 +476,12 @@
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>[글로벌 특징주] 인플레 새 복병 '슈퍼 엘니뇨'…투자 대응법은</t>
+          <t>[AI로 읽는 경제] ③ 세계 2위 농식품 수출국의 비밀...네덜란드는 왜 바...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>화사하고 재배 쉬운 ‘국산 나리’ 현장에서 경쟁력 살핀다</t>
+          <t>군위군, 여름철 엽채류 실증재배 추진</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.goodkyung.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>유럽은 왜 유전자편집 작물의 문을 열었나</t>
+          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>[AFL칼럼] 농업기술박람회, 연구성과를 농업인의 기술로</t>
+          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.queen.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>참외 수확하는 로봇 '참독'</t>
+          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>biz.chosun.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[위성 관측 리포트] 한 포기 ‘2만원’ 고랭지 배추 가격 이면에는… 재...</t>
+          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>7~9월 ‘가락시장 배추 경매’ 22시 시작</t>
+          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.jejunews.com</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>비료값 폭등 "농가 한숨 깊어진다"</t>
+          <t>부정농약 주의보… 농산물 안정성 우려</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월21일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>이른 더위에…풋고추·토마토 가격 뛰어</t>
+          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월21일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>고랭지 여름배추 불청객 '반쪽시들음병'···미생물 퇴비로 고민 끝</t>
+          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>日, 농산물 신 품종 보호 강화…韓中 '무단유출' 염두</t>
+          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>고환율에 히트플레이션, 역대급 장마까지⋯빨간불 켜진 ‘여름 물가’[...</t>
+          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>kr.aving.net</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>[요즘 이기술] 장마철 고추 병해 예방하려면…땅 적정 산성도 유지·통...</t>
+          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.hani.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>신젠타 인시피오Ⓡ, 미국·대만·일본에 등록 완료</t>
+          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>신젠타코리아(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>biz.chosun.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 바이러스 전염 차단 … 묘판 주위 방충망 촘촘히 피복</t>
+          <t>[위성 관측 리포트] 한 포기 ‘2만원’ 고랭지 배추 가격 이면에는… 재...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>신젠타코리아 인시피오®, 주요 수출국 MRL 기준 충족</t>
+          <t>7~9월 ‘가락시장 배추 경매’ 22시 시작</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>신젠타코리아(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.jejunews.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>6월 과채류 농업관측</t>
+          <t>비료값 폭등 "농가 한숨 깊어진다"</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월21일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>채소 병해충의 모든 것</t>
+          <t>이른 더위에…풋고추·토마토 가격 뛰어</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월17일</t>
+          <t>06월21일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,22 +957,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>2026년 하반기 주목해야할 농기자재</t>
+          <t>고랭지 여름배추 불청객 '반쪽시들음병'···미생물 퇴비로 고민 끝</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>日, 농산물 신 품종 보호 강화…韓中 '무단유출' 염두</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,22 +1011,76 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>장마철 고추농사 성패, 탄저병 예방에 달렸다</t>
+          <t>고환율에 히트플레이션, 역대급 장마까지⋯빨간불 켜진 ‘여름 물가’[...</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>06월16일</t>
+          <t>06월19일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t/>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>www.nongmin.com</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="1">
+        <is>
+          <t>[요즘 이기술] 장마철 고추 병해 예방하려면…땅 적정 산성도 유지·통...</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>06월19일</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>www.aflnews.co.kr</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="1">
+        <is>
+          <t>신젠타 인시피오Ⓡ, 미국·대만·일본에 등록 완료</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>06월18일</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>신젠타코리아(주)</t>
         </is>
       </c>
     </row>
@@ -1067,6 +1121,8 @@
     <hyperlink ref="C34" r:id="rId33"/>
     <hyperlink ref="C35" r:id="rId34"/>
     <hyperlink ref="C36" r:id="rId35"/>
+    <hyperlink ref="C37" r:id="rId36"/>
+    <hyperlink ref="C38" r:id="rId37"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-29 17:38
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.munhwa.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, ‘길어야 한 달’ 봄당근 저장기간 8주까지 늘려</t>
+          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
+          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
+          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
+          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
+          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월27일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
+          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월26일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,12 +255,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
+          <t>6월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.munhwa.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
+          <t>경기도농업기술원, ‘길어야 한 달’ 봄당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>충남 대표 백합 4종 소비자 만나다</t>
+          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>우주농업, 지구를 위한 미래 기술</t>
+          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
+          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.kihoilbo.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
+          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 , 7월 추천품종</t>
+          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>(주)NH농우바이오</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
+          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ③ 세계 2위 농식품 수출국의 비밀...네덜란드는 왜 바...</t>
+          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>군위군, 여름철 엽채류 실증재배 추진</t>
+          <t>충남 대표 백합 4종 소비자 만나다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
+          <t>우주농업, 지구를 위한 미래 기술</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
+          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.queen.co.kr</t>
+          <t>www.kihoilbo.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
+          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,22 +606,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
+          <t>NH농우바이오 , 7월 추천품종</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)NH농우바이오</t>
         </is>
       </c>
     </row>
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
+          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>부정농약 주의보… 농산물 안정성 우려</t>
+          <t>[AI로 읽는 경제] ③ 세계 2위 농식품 수출국의 비밀...네덜란드는 왜 바...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
+          <t>군위군, 여름철 엽채류 실증재배 추진</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
+          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
+          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.queen.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
+          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>kr.aving.net</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
+          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
+          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>biz.chosun.com</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>[위성 관측 리포트] 한 포기 ‘2만원’ 고랭지 배추 가격 이면에는… 재...</t>
+          <t>부정농약 주의보… 농산물 안정성 우려</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>7~9월 ‘가락시장 배추 경매’ 22시 시작</t>
+          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.jejunews.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>비료값 폭등 "농가 한숨 깊어진다"</t>
+          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월21일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>이른 더위에…풋고추·토마토 가격 뛰어</t>
+          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월21일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>고랭지 여름배추 불청객 '반쪽시들음병'···미생물 퇴비로 고민 끝</t>
+          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>kr.aving.net</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>日, 농산물 신 품종 보호 강화…韓中 '무단유출' 염두</t>
+          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.hani.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>고환율에 히트플레이션, 역대급 장마까지⋯빨간불 켜진 ‘여름 물가’[...</t>
+          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-06-30 13:38
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
+          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
+          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
+          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
+          <t>화훼산업, 이대로면 사라진다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
+          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월27일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
+          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월26일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>6월 채소류 농업관측</t>
+          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.munhwa.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, ‘길어야 한 달’ 봄당근 저장기간 8주까지 늘려</t>
+          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
+          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월27일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -341,12 +341,12 @@
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
+          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월26일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
+          <t>6월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,12 +390,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.munhwa.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
+          <t>경기도농업기술원, ‘길어야 한 달’ 봄당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -417,12 +417,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
+          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -444,12 +444,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
+          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
+          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>충남 대표 백합 4종 소비자 만나다</t>
+          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>우주농업, 지구를 위한 미래 기술</t>
+          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
+          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.kihoilbo.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
+          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 , 7월 추천품종</t>
+          <t>충남 대표 백합 4종 소비자 만나다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(주)NH농우바이오</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
+          <t>우주농업, 지구를 위한 미래 기술</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ③ 세계 2위 농식품 수출국의 비밀...네덜란드는 왜 바...</t>
+          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.kihoilbo.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>군위군, 여름철 엽채류 실증재배 추진</t>
+          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
+          <t>NH농우바이오 , 7월 추천품종</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)NH농우바이오</t>
         </is>
       </c>
     </row>
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
+          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -768,12 +768,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.queen.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
+          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -795,12 +795,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
+          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.queen.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
+          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>부정농약 주의보… 농산물 안정성 우려</t>
+          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
+          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
+          <t>부정농약 주의보… 농산물 안정성 우려</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
+          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
+          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>kr.aving.net</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
+          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,12 +1011,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
+          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>kr.aving.net</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>[요즘 이기술] 장마철 고추 병해 예방하려면…땅 적정 산성도 유지·통...</t>
+          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>06월19일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1065,22 +1065,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.hani.co.kr</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="1">
         <is>
-          <t>신젠타 인시피오Ⓡ, 미국·대만·일본에 등록 완료</t>
+          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>06월18일</t>
+          <t>06월22일</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>신젠타코리아(주)</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-01 14:16
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
+          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
+          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
+          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>화훼산업, 이대로면 사라진다</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
+          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
+          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
+          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
+          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
+          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월27일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
+          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월26일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>6월 채소류 농업관측</t>
+          <t>화훼산업, 이대로면 사라진다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.munhwa.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, ‘길어야 한 달’ 봄당근 저장기간 8주까지 늘려</t>
+          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
+          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
+          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
+          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
+          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월27일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
+          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월26일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
+          <t>6월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
+          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>충남 대표 백합 4종 소비자 만나다</t>
+          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>우주농업, 지구를 위한 미래 기술</t>
+          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
+          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.kihoilbo.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
+          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 , 7월 추천품종</t>
+          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>(주)NH농우바이오</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
+          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>[농업기술박람회] "농업로봇 인력양성 서둘러야"</t>
+          <t>충남 대표 백합 4종 소비자 만나다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>"특용작물 스마트팜 기술 개발···원료 생산 안정화 모색해야"</t>
+          <t>우주농업, 지구를 위한 미래 기술</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.queen.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 기후변화에 사과 탄저병 예방 방제·과수원 위생관리 당부</t>
+          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.kihoilbo.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>동오시드 '다크그린'·'카니발', 여름 시금치 시장 공략</t>
+          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>무름병·잎마름병에 강한 국산 품종…생식용 시장 공략</t>
+          <t>NH농우바이오 , 7월 추천품종</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)NH농우바이오</t>
         </is>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>부정농약 주의보… 농산물 안정성 우려</t>
+          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
+          <t>부정농약 주의보… 농산물 안정성 우려</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
+          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -984,12 +984,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
+          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
+          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월23일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>kr.aving.net</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
+          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1065,20 +1065,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>kr.aving.net</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="1">
+        <is>
+          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>06월22일</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>www.hani.co.kr</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr" s="1">
+      <c r="C39" t="inlineStr" s="1">
         <is>
           <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>06월22일</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1123,6 +1150,7 @@
     <hyperlink ref="C36" r:id="rId35"/>
     <hyperlink ref="C37" r:id="rId36"/>
     <hyperlink ref="C38" r:id="rId37"/>
+    <hyperlink ref="C39" r:id="rId38"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-02 11:49
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
+          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
+          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
+          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.mkhealth.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
+          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
+          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,22 +255,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
+          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
         </is>
       </c>
     </row>
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
+          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
+          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
+          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>화훼산업, 이대로면 사라진다</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
+          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
+          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
+          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
+          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
+          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월27일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
+          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월26일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>6월 채소류 농업관측</t>
+          <t>화훼산업, 이대로면 사라진다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
+          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
+          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
+          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
+          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
+          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월27일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
+          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월26일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
+          <t>6월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>충남 대표 백합 4종 소비자 만나다</t>
+          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>우주농업, 지구를 위한 미래 기술</t>
+          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
+          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.kihoilbo.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
+          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 , 7월 추천품종</t>
+          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(주)NH농우바이오</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
+          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>부정농약 주의보… 농산물 안정성 우려</t>
+          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>경기 농작물 병해충 발생정보 발표…과수화상병 '경보'</t>
+          <t>충남 대표 백합 4종 소비자 만나다</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>경기 고추·사과 탄저병 주의…장마 전후 방제 당부</t>
+          <t>우주농업, 지구를 위한 미래 기술</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] IMF가 팔아버린 씨앗들...한국 종자 주권 25년의 기록</t>
+          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>06월23일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.kihoilbo.co.kr</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>" 브로콜리 너마저"…한여름 아직인데 지갑 터는 '금상추'</t>
+          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1065,22 +1065,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>kr.aving.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="1">
         <is>
-          <t>아이토브에너지, AFPRO 2026서 스마트농업 자동화 솔루션 '뿌리니' 공개...</t>
+          <t>NH농우바이오 , 7월 추천품종</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)NH농우바이오</t>
         </is>
       </c>
     </row>
@@ -1092,17 +1092,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C39" t="inlineStr" s="1">
         <is>
-          <t>유럽, ‘유전자 편집 농작물’ 빗장 풀어…신유전체기술법 통과</t>
+          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>06월22일</t>
+          <t>06월24일</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-03 15:41
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,22 +93,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.econovill.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
+          <t>농협 현장에 스타트업 7곳 초대, 소풍커넥트 애그테크 실증 판 벌인다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.fetv.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
+          <t>"모종 병들면 시작도 전에 끝"… 육묘장, 여름철 병해충 관리 방법은</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
+          <t>“농약 안전 사용 길잡이”…‘작물보호제 지침서’ 4년 만에 나왔다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>gw.newdaily.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
+          <t>여름 배추 수급 '비상등' … 정부·강원도, 태백 고랭지 찾아 작황 점검...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.mkhealth.co.kr</t>
+          <t>www.tokenpost.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
+          <t>바이엘 , 3억 달러 인수·AI 신약개발 ‘투트랙’…글리포세이트 분리까...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주)</t>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
+          <t>음성 고추명인의 밭, 새로운 한 해가 시작됐다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,22 +255,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
+          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
+          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
+          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
+          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.mkhealth.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
+          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
+          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
+          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
+          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
+          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>화훼산업, 이대로면 사라진다</t>
+          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
+          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
+          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
+          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
+          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
+          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월27일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
+          <t>화훼산업, 이대로면 사라진다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월26일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>6월 채소류 농업관측</t>
+          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>홍석영 농업위성센터장 “농림위성 7월 첫 발사… 농업 패러다임 전환”...</t>
+          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ④ 반도체 나라 대만이 씨앗에 주목하는 이유...데이터...</t>
+          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>여름철 ‘배추값’ 걱정… 준고랭지-저장 기술로 극복</t>
+          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 7월 추천 품종 공개… 토마토·배추 신품종으로 하반기 ...</t>
+          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월27일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>농업 보호망 강화… 불법 식물 유통도 처벌한다</t>
+          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월26일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
+          <t>6월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>오렌지 과육 멜론 시장 확대… 아시아 종묘 '칸타타 시리즈' 주목</t>
+          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-06 09:54
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,22 +93,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.econovill.com</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>농협 현장에 스타트업 7곳 초대, 소풍커넥트 애그테크 실증 판 벌인다</t>
+          <t>희귀작물의 가능성 넓히며 우리 농업의 새로운 미래 모색하다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.fetv.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>"모종 병들면 시작도 전에 끝"… 육묘장, 여름철 병해충 관리 방법은</t>
+          <t>‘벼멸구’ 국내 유입 가능성 커…세심한 관찰로 조기 발견해야</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>“농약 안전 사용 길잡이”…‘작물보호제 지침서’ 4년 만에 나왔다</t>
+          <t>"CPTPP 가입, 검역 주권 포기…사과산업 도산 서막"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>gw.newdaily.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>여름 배추 수급 '비상등' … 정부·강원도, 태백 고랭지 찾아 작황 점검...</t>
+          <t>[AFL 칼럼] 농림위성이 여는 '과학농정'의 시대</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.tokenpost.kr</t>
+          <t>www.econovill.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>바이엘 , 3억 달러 인수·AI 신약개발 ‘투트랙’…글리포세이트 분리까...</t>
+          <t>농협 현장에 스타트업 7곳 초대, 소풍커넥트 애그테크 실증 판 벌인다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주)</t>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.fetv.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>음성 고추명인의 밭, 새로운 한 해가 시작됐다</t>
+          <t>"모종 병들면 시작도 전에 끝"… 육묘장, 여름철 병해충 관리 방법은</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
+          <t>“농약 안전 사용 길잡이”…‘작물보호제 지침서’ 4년 만에 나왔다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>gw.newdaily.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
+          <t>여름 배추 수급 '비상등' … 정부·강원도, 태백 고랭지 찾아 작황 점검...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.tokenpost.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
+          <t>바이엘 , 3억 달러 인수·AI 신약개발 ‘투트랙’…글리포세이트 분리까...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -324,7 +324,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주)</t>
         </is>
       </c>
     </row>
@@ -336,12 +336,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
+          <t>음성 고추명인의 밭, 새로운 한 해가 시작됐다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.mkhealth.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
+          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
+          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
+          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
+          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.mkhealth.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
+          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
+          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
         </is>
       </c>
     </row>
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
+          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
+          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
+          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
+          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
+          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>화훼산업, 이대로면 사라진다</t>
+          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
+          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
+          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
+          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
+          <t>화훼산업, 이대로면 사라진다</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
+          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월27일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
+          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월26일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>6월 채소류 농업관측</t>
+          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>고온기 병해충 확산에 생육관리도 중요…팜한농, 7월 맞춤형 농자재 제...</t>
+          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월28일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>충남 대표 백합 4종 소비자 만나다</t>
+          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월27일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>우주농업, 지구를 위한 미래 기술</t>
+          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월26일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>청양 고추 농가, 품종부터 스마트팜까지 현장에서 배웠다</t>
+          <t>6월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월25일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1081,33 +1081,6 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>(주)NH농우바이오</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>www.ajunews.com</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr" s="1">
-        <is>
-          <t>삼척시, 국내육성 조사료 신품종 '트리티케일' 채종 성공</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>06월24일</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -1150,7 +1123,6 @@
     <hyperlink ref="C36" r:id="rId35"/>
     <hyperlink ref="C37" r:id="rId36"/>
     <hyperlink ref="C38" r:id="rId37"/>
-    <hyperlink ref="C39" r:id="rId38"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-06 10:09
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.econovill.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농협 현장에 스타트업 7곳 초대, 소풍커넥트 애그테크 실증 판 벌인다</t>
+          <t>제주 무등록 농약 판매조직 ‘덜미’…반값 판매로 구매 유인</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.fetv.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>"모종 병들면 시작도 전에 끝"… 육묘장, 여름철 병해충 관리 방법은</t>
+          <t>지난해 배추 ·무 수입량 전년보다 5배 ‘껑충’</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.econonews.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>“농약 안전 사용 길잡이”…‘작물보호제 지침서’ 4년 만에 나왔다</t>
+          <t>농식품부, 국내 최초 농림위성 7일 발사 '과학농정 체계 구축' ...스페이...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>gw.newdaily.co.kr</t>
+          <t>www.lak.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>여름 배추 수급 '비상등' … 정부·강원도, 태백 고랭지 찾아 작황 점검...</t>
+          <t>서울시, 도시농업에 기후위기 대응 역할 더한다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,22 +309,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.tokenpost.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>바이엘 , 3억 달러 인수·AI 신약개발 ‘투트랙’…글리포세이트 분리까...</t>
+          <t>“오이 한 상자 5200원”…과채류 가격 폭락에 농가 비상</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>음성 고추명인의 밭, 새로운 한 해가 시작됐다</t>
+          <t>식품업계 로코시대 [비즈앤피플]</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>dgmbc.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
+          <t>농촌 인력난 구원투수···밭농사 기계화로 노동력 92% 절감</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월04일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -390,22 +390,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
+          <t>캐고 고르고 담고 '척척'…밭농사도 자동화</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월04일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
+          <t>기후변화· 병해충 으로 작목 전환하는 고랭지 채소밭</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
+          <t>7월 배추·양배추값 하락, 무는 보합 전망</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,22 +471,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.mkhealth.co.kr</t>
+          <t>www.econovill.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
+          <t>농협 현장에 스타트업 7곳 초대, 소풍커넥트 애그테크 실증 판 벌인다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.fetv.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
+          <t>"모종 병들면 시작도 전에 끝"… 육묘장, 여름철 병해충 관리 방법은</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,22 +525,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
+          <t>“농약 안전 사용 길잡이”…‘작물보호제 지침서’ 4년 만에 나왔다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>gw.newdaily.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
+          <t>여름 배추 수급 '비상등' … 정부·강원도, 태백 고랭지 찾아 작황 점검...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.tokenpost.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
+          <t>바이엘 , 3억 달러 인수·AI 신약개발 ‘투트랙’…글리포세이트 분리까...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주)</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
+          <t>음성 고추명인의 밭, 새로운 한 해가 시작됐다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
+          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
+          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
+          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월02일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.mkhealth.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>작년 식품 수입 366억달러… 배추 ·무 수입 급증</t>
+          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
+          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
+          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
+          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.enewstoday.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>화훼산업, 이대로면 사라진다</t>
+          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>늦어지는 '장마'·무더위에 농산물값, 체리·파프리카↓ , 다다기오이·...</t>
+          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>해남군 '고온다습 장마철 '고추 병해충 예방 당부</t>
+          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06월29일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>‘입는 로봇’ 입어봤습니다…포도 곁순따기, 어깨 통증 없이 ‘거뜬’</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>07월01일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>도시농업으로 키운 작물, 지역경제도 ‘쑥쑥’ 키운다 [밀착취재]</t>
+          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월28일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>“그냥 수박 말고 블랙위너”… 과일 쇼핑, 품종까지 따진다</t>
+          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월27일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>[AI로 읽는 경제] ⑤ 씨앗 한 알에 특허 수십 개...글로벌 기업이 만드는...</t>
+          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06월26일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>6월 채소류 농업관측</t>
+          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>06월25일</t>
+          <t>06월30일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>www.kihoilbo.co.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>불법 수입 과일·곤충 유통도 처벌…식물방역법 개정</t>
+          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1065,22 +1065,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C38" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 , 7월 추천품종</t>
+          <t>화훼산업, 이대로면 사라진다</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>06월24일</t>
+          <t>06월29일</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>(주)NH농우바이오</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-09 16:27
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.newscj.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>희귀작물의 가능성 넓히며 우리 농업의 새로운 미래 모색하다</t>
+          <t>충청·전북 등 장마 본격, 시간당 50㎜ 폭우… 주민 대피·열차 운행 중...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>‘벼멸구’ 국내 유입 가능성 커…세심한 관찰로 조기 발견해야</t>
+          <t>농업이 우주를 만난 날…美반데버그에서 울컥한 여성연구자</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>"CPTPP 가입, 검역 주권 포기…사과산업 도산 서막"</t>
+          <t>먹거리 물가 뛰는데 농가는 적자…고유가·고환율 '이중고' [물가 돋보기...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>[AFL 칼럼] 농림위성이 여는 '과학농정'의 시대</t>
+          <t>[농가월령가] 충남 멜론의 미래 품종 다변화와 프리미엄 전략에 달렸다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.jemin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>제주 무등록 농약 판매조직 ‘덜미’…반값 판매로 구매 유인</t>
+          <t>[사설] 종자 산업 육성은 제주농업 생존전략</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>지난해 배추 ·무 수입량 전년보다 5배 ‘껑충’</t>
+          <t>[김재서 박사의 꽃 예찬] 백합 한 품종이 화훼산업의 미래를 바꾼다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.econonews.co.kr</t>
+          <t>hbnpress.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>농식품부, 국내 최초 농림위성 7일 발사 '과학농정 체계 구축' ...스페이...</t>
+          <t>고창군, 돌발해충·탄저병 등 방제 약제 농가 공급</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.lak.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>서울시, 도시농업에 기후위기 대응 역할 더한다</t>
+          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -314,12 +314,12 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>“오이 한 상자 5200원”…과채류 가격 폭락에 농가 비상</t>
+          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>식품업계 로코시대 [비즈앤피플]</t>
+          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>dgmbc.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>농촌 인력난 구원투수···밭농사 기계화로 노동력 92% 절감</t>
+          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월04일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -390,22 +390,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>캐고 고르고 담고 '척척'…밭농사도 자동화</t>
+          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월04일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>기후변화· 병해충 으로 작목 전환하는 고랭지 채소밭</t>
+          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>7월 배추·양배추값 하락, 무는 보합 전망</t>
+          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -471,22 +471,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.econovill.com</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>농협 현장에 스타트업 7곳 초대, 소풍커넥트 애그테크 실증 판 벌인다</t>
+          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.fetv.co.kr</t>
+          <t>www.kmib.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>"모종 병들면 시작도 전에 끝"… 육묘장, 여름철 병해충 관리 방법은</t>
+          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>“농약 안전 사용 길잡이”…‘작물보호제 지침서’ 4년 만에 나왔다</t>
+          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>gw.newdaily.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>여름 배추 수급 '비상등' … 정부·강원도, 태백 고랭지 찾아 작황 점검...</t>
+          <t>상주시, 노지오이 초기관리 지도 강화</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.tokenpost.kr</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>바이엘 , 3억 달러 인수·AI 신약개발 ‘투트랙’…글리포세이트 분리까...</t>
+          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주)</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>음성 고추명인의 밭, 새로운 한 해가 시작됐다</t>
+          <t>7월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>기름값 24.7% 급등·밥상물가도 들썩…6월 물가 3.2%↑, 30개월만에 최고...</t>
+          <t>‘벼멸구’ 국내 유입 가능성 커…세심한 관찰로 조기 발견해야</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>7월엔 이 동물을 조심하세요...옥수수 수십 개씩 먹고 갑니다</t>
+          <t>"CPTPP 가입, 검역 주권 포기…사과산업 도산 서막"</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>증평군, 돌봄·순찰로봇 등 온디바이스 AI 실증사업 벌인다</t>
+          <t>[AFL 칼럼] 농림위성이 여는 '과학농정'의 시대</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>2035년 韓 곡물자급률 16%대 추락…식량안보 취약해져</t>
+          <t>제주 무등록 농약 판매조직 ‘덜미’…반값 판매로 구매 유인</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월02일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.mkhealth.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>여름 대표 간식 옥수수…찰옥수수 vs 초당옥수수, 뭐가 다를까</t>
+          <t>지난해 배추 ·무 수입량 전년보다 5배 ‘껑충’</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.econonews.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>[특별기획①-2026 K-원예 희망 보고서 : 위기를 넘어 희망을 짓다] 원예...</t>
+          <t>농식품부, 국내 최초 농림위성 7일 발사 '과학농정 체계 구축' ...스페이...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.lak.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>뜨거운 여름의 건조·고온 환경에서 밀도가 높아지는 ‘진딧물’</t>
+          <t>서울시, 도시농업에 기후위기 대응 역할 더한다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>바이엘크롭사이언스(주), 신젠타코리아(주), (주)팜한농, (주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.enewstoday.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>김포시, 공공빅데이터·GIS로 벼 항공방제 '스마트 관리'</t>
+          <t>“오이 한 상자 5200원”…과채류 가격 폭락에 농가 비상</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>"인프라·환경 다 좋아요"…네덜란드 '라익즈완' 한국 투자처로 광명 선...</t>
+          <t>식품업계 로코시대 [비즈앤피플]</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>dgmbc.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>고온기 육묘장 병해충 확산 우려, 시설 안팎 관리 강화해야</t>
+          <t>농촌 인력난 구원투수···밭농사 기계화로 노동력 92% 절감</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월04일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -903,22 +903,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>캐고 고르고 담고 '척척'…밭농사도 자동화</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07월01일</t>
+          <t>07월04일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>국산보다 비싼 수입 양파…농가 보호 대책 시급</t>
+          <t>기후변화· 병해충 으로 작목 전환하는 고랭지 채소밭</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,128 +957,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>생산량 증가···제주 월동채소 '가격 뚝'</t>
+          <t>7월 배추·양배추값 하락, 무는 보합 전망</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06월30일</t>
+          <t>07월03일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.newsfarm.co.kr</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>경기도농업기술원, 봄 당근 저장기간 8주까지 늘려</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>06월30일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.seoul.co.kr</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>군위, ‘올레산 4배’ 기능성 콩 등 특화작물 키운다</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>06월30일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>www.mk.co.kr</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr" s="1">
-        <is>
-          <t>[정혁훈의 아그리젠토] 농산물 유전자 교정, 선택 아닌 생존문제</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>06월29일</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>www.farmnmarket.com</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr" s="1">
-        <is>
-          <t>화훼산업, 이대로면 사라진다</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>06월29일</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1119,10 +1011,6 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
-    <hyperlink ref="C38" r:id="rId37"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-10 10:21
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newscj.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>충청·전북 등 장마 본격, 시간당 50㎜ 폭우… 주민 대피·열차 운행 중...</t>
+          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>농업이 우주를 만난 날…美반데버그에서 울컥한 여성연구자</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>news.tf.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>먹거리 물가 뛰는데 농가는 적자…고유가·고환율 '이중고' [물가 돋보기...</t>
+          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>[농가월령가] 충남 멜론의 미래 품종 다변화와 프리미엄 전략에 달렸다</t>
+          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.jemin.com</t>
+          <t>www.newscj.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>[사설] 종자 산업 육성은 제주농업 생존전략</t>
+          <t>충청·전북 등 장마 본격, 시간당 50㎜ 폭우… 주민 대피·열차 운행 중...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[김재서 박사의 꽃 예찬] 백합 한 품종이 화훼산업의 미래를 바꾼다</t>
+          <t>농업이 우주를 만난 날…美반데버그에서 울컥한 여성연구자</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hbnpress.com</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>고창군, 돌발해충·탄저병 등 방제 약제 농가 공급</t>
+          <t>먹거리 물가 뛰는데 농가는 적자…고유가·고환율 '이중고' [물가 돋보기...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
+          <t>고유가·고환율에 '밥상 물가' 급등…가격폭락 농가도 '이중고'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
+          <t>[농가월령가] 충남 멜론의 미래 품종 다변화와 프리미엄 전략에 달렸다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,12 +336,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.jemin.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
+          <t>[사설] 종자 산업 육성은 제주농업 생존전략</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
+          <t>[김재서 박사의 꽃 예찬] 백합 한 품종이 화훼산업의 미래를 바꾼다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>hbnpress.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
+          <t>고창군, 돌발해충·탄저병 등 방제 약제 농가 공급</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
+          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
+          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
+          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.kmib.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
+          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
+          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>상주시, 노지오이 초기관리 지도 강화</t>
+          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.edaily.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
+          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>7월 이달의 추천품종</t>
+          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.kmib.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>‘벼멸구’ 국내 유입 가능성 커…세심한 관찰로 조기 발견해야</t>
+          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>"CPTPP 가입, 검역 주권 포기…사과산업 도산 서막"</t>
+          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>[AFL 칼럼] 농림위성이 여는 '과학농정'의 시대</t>
+          <t>상주시, 노지오이 초기관리 지도 강화</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>제주 무등록 농약 판매조직 ‘덜미’…반값 판매로 구매 유인</t>
+          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>지난해 배추 ·무 수입량 전년보다 5배 ‘껑충’</t>
+          <t>7월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.econonews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>농식품부, 국내 최초 농림위성 7일 발사 '과학농정 체계 구축' ...스페이...</t>
+          <t>제주 무등록 농약 판매조직 ‘덜미’…반값 판매로 구매 유인</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.lak.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>서울시, 도시농업에 기후위기 대응 역할 더한다</t>
+          <t>지난해 배추 ·무 수입량 전년보다 5배 ‘껑충’</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.econonews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>“오이 한 상자 5200원”…과채류 가격 폭락에 농가 비상</t>
+          <t>농식품부, 국내 최초 농림위성 7일 발사 '과학농정 체계 구축' ...스페이...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.lak.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>식품업계 로코시대 [비즈앤피플]</t>
+          <t>서울시, 도시농업에 기후위기 대응 역할 더한다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>dgmbc.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>농촌 인력난 구원투수···밭농사 기계화로 노동력 92% 절감</t>
+          <t>“오이 한 상자 5200원”…과채류 가격 폭락에 농가 비상</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월04일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -903,22 +903,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>캐고 고르고 담고 '척척'…밭농사도 자동화</t>
+          <t>식품업계 로코시대 [비즈앤피플]</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07월04일</t>
+          <t>07월05일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -930,22 +930,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>dgmbc.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>기후변화· 병해충 으로 작목 전환하는 고랭지 채소밭</t>
+          <t>농촌 인력난 구원투수···밭농사 기계화로 노동력 92% 절감</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월04일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -957,20 +957,74 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>www.yonhapnewstv.co.kr</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>캐고 고르고 담고 '척척'…밭농사도 자동화</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>07월04일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>한국농업기술진흥원</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>www.nongmin.com</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>기후변화· 병해충 으로 작목 전환하는 고랭지 채소밭</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>07월03일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>www.farmnmarket.com</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr" s="1">
+      <c r="C36" t="inlineStr" s="1">
         <is>
           <t>7월 배추·양배추값 하락, 무는 보합 전망</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>07월03일</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1011,6 +1065,8 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-13 16:54
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
+          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>news.tf.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
+          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
+          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.newscj.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>충청·전북 등 장마 본격, 시간당 50㎜ 폭우… 주민 대피·열차 운행 중...</t>
+          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>농업이 우주를 만난 날…美반데버그에서 울컥한 여성연구자</t>
+          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>먹거리 물가 뛰는데 농가는 적자…고유가·고환율 '이중고' [물가 돋보기...</t>
+          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>고유가·고환율에 '밥상 물가' 급등…가격폭락 농가도 '이중고'</t>
+          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월11일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[농가월령가] 충남 멜론의 미래 품종 다변화와 프리미엄 전략에 달렸다</t>
+          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.jemin.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[사설] 종자 산업 육성은 제주농업 생존전략</t>
+          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[김재서 박사의 꽃 예찬] 백합 한 품종이 화훼산업의 미래를 바꾼다</t>
+          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>hbnpress.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>고창군, 돌발해충·탄저병 등 방제 약제 농가 공급</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>news.tf.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
+          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
+          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.newscj.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
+          <t>충청·전북 등 장마 본격, 시간당 50㎜ 폭우… 주민 대피·열차 운행 중...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
+          <t>농업이 우주를 만난 날…美반데버그에서 울컥한 여성연구자</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
+          <t>먹거리 물가 뛰는데 농가는 적자…고유가·고환율 '이중고' [물가 돋보기...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
+          <t>고유가·고환율에 '밥상 물가' 급등…가격폭락 농가도 '이중고'</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
+          <t>[농가월령가] 충남 멜론의 미래 품종 다변화와 프리미엄 전략에 달렸다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.jemin.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
+          <t>[사설] 종자 산업 육성은 제주농업 생존전략</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.kmib.co.kr</t>
+          <t>www.jeonmae.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
+          <t>[김재서 박사의 꽃 예찬] 백합 한 품종이 화훼산업의 미래를 바꾼다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>hbnpress.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
+          <t>고창군, 돌발해충·탄저병 등 방제 약제 농가 공급</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>상주시, 노지오이 초기관리 지도 강화</t>
+          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.edaily.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
+          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>7월 이달의 추천품종</t>
+          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>제주 무등록 농약 판매조직 ‘덜미’…반값 판매로 구매 유인</t>
+          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월08일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>지난해 배추 ·무 수입량 전년보다 5배 ‘껑충’</t>
+          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월06일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.econonews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>농식품부, 국내 최초 농림위성 7일 발사 '과학농정 체계 구축' ...스페이...</t>
+          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,22 +849,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.lak.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>서울시, 도시농업에 기후위기 대응 역할 더한다</t>
+          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>“오이 한 상자 5200원”…과채류 가격 폭락에 농가 비상</t>
+          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.kmib.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>식품업계 로코시대 [비즈앤피플]</t>
+          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07월05일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,22 +930,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>dgmbc.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>농촌 인력난 구원투수···밭농사 기계화로 노동력 92% 절감</t>
+          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07월04일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -957,22 +957,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>캐고 고르고 담고 '척척'…밭농사도 자동화</t>
+          <t>상주시, 노지오이 초기관리 지도 강화</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>07월04일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>기후변화· 병해충 으로 작목 전환하는 고랭지 채소밭</t>
+          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>7월 배추·양배추값 하락, 무는 보합 전망</t>
+          <t>7월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>07월03일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-14 15:08
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.eroun.net</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
+          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
+          <t>제놀루션, 고추 바이러스 표적 RNA 농약 특허 출원…글로벌 시장 공략</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
+          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.jnilbo.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
+          <t>함평군, 미니단호박 특화작목 육성</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
+          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
+          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
+          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
+          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월11일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
+          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
+          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
+          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>news.tf.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
+          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월11일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
+          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newscj.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>충청·전북 등 장마 본격, 시간당 50㎜ 폭우… 주민 대피·열차 운행 중...</t>
+          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>농업이 우주를 만난 날…美반데버그에서 울컥한 여성연구자</t>
+          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>먹거리 물가 뛰는데 농가는 적자…고유가·고환율 '이중고' [물가 돋보기...</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>news.tf.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>고유가·고환율에 '밥상 물가' 급등…가격폭락 농가도 '이중고'</t>
+          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>[농가월령가] 충남 멜론의 미래 품종 다변화와 프리미엄 전략에 달렸다</t>
+          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.jemin.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[사설] 종자 산업 육성은 제주농업 생존전략</t>
+          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.jeonmae.co.kr</t>
+          <t>www.domin.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>[김재서 박사의 꽃 예찬] 백합 한 품종이 화훼산업의 미래를 바꾼다</t>
+          <t>고창군 과수화상병 청정 유지, 병해충 예찰 강화</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>hbnpress.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>고창군, 돌발해충·탄저병 등 방제 약제 농가 공급</t>
+          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
+          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
+          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
+          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
+          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
+          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
+          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.kmib.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
+          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -876,12 +876,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
+          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.kmib.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
+          <t>상주시, 노지오이 초기관리 지도 강화</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
+          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>상주시, 노지오이 초기관리 지도 강화</t>
+          <t>7월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -971,60 +971,6 @@
         </is>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.edaily.co.kr</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.hortitimes.com</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>7월 이달의 추천품종</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1065,8 +1011,6 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-14 16:47
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,12 +93,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.eroun.net</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -120,12 +120,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.edaily.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 고추 바이러스 표적 RNA 농약 특허 출원…글로벌 시장 공략</t>
+          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
+          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.jnilbo.com</t>
+          <t>www.eroun.net</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>함평군, 미니단호박 특화작목 육성</t>
+          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
+          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.jnilbo.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
+          <t>함평군, 미니단호박 특화작목 육성</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,12 +255,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
+          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
+          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -309,12 +309,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
+          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -336,12 +336,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
+          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
+          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
+          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
+          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월11일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
+          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
+          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월11일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
+          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>news.tf.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
+          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>news.tf.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>'26~'27년산 제주 월동채소 작황관측 확대</t>
+          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.domin.co.kr</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>고창군 과수화상병 청정 유지, 병해충 예찰 강화</t>
+          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>[주산지 르포] 벼랑 끝 내몰린 농가…“양 배추 수확할수록 손해”</t>
+          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
+          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
+          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월07일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
+          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
+          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -795,12 +795,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
+          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.kmib.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
+          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.kmib.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
+          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
+          <t>상주시, 노지오이 초기관리 지도 강화</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>상주시, 노지오이 초기관리 지도 강화</t>
+          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.edaily.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
+          <t>7월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -944,33 +944,6 @@
         </is>
       </c>
       <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.hortitimes.com</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>7월 이달의 추천품종</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1010,7 +983,6 @@
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-15 09:17
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>밭 갈아엎는 농민·상추 못 주는 식당…유통 비용 줄여 모순 깬다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
+          <t>“하룻밤 새 번지던 흰가루병…한번 살포로 발생 뚝”</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
+          <t>돼지 도축하고 딸기 따는 로봇… 피지컬 AI 현장에 나서다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.eroun.net</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
+          <t>"진한 향, 달콤함 가득" 주황 멜론이 뜬다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.jnilbo.com</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>함평군, 미니단호박 특화작목 육성</t>
+          <t>예천서 증식한 국가보급종 꿀벌 '젤리킹' 경북 첫 보급</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
+          <t>함평군 '국산 미니단호박 육성 박차' 농가 의견 수렴</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
+          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
+          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.eroun.net</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
+          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
+          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
+          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
+          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
+          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월11일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
+          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
+          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
+          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
+          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>news.tf.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
+          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월12일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
+          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월09일</t>
+          <t>07월11일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>여름철 상추 ‘순수 수경재배’ 때 양액 이온 균형 관리 중요</t>
+          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 동부지원, 종자 ·묘 유통 단속 실시</t>
+          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월08일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>내병성 토마토·저장성 우수 양파·비대력 좋은 수박 '강추'</t>
+          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>반복되는 채소 산지폐기, 이제 끝내야</t>
+          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,22 +768,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>news.tf.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>생분해 비닐 또···괴산 농가 '조기 분해' 피해 잇따라</t>
+          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>(주)팜한농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>[오마이포토] 참외 1kg 800원, 양파 1kg 650원... 7·7 전국농민대회</t>
+          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월09일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.kmib.co.kr</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>제주, 종자 산업에 2030년까지 584억 투입</t>
+          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,101 +849,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>종이 대신 전자증명서…농산물 검역, 22개국과 실시간 연결</t>
+          <t>7월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월07일</t>
+          <t>07월06일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>www.idaegu.co.kr</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>상주시, 노지오이 초기관리 지도 강화</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>www.edaily.co.kr</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>www.hortitimes.com</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="1">
-        <is>
-          <t>7월 이달의 추천품종</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -980,9 +899,6 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-16 15:41
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>jejumbc.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>밭 갈아엎는 농민·상추 못 주는 식당…유통 비용 줄여 모순 깬다</t>
+          <t>월동무 ·양배추 재배면적 줄고 양파 늘어</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,12 +120,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.gnmaeil.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>“하룻밤 새 번지던 흰가루병…한번 살포로 발생 뚝”</t>
+          <t>남해군, 새 소득원 아열대 채소 육성 주력</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>돼지 도축하고 딸기 따는 로봇… 피지컬 AI 현장에 나서다</t>
+          <t>팜한농 '비채', 현대백화점 판교점 정식 입점…프리미엄 기능성 채소 유...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>"진한 향, 달콤함 가득" 주황 멜론이 뜬다</t>
+          <t>남해군 '아열대 채소 공심채·여주' 판로 확대 추진</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.jejusori.net</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>2026~27년 월동채소 " 무 ·양배추 감소, 양파 증가" 예상</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>예천서 증식한 국가보급종 꿀벌 '젤리킹' 경북 첫 보급</t>
+          <t>가을 파종용 수입 종자 특별검역 실시</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>함평군 '국산 미니단호박 육성 박차' 농가 의견 수렴</t>
+          <t>농사포인트 - 고추탄저병 6월 상순부터 10일 간격 약액 잘 묻도록 밑에...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>밭 갈아엎는 농민·상추 못 주는 식당…유통 비용 줄여 모순 깬다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
+          <t>“하룻밤 새 번지던 흰가루병…한번 살포로 발생 뚝”</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
+          <t>돼지 도축하고 딸기 따는 로봇… 피지컬 AI 현장에 나서다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.eroun.net</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
+          <t>"진한 향, 달콤함 가득" 주황 멜론이 뜬다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,12 +390,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
+          <t>예천서 증식한 국가보급종 꿀벌 '젤리킹' 경북 첫 보급</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 생물농약 dsRNA, 국내 도입 급물살-RNA 농약, 화학농약 대체 차...</t>
+          <t>함평군 '국산 미니단호박 육성 박차' 농가 의견 수렴</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>[Issue+] 농업용 로봇의 현재와 미래</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>[전국 톡톡] '무더위를 잡아라'‥폭염 대책도 '역대급'</t>
+          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>농작물 436.2㏊ 침수…충남 물폭탄 집중</t>
+          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.eroun.net</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>농민·농협 임직원 위한 ‘생성형 AI’ 개발</t>
+          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>농업수입안정보험 1203억 지급…농가 2만700호 혜택</t>
+          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>옥수수의 고장 충주…신품종 '찰옥5호' 대학찰옥수수 넘어설까</t>
+          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월12일</t>
+          <t>07월13일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>여름에 먹으면 최고인데… 하염없이 가격 폭락 중이라는 '제철 채소'</t>
+          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월11일</t>
+          <t>07월10일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
+          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -674,195 +674,6 @@
         </is>
       </c>
       <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>www.agrinet.co.kr</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr" s="1">
-        <is>
-          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>07월10일</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>www.farmnmarket.com</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr" s="1">
-        <is>
-          <t>한국작물보호협회, ‘2026 작물보호제(농약) 지침서’ 발간</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>07월10일</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>www.ytn.co.kr</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr" s="1">
-        <is>
-          <t>폭우와 폭염 사이...농작물·가축 피해 줄이려면</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>07월10일</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>news.tf.co.kr</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr" s="1">
-        <is>
-          <t>청년·고령층 '식집사' 늘어난다…댕댕이보다 정겨운 반려식물</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>07월10일</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>www.ccdn.co.kr</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr" s="1">
-        <is>
-          <t>농산물 값 폭락·생산비 급등 농민 이중고</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>07월09일</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>www.edaily.co.kr</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr" s="1">
-        <is>
-          <t>NH농우바이오 “국내 1위 넘어 글로벌 톱10…해외법인 확대 속도낼 것”...</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>www.hortitimes.com</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr" s="1">
-        <is>
-          <t>7월 이달의 추천품종</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>07월06일</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -892,13 +703,6 @@
     <hyperlink ref="C21" r:id="rId20"/>
     <hyperlink ref="C22" r:id="rId21"/>
     <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
-    <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
-    <hyperlink ref="C27" r:id="rId26"/>
-    <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-20 10:24
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>jejumbc.com</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>월동무 ·양배추 재배면적 줄고 양파 늘어</t>
+          <t>"국민 체감하는 현장 성과 창출에 역량 집중할 것"</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.gnmaeil.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>남해군, 새 소득원 아열대 채소 육성 주력</t>
+          <t>연중 재배 가능 '올시즌 시금치' 추천</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.fsnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>팜한농 '비채', 현대백화점 판교점 정식 입점…프리미엄 기능성 채소 유...</t>
+          <t>더 달고 쫄깃한 옥수수 '찰옥5호'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>남해군 '아열대 채소 공심채·여주' 판로 확대 추진</t>
+          <t>중국판 ‘노아의 방주’에 풀 종자 6만점 “식량안보 위한 빅데이터”</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.jejusori.net</t>
+          <t>www.dkilbo.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>2026~27년 월동채소 " 무 ·양배추 감소, 양파 증가" 예상</t>
+          <t>경북도, 초당옥수수 신품종'청밀옥'개발</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.jejumaeil.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>가을 파종용 수입 종자 특별검역 실시</t>
+          <t>국비 지원으로 덩치 키운 '푸파페 제주'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 고추탄저병 6월 상순부터 10일 간격 약액 잘 묻도록 밑에...</t>
+          <t>팜한농 '비채', 현대백화점 입점 성사</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.nocutnews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>밭 갈아엎는 농민·상추 못 주는 식당…유통 비용 줄여 모순 깬다</t>
+          <t>'국토 27%가 사막' 중국이 생태복원에 매진하는 이유는</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월18일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>“하룻밤 새 번지던 흰가루병…한번 살포로 발생 뚝”</t>
+          <t>20년 유기농 고추 명인도 반해버린 ‘솔로아그리’</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>돼지 도축하고 딸기 따는 로봇… 피지컬 AI 현장에 나서다</t>
+          <t>농식품부, AI 가격비교앱·가격안정제 도입…'국민 체감 농정' 속도</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>jejumbc.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>"진한 향, 달콤함 가득" 주황 멜론이 뜬다</t>
+          <t>월동무 ·양배추 재배면적 줄고 양파 늘어</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.gnmaeil.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>남해군, 새 소득원 아열대 채소 육성 주력</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>예천서 증식한 국가보급종 꿀벌 '젤리킹' 경북 첫 보급</t>
+          <t>남해군 '아열대 채소 공심채·여주' 판로 확대 추진</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.jejusori.net</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>함평군 '국산 미니단호박 육성 박차' 농가 의견 수렴</t>
+          <t>2026~27년 월동채소 " 무 ·양배추 감소, 양파 증가" 예상</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>가을 파종용 수입 종자 특별검역 실시</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
+          <t>"제주 월동무 ·양배추 재배 줄고 양파 늘듯…종자 신청량 예측"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
+          <t>농사포인트 - 고추탄저병 6월 상순부터 10일 간격 약액 잘 묻도록 밑에...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.eroun.net</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>고창 건 고추 장터 18일 개장…11월까지 주말·장날 직거래 운영</t>
+          <t>밭 갈아엎는 농민·상추 못 주는 식당…유통 비용 줄여 모순 깬다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>'극한더위'에 신음하는 농민들…온열질환에도 노출</t>
+          <t>“하룻밤 새 번지던 흰가루병…한번 살포로 발생 뚝”</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
+          <t>돼지 도축하고 딸기 따는 로봇… 피지컬 AI 현장에 나서다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>정부, 여름 무 ·배추 기준가격 하향조정···산지는 '속앓이'</t>
+          <t>"진한 향, 달콤함 가득" 주황 멜론이 뜬다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,20 +660,182 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>" 메론 매입 늦추고 단가 인하" 유통업체 횡포에 시름</t>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월10일</t>
+          <t>07월14일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>www.imaeil.com</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="1">
+        <is>
+          <t>예천서 증식한 국가보급종 꿀벌 '젤리킹' 경북 첫 보급</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>07월14일</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>www.namdonews.com</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="1">
+        <is>
+          <t>함평군 '국산 미니단호박 육성 박차' 농가 의견 수렴</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>07월14일</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>www.dynews.co.kr</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr" s="1">
+        <is>
+          <t>주간농사정보</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>07월14일</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>www.newspim.com</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr" s="1">
+        <is>
+          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>07월14일</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>www.ccdailynews.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr" s="1">
+        <is>
+          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>07월14일</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>www.newsam.co.kr</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="1">
+        <is>
+          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>07월13일</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -703,6 +865,12 @@
     <hyperlink ref="C21" r:id="rId20"/>
     <hyperlink ref="C22" r:id="rId21"/>
     <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
+    <hyperlink ref="C25" r:id="rId24"/>
+    <hyperlink ref="C26" r:id="rId25"/>
+    <hyperlink ref="C27" r:id="rId26"/>
+    <hyperlink ref="C28" r:id="rId27"/>
+    <hyperlink ref="C29" r:id="rId28"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-22 09:25
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>"국민 체감하는 현장 성과 창출에 역량 집중할 것"</t>
+          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>연중 재배 가능 '올시즌 시금치' 추천</t>
+          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.fsnews.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>더 달고 쫄깃한 옥수수 '찰옥5호'</t>
+          <t>채소·과일, 폭염에도 가격 안정세</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>중국판 ‘노아의 방주’에 풀 종자 6만점 “식량안보 위한 빅데이터”</t>
+          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.dkilbo.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>경북도, 초당옥수수 신품종'청밀옥'개발</t>
+          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.jejumaeil.net</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>국비 지원으로 덩치 키운 '푸파페 제주'</t>
+          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>팜한농 '비채', 현대백화점 입점 성사</t>
+          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.nocutnews.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>'국토 27%가 사막' 중국이 생태복원에 매진하는 이유는</t>
+          <t>예산읍 제철 고추 임시 직거래장 25일 개장</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월18일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -314,12 +314,12 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>20년 유기농 고추 명인도 반해버린 ‘솔로아그리’</t>
+          <t>손목 장치가 폭염 위험 알린다…농업인 온열질환 예방 기술 현장 실증</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,22 +336,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>농식품부, AI 가격비교앱·가격안정제 도입…'국민 체감 농정' 속도</t>
+          <t>찰옥수수 '찰옥5호', 기계수확으로 인력 86% 절감</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>jejumbc.com</t>
+          <t>www.foodnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>월동무 ·양배추 재배면적 줄고 양파 늘어</t>
+          <t>한 컷으로 만나는 미래의 씨앗… 종자 사진 공모전</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.gnmaeil.com</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>남해군, 새 소득원 아열대 채소 육성 주력</t>
+          <t>농산물 가격 폭락하는 와중에 혼자 역주행… 폭염·장마 직격탄 맞고 금...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>남해군 '아열대 채소 공심채·여주' 판로 확대 추진</t>
+          <t>다산바이오, 제주 성산농협에 월동무 신품종 '무궁무진' 공급</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.jejusori.net</t>
+          <t>news.skbroadband.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>2026~27년 월동채소 " 무 ·양배추 감소, 양파 증가" 예상</t>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>가을 파종용 수입 종자 특별검역 실시</t>
+          <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>"제주 월동무 ·양배추 재배 줄고 양파 늘듯…종자 신청량 예측"</t>
+          <t>"국민 체감하는 현장 성과 창출에 역량 집중할 것"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 고추탄저병 6월 상순부터 10일 간격 약액 잘 묻도록 밑에...</t>
+          <t>연중 재배 가능 '올시즌 시금치' 추천</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>밭 갈아엎는 농민·상추 못 주는 식당…유통 비용 줄여 모순 깬다</t>
+          <t>중국판 ‘노아의 방주’에 풀 종자 6만점 “식량안보 위한 빅데이터”</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.dkilbo.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>“하룻밤 새 번지던 흰가루병…한번 살포로 발생 뚝”</t>
+          <t>경북도, 초당옥수수 신품종'청밀옥'개발</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,22 +606,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.jejumaeil.net</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>돼지 도축하고 딸기 따는 로봇… 피지컬 AI 현장에 나서다</t>
+          <t>국비 지원으로 덩치 키운 '푸파페 제주'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>"진한 향, 달콤함 가득" 주황 멜론이 뜬다</t>
+          <t>팜한농 '비채', 현대백화점 입점 성사</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>www.nocutnews.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>'국토 27%가 사막' 중국이 생태복원에 매진하는 이유는</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월18일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>예천서 증식한 국가보급종 꿀벌 '젤리킹' 경북 첫 보급</t>
+          <t>20년 유기농 고추 명인도 반해버린 ‘솔로아그리’</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>함평군 '국산 미니단호박 육성 박차' 농가 의견 수렴</t>
+          <t>농식품부, AI 가격비교앱·가격안정제 도입…'국민 체감 농정' 속도</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.gnmaeil.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>남해군, 새 소득원 아열대 채소 육성 주력</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 고추 BBWV2 표적 RNA 작물보호제 특허 출원</t>
+          <t>남해군 '아열대 채소 공심채·여주' 판로 확대 추진</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.jejusori.net</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>서산시, 농작물 병해충 방제약제 선정 및 적기 방제 준비</t>
+          <t>2026~27년 월동채소 " 무 ·양배추 감소, 양파 증가" 예상</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월14일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,20 +822,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>내서성, 내습성 최강 아시아 종묘 시금치 ‘올시즌’</t>
+          <t>가을 파종용 수입 종자 특별검역 실시</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월13일</t>
+          <t>07월15일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>www.wonyesanup.co.kr</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="1">
+        <is>
+          <t>농사포인트 - 고추탄저병 6월 상순부터 10일 간격 약액 잘 묻도록 밑에...</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>07월15일</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -871,6 +898,7 @@
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-23 15:11
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
+          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.wowtv.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
+          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>채소·과일, 폭염에도 가격 안정세</t>
+          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
+          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
+          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsfreezone.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
+          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
+          <t>7월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>예산읍 제철 고추 임시 직거래장 25일 개장</t>
+          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>손목 장치가 폭염 위험 알린다…농업인 온열질환 예방 기술 현장 실증</t>
+          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,22 +336,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>찰옥수수 '찰옥5호', 기계수확으로 인력 86% 절감</t>
+          <t>채소·과일, 폭염에도 가격 안정세</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.foodnews.co.kr</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>한 컷으로 만나는 미래의 씨앗… 종자 사진 공모전</t>
+          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 폭락하는 와중에 혼자 역주행… 폭염·장마 직격탄 맞고 금...</t>
+          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>다산바이오, 제주 성산농협에 월동무 신품종 '무궁무진' 공급</t>
+          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>news.skbroadband.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
+          <t>예산읍 제철 고추 임시 직거래장 25일 개장</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>"국민 체감하는 현장 성과 창출에 역량 집중할 것"</t>
+          <t>손목 장치가 폭염 위험 알린다…농업인 온열질환 예방 기술 현장 실증</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,22 +525,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>연중 재배 가능 '올시즌 시금치' 추천</t>
+          <t>찰옥수수 '찰옥5호', 기계수확으로 인력 86% 절감</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>중국판 ‘노아의 방주’에 풀 종자 6만점 “식량안보 위한 빅데이터”</t>
+          <t>농산물 가격 폭락하는 와중에 혼자 역주행… 폭염·장마 직격탄 맞고 금...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.dkilbo.com</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>경북도, 초당옥수수 신품종'청밀옥'개발</t>
+          <t>다산바이오, 제주 성산농협에 월동무 신품종 '무궁무진' 공급</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,22 +606,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.jejumaeil.net</t>
+          <t>news.skbroadband.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>국비 지원으로 덩치 키운 '푸파페 제주'</t>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>팜한농 '비채', 현대백화점 입점 성사</t>
+          <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.nocutnews.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>'국토 27%가 사막' 중국이 생태복원에 매진하는 이유는</t>
+          <t>중국판 ‘노아의 방주’에 풀 종자 6만점 “식량안보 위한 빅데이터”</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월18일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.dkilbo.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>20년 유기농 고추 명인도 반해버린 ‘솔로아그리’</t>
+          <t>경북도, 초당옥수수 신품종'청밀옥'개발</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.jejumaeil.net</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>농식품부, AI 가격비교앱·가격안정제 도입…'국민 체감 농정' 속도</t>
+          <t>국비 지원으로 덩치 키운 '푸파페 제주'</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.gnmaeil.com</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>남해군, 새 소득원 아열대 채소 육성 주력</t>
+          <t>팜한농 '비채', 현대백화점 입점 성사</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월19일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.nocutnews.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>남해군 '아열대 채소 공심채·여주' 판로 확대 추진</t>
+          <t>'국토 27%가 사막' 중국이 생태복원에 매진하는 이유는</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월18일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.jejusori.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>2026~27년 월동채소 " 무 ·양배추 감소, 양파 증가" 예상</t>
+          <t>20년 유기농 고추 명인도 반해버린 ‘솔로아그리’</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,47 +822,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>가을 파종용 수입 종자 특별검역 실시</t>
+          <t>농식품부, AI 가격비교앱·가격안정제 도입…'국민 체감 농정' 속도</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월15일</t>
+          <t>07월16일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>www.wonyesanup.co.kr</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr" s="1">
-        <is>
-          <t>농사포인트 - 고추탄저병 6월 상순부터 10일 간격 약액 잘 묻도록 밑에...</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>07월15일</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -898,7 +871,6 @@
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-24 11:24
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
+          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.wowtv.co.kr</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
+          <t>K-농기자재 수출 협약 373만 달러 체결</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
+          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.fntimes.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
+          <t>강원특별자치도·강원농협, 농산물 가격안정 총력…소비촉진·가격보전...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.greened.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
+          <t>농어촌公, 안전관리·K-농기자재 수출 지원 '두 토끼' 잡는다</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newsfreezone.co.kr</t>
+          <t>www.seoulfn.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
+          <t>수박값 1년 새 36%↓···여름 과일·채소값도 안정세</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>7월 채소류 농업관측</t>
+          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.wowtv.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
+          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,22 +309,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
+          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>채소·과일, 폭염에도 가격 안정세</t>
+          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
+          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newsfreezone.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
+          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
+          <t>7월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
+          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>예산읍 제철 고추 임시 직거래장 25일 개장</t>
+          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>손목 장치가 폭염 위험 알린다…농업인 온열질환 예방 기술 현장 실증</t>
+          <t>채소·과일, 폭염에도 가격 안정세</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,22 +525,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>찰옥수수 '찰옥5호', 기계수확으로 인력 86% 절감</t>
+          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 폭락하는 와중에 혼자 역주행… 폭염·장마 직격탄 맞고 금...</t>
+          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>다산바이오, 제주 성산농협에 월동무 신품종 '무궁무진' 공급</t>
+          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>news.skbroadband.com</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
+          <t>예산읍 제철 고추 임시 직거래장 25일 개장</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>중국판 ‘노아의 방주’에 풀 종자 6만점 “식량안보 위한 빅데이터”</t>
+          <t>손목 장치가 폭염 위험 알린다…농업인 온열질환 예방 기술 현장 실증</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,22 +687,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.dkilbo.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>경북도, 초당옥수수 신품종'청밀옥'개발</t>
+          <t>찰옥수수 '찰옥5호', 기계수확으로 인력 86% 절감</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월21일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.jejumaeil.net</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>국비 지원으로 덩치 키운 '푸파페 제주'</t>
+          <t>농산물 가격 폭락하는 와중에 혼자 역주행… 폭염·장마 직격탄 맞고 금...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>팜한농 '비채', 현대백화점 입점 성사</t>
+          <t>다산바이오, 제주 성산농협에 월동무 신품종 '무궁무진' 공급</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월19일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.nocutnews.co.kr</t>
+          <t>news.skbroadband.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>'국토 27%가 사막' 중국이 생태복원에 매진하는 이유는</t>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월18일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,47 +795,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>20년 유기농 고추 명인도 반해버린 ‘솔로아그리’</t>
+          <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월16일</t>
+          <t>07월20일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>www.newspim.com</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr" s="1">
-        <is>
-          <t>농식품부, AI 가격비교앱·가격안정제 도입…'국민 체감 농정' 속도</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>07월16일</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -870,7 +843,6 @@
     <hyperlink ref="C26" r:id="rId25"/>
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-27 09:36
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.shinailbo.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
+          <t>예산군, 멜론 재배에 '뒤영벌' 활용…꿀벌 부족 대응 시범사업 성과</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>K-농기자재 수출 협약 373만 달러 체결</t>
+          <t>고추 세척기·차열막 ‘맞춤형 지원’ 호평</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
+          <t>제주 브로콜리 ‘삼다그린’ 국산화 속도</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.fntimes.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>강원특별자치도·강원농협, 농산물 가격안정 총력…소비촉진·가격보전...</t>
+          <t>［이슈현장］홍천 내면 고랭지 채소 폐기 속출 “저장고 확충 시급”</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.greened.kr</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>농어촌公, 안전관리·K-농기자재 수출 지원 '두 토끼' 잡는다</t>
+          <t>미원면 양채류 재배단지, 가을작물 모종 심기 시작</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.seoulfn.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>수박값 1년 새 36%↓···여름 과일·채소값도 안정세</t>
+          <t>한 컷으로 만나는 미래의 씨앗 생명·희망 품은 종자 , 사진에 담는다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
+          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.wowtv.co.kr</t>
+          <t>www.joongang.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
+          <t>‘수출 4강’ 들겠다는 한국…바로 앞줄에 네덜란드 버틴다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -314,17 +314,17 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
+          <t>검역본부, 유전자변형생물체 검사 효율 높이는 신기술 개발</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월25일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
+          <t>다산바이오, '혁신 프리미어 1000' 선정... AI 디지털육종 고도화</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
+          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.newsfreezone.co.kr</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
+          <t>K-농기자재 수출 협약 373만 달러 체결</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>7월 채소류 농업관측</t>
+          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.fntimes.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
+          <t>강원특별자치도·강원농협, 농산물 가격안정 총력…소비촉진·가격보전...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.seoulfn.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
+          <t>수박값 1년 새 36%↓···여름 과일·채소값도 안정세</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>채소·과일, 폭염에도 가격 안정세</t>
+          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.wowtv.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
+          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
+          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
+          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
+          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.newsfreezone.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>예산읍 제철 고추 임시 직거래장 25일 개장</t>
+          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>손목 장치가 폭염 위험 알린다…농업인 온열질환 예방 기술 현장 실증</t>
+          <t>7월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,22 +687,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>찰옥수수 '찰옥5호', 기계수확으로 인력 86% 절감</t>
+          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>농산물 가격 폭락하는 와중에 혼자 역주행… 폭염·장마 직격탄 맞고 금...</t>
+          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>다산바이오, 제주 성산농협에 월동무 신품종 '무궁무진' 공급</t>
+          <t>채소·과일, 폭염에도 가격 안정세</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>news.skbroadband.com</t>
+          <t>www.ggilbo.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,20 +795,128 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>www.agrinet.co.kr</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr" s="1">
+        <is>
+          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>07월21일</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>www.youngnong.co.kr</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="1">
+        <is>
+          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>07월21일</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>www.segye.com</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="1">
+        <is>
+          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>07월21일</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>news.skbroadband.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>07월20일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>www.seoul.co.kr</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr" s="1">
+      <c r="C32" t="inlineStr" s="1">
         <is>
           <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>07월20일</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -843,6 +951,10 @@
     <hyperlink ref="C26" r:id="rId25"/>
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
+    <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-29 14:16
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.shinailbo.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>예산군, 멜론 재배에 '뒤영벌' 활용…꿀벌 부족 대응 시범사업 성과</t>
+          <t>‘슈퍼오닝’ 쌀 항공방제 팔걷어</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>고추 세척기·차열막 ‘맞춤형 지원’ 호평</t>
+          <t>"가락시장 수수료도 안 나와"...밭에서 썩는 고랭지 배추</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>제주 브로콜리 ‘삼다그린’ 국산화 속도</t>
+          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>［이슈현장］홍천 내면 고랭지 채소 폐기 속출 “저장고 확충 시급”</t>
+          <t>극한 가뭄…유럽·미국에서 현실이 된 ‘물 전쟁’</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>미원면 양채류 재배단지, 가을작물 모종 심기 시작</t>
+          <t>중국, 종자산업 지식재산권 보호 강화</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>한 컷으로 만나는 미래의 씨앗 생명·희망 품은 종자 , 사진에 담는다</t>
+          <t>‘종이 농업’ 스캔들의 中 식량 안보… 베이더우 위성과 드론, 허위 보...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.lak.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
+          <t>한수정, 글로벌 정원산업 거점화 추진</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>‘수출 4강’ 들겠다는 한국…바로 앞줄에 네덜란드 버틴다</t>
+          <t>가을 무 ·배추, 밑거름 선택이 수확을 좌우한다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>검역본부, 유전자변형생물체 검사 효율 높이는 신기술 개발</t>
+          <t>조비, '강추' 밑거름 가을 무 ·배추 '초기 생육' 잡는다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월25일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.shinailbo.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>다산바이오, '혁신 프리미어 1000' 선정... AI 디지털육종 고도화</t>
+          <t>예산군, 멜론 재배에 '뒤영벌' 활용…꿀벌 부족 대응 시범사업 성과</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
+          <t>고추 세척기·차열막 ‘맞춤형 지원’ 호평</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>K-농기자재 수출 협약 373만 달러 체결</t>
+          <t>제주 브로콜리 ‘삼다그린’ 국산화 속도</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
+          <t>［이슈현장］홍천 내면 고랭지 채소 폐기 속출 “저장고 확충 시급”</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.fntimes.com</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>강원특별자치도·강원농협, 농산물 가격안정 총력…소비촉진·가격보전...</t>
+          <t>미원면 양채류 재배단지, 가을작물 모종 심기 시작</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.seoulfn.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>수박값 1년 새 36%↓···여름 과일·채소값도 안정세</t>
+          <t>한 컷으로 만나는 미래의 씨앗 생명·희망 품은 종자 , 사진에 담는다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
+          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.wowtv.co.kr</t>
+          <t>www.joongang.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
+          <t>‘수출 4강’ 들겠다는 한국…바로 앞줄에 네덜란드 버틴다</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -557,17 +557,17 @@
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
+          <t>검역본부, 유전자변형생물체 검사 효율 높이는 신기술 개발</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월25일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
+          <t>다산바이오, '혁신 프리미어 1000' 선정... AI 디지털육종 고도화</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
+          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.newsfreezone.co.kr</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
+          <t>K-농기자재 수출 협약 373만 달러 체결</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>7월 채소류 농업관측</t>
+          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.fntimes.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>양파 재사용 육묘판 관리, 기계 정식률 향상 첫걸음</t>
+          <t>강원특별자치도·강원농협, 농산물 가격안정 총력…소비촉진·가격보전...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.seoulfn.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>농작물 41.6㏊ 침수…경북지역 ‘물폭탄’</t>
+          <t>수박값 1년 새 36%↓···여름 과일·채소값도 안정세</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>채소·과일, 폭염에도 가격 안정세</t>
+          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.ggilbo.com</t>
+          <t>www.wowtv.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>상추 값 160% 뛰었다… 고기쌈, 이제 뭘로 싸 먹을까?</t>
+          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월22일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>생산량 급감에 채소가격 올랐지만···평년 시세 회복은 '불투명'</t>
+          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>"로열티 8억 아꼈다"… 경기도, 폭염 이기는 'K-국화' 개발</t>
+          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월23일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>자생 식물 발굴부터 판로 확대까지…한수정, 정원산업 생태계 키운다</t>
+          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월21일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>news.skbroadband.com</t>
+          <t>www.newsfreezone.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>고지대도 30도 이상 폭염…고랭지 배추 '전전긍긍'</t>
+          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>제주어도 알아듣는 ‘AI 농업비서’… 월동무 ·브로콜리 생산량도 미리...</t>
+          <t>7월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07월20일</t>
+          <t>07월22일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-07-30 09:27
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>‘슈퍼오닝’ 쌀 항공방제 팔걷어</t>
+          <t>폭염이 밀어 올린 수박 값</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.kenews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>"가락시장 수수료도 안 나와"...밭에서 썩는 고랭지 배추</t>
+          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
+          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>극한 가뭄…유럽·미국에서 현실이 된 ‘물 전쟁’</t>
+          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>중국, 종자산업 지식재산권 보호 강화</t>
+          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>‘종이 농업’ 스캔들의 中 식량 안보… 베이더우 위성과 드론, 허위 보...</t>
+          <t>NH농우바이오, 8월 추천품종</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.lak.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>한수정, 글로벌 정원산업 거점화 추진</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추, 밑거름 선택이 수확을 좌우한다</t>
+          <t>‘슈퍼오닝’ 쌀 항공방제 팔걷어</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>조비, '강추' 밑거름 가을 무 ·배추 '초기 생육' 잡는다</t>
+          <t>"가락시장 수수료도 안 나와"...밭에서 썩는 고랭지 배추</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,22 +336,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.shinailbo.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>예산군, 멜론 재배에 '뒤영벌' 활용…꿀벌 부족 대응 시범사업 성과</t>
+          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -368,12 +368,12 @@
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>고추 세척기·차열막 ‘맞춤형 지원’ 호평</t>
+          <t>극한 가뭄…유럽·미국에서 현실이 된 ‘물 전쟁’</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>제주 브로콜리 ‘삼다그린’ 국산화 속도</t>
+          <t>중국, 종자산업 지식재산권 보호 강화</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>［이슈현장］홍천 내면 고랭지 채소 폐기 속출 “저장고 확충 시급”</t>
+          <t>‘종이 농업’ 스캔들의 中 식량 안보… 베이더우 위성과 드론, 허위 보...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.lak.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>미원면 양채류 재배단지, 가을작물 모종 심기 시작</t>
+          <t>한수정, 글로벌 정원산업 거점화 추진</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>한 컷으로 만나는 미래의 씨앗 생명·희망 품은 종자 , 사진에 담는다</t>
+          <t>가을 무 ·배추, 밑거름 선택이 수확을 좌우한다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
+          <t>조비, '강추' 밑거름 가을 무 ·배추 '초기 생육' 잡는다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>www.shinailbo.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>‘수출 4강’ 들겠다는 한국…바로 앞줄에 네덜란드 버틴다</t>
+          <t>예산군, 멜론 재배에 '뒤영벌' 활용…꿀벌 부족 대응 시범사업 성과</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>검역본부, 유전자변형생물체 검사 효율 높이는 신기술 개발</t>
+          <t>고추 세척기·차열막 ‘맞춤형 지원’ 호평</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월25일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>다산바이오, '혁신 프리미어 1000' 선정... AI 디지털육종 고도화</t>
+          <t>제주 브로콜리 ‘삼다그린’ 국산화 속도</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
+          <t>［이슈현장］홍천 내면 고랭지 채소 폐기 속출 “저장고 확충 시급”</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.ccdailynews.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>K-농기자재 수출 협약 373만 달러 체결</t>
+          <t>미원면 양채류 재배단지, 가을작물 모종 심기 시작</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
+          <t>한 컷으로 만나는 미래의 씨앗 생명·희망 품은 종자 , 사진에 담는다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.fntimes.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>강원특별자치도·강원농협, 농산물 가격안정 총력…소비촉진·가격보전...</t>
+          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.seoulfn.com</t>
+          <t>www.joongang.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>수박값 1년 새 36%↓···여름 과일·채소값도 안정세</t>
+          <t>‘수출 4강’ 들겠다는 한국…바로 앞줄에 네덜란드 버틴다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월26일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>마른 장마에 펄펄 끓는 남부…댐까지 말라 '물 비상'</t>
+          <t>검역본부, 유전자변형생물체 검사 효율 높이는 신기술 개발</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월25일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.wowtv.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>"작년엔 너무 비쌌는데"...여름 대표 과일 가격 '뚝'</t>
+          <t>다산바이오, '혁신 프리미어 1000' 선정... AI 디지털육종 고도화</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>LG전자 기술 이 농업 으로…농진원, 공공 기술 ·민간 기술 융합 성과 공개</t>
+          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -822,101 +822,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>가격 폭락과 폭염에 시름하는 배추 농가⋯작물 변경도 불사</t>
+          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월23일</t>
+          <t>07월24일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>www.youngnong.co.kr</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr" s="1">
-        <is>
-          <t>국립 종자 원, 제2회 종자 사진 공모전 개최…'미래의 씨앗' 담은 작품 9월...</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>07월22일</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>www.newsfreezone.co.kr</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>김장철 앞둔 종자 시장 점검…온라인 불법거래도 겨눈다</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>07월22일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>www.wonyesanup.co.kr</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>7월 채소류 농업관측</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>07월22일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -952,9 +871,6 @@
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-03 13:46
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>폭염이 밀어 올린 수박 값</t>
+          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.kenews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
+          <t>[기자의시각]] "지역이냐, 국제냐"… 종자 박람회, 행사 성격 명확히 해야</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
+          <t>작물보호협회, 최신 농약 정보 14만건 디지털 시스템 구축</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
+          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
+          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 8월 추천품종</t>
+          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -287,12 +287,12 @@
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>‘슈퍼오닝’ 쌀 항공방제 팔걷어</t>
+          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>"가락시장 수수료도 안 나와"...밭에서 썩는 고랭지 배추</t>
+          <t>“더위·병충해 강한 품종 개발 급선무”</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,22 +336,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
+          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>극한 가뭄…유럽·미국에서 현실이 된 ‘물 전쟁’</t>
+          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>08월01일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>중국, 종자산업 지식재산권 보호 강화</t>
+          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>‘종이 농업’ 스캔들의 中 식량 안보… 베이더우 위성과 드론, 허위 보...</t>
+          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.lak.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>한수정, 글로벌 정원산업 거점화 추진</t>
+          <t>아시아종묘 8월 추천 품종</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추, 밑거름 선택이 수확을 좌우한다</t>
+          <t>폭염이 밀어 올린 수박 값</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.kenews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>조비, '강추' 밑거름 가을 무 ·배추 '초기 생육' 잡는다</t>
+          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.shinailbo.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>예산군, 멜론 재배에 '뒤영벌' 활용…꿀벌 부족 대응 시범사업 성과</t>
+          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>고추 세척기·차열막 ‘맞춤형 지원’ 호평</t>
+          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>제주 브로콜리 ‘삼다그린’ 국산화 속도</t>
+          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>［이슈현장］홍천 내면 고랭지 채소 폐기 속출 “저장고 확충 시급”</t>
+          <t>NH농우바이오, 8월 추천품종</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.ccdailynews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>미원면 양채류 재배단지, 가을작물 모종 심기 시작</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>한 컷으로 만나는 미래의 씨앗 생명·희망 품은 종자 , 사진에 담는다</t>
+          <t>‘슈퍼오닝’ 쌀 항공방제 팔걷어</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
+          <t>"가락시장 수수료도 안 나와"...밭에서 썩는 고랭지 배추</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>‘수출 4강’ 들겠다는 한국…바로 앞줄에 네덜란드 버틴다</t>
+          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월26일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>검역본부, 유전자변형생물체 검사 효율 높이는 신기술 개발</t>
+          <t>극한 가뭄…유럽·미국에서 현실이 된 ‘물 전쟁’</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월25일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>다산바이오, '혁신 프리미어 1000' 선정... AI 디지털육종 고도화</t>
+          <t>중국, 종자산업 지식재산권 보호 강화</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>수입 꽃 2억 송이 육박…화훼농가 피해 우려 커져</t>
+          <t>‘종이 농업’ 스캔들의 中 식량 안보… 베이더우 위성과 드론, 허위 보...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,20 +822,101 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.lak.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>“올해도 빚만”… 배추 밭 갈아엎는 강원 고랭지 농가, 왜?</t>
+          <t>한수정, 글로벌 정원산업 거점화 추진</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월24일</t>
+          <t>07월27일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>www.newsam.co.kr</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="1">
+        <is>
+          <t>가을 무 ·배추, 밑거름 선택이 수확을 좌우한다</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>07월27일</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>www.newsfarm.co.kr</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>조비, '강추' 밑거름 가을 무 ·배추 '초기 생육' 잡는다</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>07월27일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>sjbnews.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="1">
+        <is>
+          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>07월26일</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -871,6 +952,9 @@
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-04 14:57
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
+          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[기자의시각]] "지역이냐, 국제냐"… 종자 박람회, 행사 성격 명확히 해야</t>
+          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.mtn.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>작물보호협회, 최신 농약 정보 14만건 디지털 시스템 구축</t>
+          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
+          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
+          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -216,7 +216,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
+          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
+          <t>8월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
+          <t>김장철 대박 예감! 농가가 먼저 찾는 동오시드 4대 명품 품종</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.mdilbo.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>“더위·병충해 강한 품종 개발 급선무”</t>
+          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
+          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
+          <t>[기자의시각]] "지역이냐, 국제냐"… 종자 박람회, 행사 성격 명확히 해야</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월01일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
+          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07월31일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
+          <t>작물보호협회, 최신 농약 정보 14만건 디지털 시스템 구축</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>07월31일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘 8월 추천 품종</t>
+          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>폭염이 밀어 올린 수박 값</t>
+          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.kenews.co.kr</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
+          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -530,12 +530,12 @@
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
+          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
+          <t>“더위·병충해 강한 품종 개발 급선무”</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
+          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 8월 추천품종</t>
+          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>08월01일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>‘슈퍼오닝’ 쌀 항공방제 팔걷어</t>
+          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>"가락시장 수수료도 안 나와"...밭에서 썩는 고랭지 배추</t>
+          <t>아시아종묘 8월 추천 품종</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
+          <t>폭염이 밀어 올린 수박 값</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kenews.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>극한 가뭄…유럽·미국에서 현실이 된 ‘물 전쟁’</t>
+          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>중국, 종자산업 지식재산권 보호 강화</t>
+          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>‘종이 농업’ 스캔들의 中 식량 안보… 베이더우 위성과 드론, 허위 보...</t>
+          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월28일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.lak.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>한수정, 글로벌 정원산업 거점화 추진</t>
+          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추, 밑거름 선택이 수확을 좌우한다</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월29일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,49 +876,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>조비, '강추' 밑거름 가을 무 ·배추 '초기 생육' 잡는다</t>
+          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월27일</t>
+          <t>07월28일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>sjbnews.com</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>농촌진흥청, 2026 데이터·인공지능 현장 활용 경진대회 열려</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>07월26일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -954,7 +927,6 @@
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
     <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-05 11:39
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
+          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
+          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>news.mtn.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
+          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
+          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
+          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>8월 이달의 추천품종</t>
+          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>김장철 대박 예감! 농가가 먼저 찾는 동오시드 4대 명품 품종</t>
+          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.mdilbo.com</t>
+          <t>news.mtn.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
+          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,12 +336,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
+          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -363,12 +363,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[기자의시각]] "지역이냐, 국제냐"… 종자 박람회, 행사 성격 명확히 해야</t>
+          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -378,7 +378,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -390,12 +390,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
+          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -417,12 +417,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>작물보호협회, 최신 농약 정보 14만건 디지털 시스템 구축</t>
+          <t>8월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -444,12 +444,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
+          <t>김장철 대박 예감! 농가가 먼저 찾는 동오시드 4대 명품 품종</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.mdilbo.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
+          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
+          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
+          <t>[기자의시각]] "지역이냐, 국제냐"… 종자 박람회, 행사 성격 명확히 해야</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>“더위·병충해 강한 품종 개발 급선무”</t>
+          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
+          <t>작물보호협회, 최신 농약 정보 14만건 디지털 시스템 구축</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
+          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08월01일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
+          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07월31일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
+          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07월31일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘 8월 추천 품종</t>
+          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>폭염이 밀어 올린 수박 값</t>
+          <t>“더위·병충해 강한 품종 개발 급선무”</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.kenews.co.kr</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
+          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
+          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월01일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
+          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
+          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>아시아종묘 8월 추천 품종</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,22 +876,157 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>www.newsis.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>수박 가격 급등</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>07월30일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>www.kenews.co.kr</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="1">
+        <is>
+          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>07월30일</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>www.nongmin.com</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="1">
+        <is>
+          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>07월30일</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>www.donga.com</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>07월30일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>www.youngnong.co.kr</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>농진원, 농약공정분석방법 고도화 추진…유통 농약 품질관리 신뢰성 높...</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>07월28일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>한국농업기술진흥원</t>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>07월29일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>www.wonyesanup.co.kr</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="1">
+        <is>
+          <t>신기술 &amp; 새상품</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>07월29일</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -927,6 +1062,11 @@
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
     <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
+    <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-06 13:32
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.joongang.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
+          <t>스테비아 토마토 , ‘천연 감미료’ 둔갑 판매 광고한 업체 15곳 적발</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.sedaily.com</t>
+          <t>www.munhwa.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
+          <t>“37도 넘는데 밭일하면 안돼요”…드론 띄워 ‘농민 지키기’</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.knnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
+          <t>유럽 폭염에 남해 시금치 농가 비상</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.insight.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
+          <t>폭염 여파로 채소값 급등... 오이 59%·애호박 47% '껑충'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.mhns.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>[박근종 칼럼] 소비자물가 석달 만에 2%대 복귀, '히트플레이션' 충격 최...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
+          <t>' 당근 플레이션' 오나?...폭염·가뭄에 제주 당근 비상</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
+          <t>병해엔 강하고 맛은 높였다…NH농우바이오, 가을 재배 겨냥 8월 추천 품...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
+          <t>예천군, '젤리킹' 여왕벌 보급 확대…양봉 경쟁력 강화</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>news.mtn.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
+          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
+          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
+          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
+          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>8월 이달의 추천품종</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>김장철 대박 예감! 농가가 먼저 찾는 동오시드 4대 명품 품종</t>
+          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.mdilbo.com</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
+          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
+          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.mtn.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[기자의시각]] "지역이냐, 국제냐"… 종자 박람회, 행사 성격 명확히 해야</t>
+          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
+          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>작물보호협회, 최신 농약 정보 14만건 디지털 시스템 구축</t>
+          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
+          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
+          <t>8월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.mdilbo.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
+          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.samdailbo.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
+          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>“더위·병충해 강한 품종 개발 급선무”</t>
+          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
+          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
+          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08월01일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
+          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07월31일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.jeollailbo.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
+          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07월31일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘 8월 추천 품종</t>
+          <t>“더위·병충해 강한 품종 개발 급선무”</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>수박 가격 급등</t>
+          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월02일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.kenews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>대아청과, "고랭지 무 산지작황 양호"...출하 청신호!</t>
+          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>08월01일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>속타는 여름무 산지…이상기후·공급 증가 겹쳐 생산기반 ‘흔들’</t>
+          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>폭염에 가뭄 겹쳐 강으로 바닷물 역류 “수돗물서 짠맛 난다”</t>
+          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>07월30일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,47 +984,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>가을 무 ·배추 수확량, 밑거름이 좌우한다…조비, 맞춤형 비료 3종 제안</t>
+          <t>아시아종묘 8월 추천 품종</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>07월29일</t>
+          <t>07월30일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.wonyesanup.co.kr</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>신기술 &amp; 새상품</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>07월29일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1066,7 +1039,6 @@
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
     <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-10 09:36
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>www.headlinejeju.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>스테비아 토마토 , ‘천연 감미료’ 둔갑 판매 광고한 업체 15곳 적발</t>
+          <t>[종합] 비는 찔끔, 농심은 애타고… 당근 파종은 더욱 바빠졌다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.munhwa.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>“37도 넘는데 밭일하면 안돼요”…드론 띄워 ‘농민 지키기’</t>
+          <t>고랭지 배추 작황 호조...저장 배추 방출이 시세하락 '주범'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.knnews.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>유럽 폭염에 남해 시금치 농가 비상</t>
+          <t>CPTPP 문턱서 커지는 '후쿠시마 수산물' 개방 압력 [수출과 식량주권 사...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.insight.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>폭염 여파로 채소값 급등... 오이 59%·애호박 47% '껑충'</t>
+          <t>우장춘 박사 67주기, 후손 방한…추모에서 한일 원예 산업 교류로</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월09일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.mhns.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>[박근종 칼럼] 소비자물가 석달 만에 2%대 복귀, '히트플레이션' 충격 최...</t>
+          <t>폭염에 시금치· 열무 ·상추 출하량 '뚝'…채소값 급등</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월09일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>' 당근 플레이션' 오나?...폭염·가뭄에 제주 당근 비상</t>
+          <t>김장 채소 파종기, 재배 안정성·복합 내병성 챙기세요</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월07일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>병해엔 강하고 맛은 높였다…NH농우바이오, 가을 재배 겨냥 8월 추천 품...</t>
+          <t>NH농우바이오, 8월 추천 품종</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월07일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.joongang.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>예천군, '젤리킹' 여왕벌 보급 확대…양봉 경쟁력 강화</t>
+          <t>스테비아 토마토 , ‘천연 감미료’ 둔갑 판매 광고한 업체 15곳 적발</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.munhwa.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
+          <t>“37도 넘는데 밭일하면 안돼요”…드론 띄워 ‘농민 지키기’</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.sedaily.com</t>
+          <t>www.knnews.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
+          <t>유럽 폭염에 남해 시금치 농가 비상</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.insight.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
+          <t>폭염 여파로 채소값 급등... 오이 59%·애호박 47% '껑충'</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.mhns.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
+          <t>[박근종 칼럼] 소비자물가 석달 만에 2%대 복귀, '히트플레이션' 충격 최...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>' 당근 플레이션' 오나?...폭염·가뭄에 제주 당근 비상</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
+          <t>예천군, '젤리킹' 여왕벌 보급 확대…양봉 경쟁력 강화</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
+          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
+          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>news.mtn.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
+          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
+          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
+          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>8월 이달의 추천품종</t>
+          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.mdilbo.com</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
+          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.samdailbo.com</t>
+          <t>news.mtn.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>가뭄에 당근 파종 차질..."복합기후재난 대응체계 필요"</t>
+          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>[현장] 소비 부진에 저장무 출하 겹쳐…여름무 농가 '시름'</t>
+          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>李 대통령 “한·칠레 FTA 현대화”…농산물 추가 개방 촉각</t>
+          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>"갓 딴 상추 도 시들어 팔기가…" 42.5도 찍은 양산, 시장 상인들의 한숨...</t>
+          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>'농장에서 일하는 AI 로봇'…충북도, 스마트팜 휴머노이드 기술 개발 박...</t>
+          <t>8월 이달의 추천품종</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.mdilbo.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>‘키 크는 쌀’ ‘비만 잡는 고추’…기능성 품종 “눈에 띄네”</t>
+          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>“더위·병충해 강한 품종 개발 급선무”</t>
+          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
+          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,101 +903,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.jeollailbo.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>심하면 배추 전체를 썩게 만드는 ‘무름병’</t>
+          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08월01일</t>
+          <t>07월31일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>www.agrinet.co.kr</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="1">
-        <is>
-          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>07월31일</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.jeollailbo.com</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>07월31일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.newsam.co.kr</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>아시아종묘 8월 추천 품종</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>07월30일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1036,9 +955,6 @@
     <hyperlink ref="C30" r:id="rId29"/>
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-11 09:52
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>tjmbc.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[종합] 비는 찔끔, 농심은 애타고… 당근 파종은 더욱 바빠졌다</t>
+          <t>[리포트]잎채소 물러지고 고추는 탄저병⋯번지는 농작물 피해</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>고랭지 배추 작황 호조...저장 배추 방출이 시세하락 '주범'</t>
+          <t>0.2mm '찔끔비'‥논바닥도 농심도 "쩍쩍 갈라져"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>CPTPP 문턱서 커지는 '후쿠시마 수산물' 개방 압력 [수출과 식량주권 사...</t>
+          <t>﻿[AI로 읽는 경제] ﻿② 밭 전체에 농약 뿌리던 시대 끝난다…AI 농업의...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>우장춘 박사 67주기, 후손 방한…추모에서 한일 원예 산업 교류로</t>
+          <t>'바이킹 후예' 노르웨이, 농수산물 '수확 후 관리공학' 최고인 이유</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월09일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>폭염에 시금치· 열무 ·상추 출하량 '뚝'…채소값 급등</t>
+          <t>고창군, 농작물재해보험 ‘가을배추’ 신규 가입</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월09일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>김장 채소 파종기, 재배 안정성·복합 내병성 챙기세요</t>
+          <t>“밖은 42℃, 안은 29℃"…가락시장, 농산물 신선도 유지 ‘안간힘’</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월07일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 8월 추천 품종</t>
+          <t>국산 주황색 미니단호박 제농 '황금미니단호박', 뛰어난 식미와 높은 수...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월07일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>www.lecturernews.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>스테비아 토마토 , ‘천연 감미료’ 둔갑 판매 광고한 업체 15곳 적발</t>
+          <t>경기도농업기술원, 꿀벌 질병 대응·봉군 관리 기술 전수 '양봉농가 대...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.munhwa.com</t>
+          <t>www.headlinejeju.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>“37도 넘는데 밭일하면 안돼요”…드론 띄워 ‘농민 지키기’</t>
+          <t>[종합] 비는 찔끔, 농심은 애타고… 당근 파종은 더욱 바빠졌다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.knnews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>유럽 폭염에 남해 시금치 농가 비상</t>
+          <t>고랭지 배추 작황 호조...저장 배추 방출이 시세하락 '주범'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.insight.co.kr</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>폭염 여파로 채소값 급등... 오이 59%·애호박 47% '껑충'</t>
+          <t>CPTPP 문턱서 커지는 '후쿠시마 수산물' 개방 압력 [수출과 식량주권 사...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.mhns.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>[박근종 칼럼] 소비자물가 석달 만에 2%대 복귀, '히트플레이션' 충격 최...</t>
+          <t>우장춘 박사 67주기, 후손 방한…추모에서 한일 원예 산업 교류로</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월09일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>' 당근 플레이션' 오나?...폭염·가뭄에 제주 당근 비상</t>
+          <t>폭염에 시금치· 열무 ·상추 출하량 '뚝'…채소값 급등</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월09일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>예천군, '젤리킹' 여왕벌 보급 확대…양봉 경쟁력 강화</t>
+          <t>김장 채소 파종기, 재배 안정성·복합 내병성 챙기세요</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월07일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
+          <t>NH농우바이오, 8월 추천 품종</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월07일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.sedaily.com</t>
+          <t>www.joongang.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
+          <t>스테비아 토마토 , ‘천연 감미료’ 둔갑 판매 광고한 업체 15곳 적발</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.munhwa.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
+          <t>“37도 넘는데 밭일하면 안돼요”…드론 띄워 ‘농민 지키기’</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.knnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
+          <t>유럽 폭염에 남해 시금치 농가 비상</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.insight.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>폭염 여파로 채소값 급등... 오이 59%·애호박 47% '껑충'</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.mhns.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
+          <t>[박근종 칼럼] 소비자물가 석달 만에 2%대 복귀, '히트플레이션' 충격 최...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>진안고원 마이산 고추 시장 8월 4일 개장…생산농가 직거래 운영</t>
+          <t>' 당근 플레이션' 오나?...폭염·가뭄에 제주 당근 비상</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월06일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>7월 물가 2.8%↑, 석달 만에 2%대로…유가·농산물 둔화 영향(상보)</t>
+          <t>예천군, '젤리킹' 여왕벌 보급 확대…양봉 경쟁력 강화</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>news.mtn.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>연이은 폭염에 장바구니 '비상'… 시금치 가격, 한 달 만에 두 배 올라</t>
+          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>"물러서 폭삭" 썩고 악취 진동…없던 병까지 생겼다</t>
+          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월05일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>누가 더 최적의 재배환경 만드나…농진원, 스마트팜 AI 경진대회 개최</t>
+          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
+          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>8월 이달의 추천품종</t>
+          <t>주간농사정보</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.mdilbo.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>‘무등산 수박’ 부흥 기회 만든 공무원 떠나자 농민들 “명맥 유지 안...</t>
+          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08월03일</t>
+          <t>08월04일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,74 +849,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>‘환상’ 너머 현실로… 中, 과학기술 기반 곡물 초고수확량 시대 진입</t>
+          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08월02일</t>
+          <t>08월03일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>www.agrinet.co.kr</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>'중국산 양상추' 파상공세···여름철 국산 수급 공백 틈 노린다</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>07월31일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>www.jeollailbo.com</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>국립 종자 원 전북지원, 불법 씨앗·모종 유통 조사</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>07월31일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -953,8 +899,6 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-13 10:37
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tjmbc.co.kr</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[리포트]잎채소 물러지고 고추는 탄저병⋯번지는 농작물 피해</t>
+          <t>폭염·고수온에 밥상물가 비상…정부, 농축수산 물 수급 총력 대응</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>kjmbc.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>0.2mm '찔끔비'‥논바닥도 농심도 "쩍쩍 갈라져"</t>
+          <t>장성호 저수율 27%... 말라가는 농작물에 농민들 마음도 '쩍쩍'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>﻿[AI로 읽는 경제] ﻿② 밭 전체에 농약 뿌리던 시대 끝난다…AI 농업의...</t>
+          <t>영광군, 콩 개화기 병해충 증가 우려…노린재·나방류 예찰 강화 당부</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -179,12 +179,12 @@
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>'바이킹 후예' 노르웨이, 농수산물 '수확 후 관리공학' 최고인 이유</t>
+          <t>아시아 15개국 종자 전문가 서울 집결…품종보호 협력 논의</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>고창군, 농작물재해보험 ‘가을배추’ 신규 가입</t>
+          <t>아시아 종묘 , 청송 고추 농가 80여명에 품종 경쟁력 소개</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.betanews.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>“밖은 42℃, 안은 29℃"…가락시장, 농산물 신선도 유지 ‘안간힘’</t>
+          <t>전남광주 저탄소 농산물 인증면적 7810㏊…전국 36%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>국산 주황색 미니단호박 제농 '황금미니단호박', 뛰어난 식미와 높은 수...</t>
+          <t>토종 '풀·꽃·나무'를 우리곁에… 전국 확산 팔걷은 농식품부</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.lecturernews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 꿀벌 질병 대응·봉군 관리 기술 전수 '양봉농가 대...</t>
+          <t>농사포인트 - 기온 31℃ 이상일 때, 과실에 직사광선 노출 예상될 때 미...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.headlinejeju.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[종합] 비는 찔끔, 농심은 애타고… 당근 파종은 더욱 바빠졌다</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>고랭지 배추 작황 호조...저장 배추 방출이 시세하락 '주범'</t>
+          <t>폭염 견딘 안반데기 배추밭…농촌진흥청장 직접 찾아 점검</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.mhns.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>CPTPP 문턱서 커지는 '후쿠시마 수산물' 개방 압력 [수출과 식량주권 사...</t>
+          <t>경북도, 폭염으로 인한 고추 응애 발생 주의</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.abcn.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>우장춘 박사 67주기, 후손 방한…추모에서 한일 원예 산업 교류로</t>
+          <t>폭염 시대, 30년 뒤에도 여름에 수박을 먹을 수 있을까?</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월09일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.jndn.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>폭염에 시금치· 열무 ·상추 출하량 '뚝'…채소값 급등</t>
+          <t>마라탕 유행에 ‘녹두’ 인기…기계수확 품종 ‘채흔’ 주목</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월09일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.getnews.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>김장 채소 파종기, 재배 안정성·복합 내병성 챙기세요</t>
+          <t>폭염에 시금치가 '시金치'로... 8월 채소류 가격 급등에 '히트플레이션...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월07일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>tjmbc.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 8월 추천 품종</t>
+          <t>[리포트]잎채소 물러지고 고추는 탄저병⋯번지는 농작물 피해</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월07일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.joongang.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>스테비아 토마토 , ‘천연 감미료’ 둔갑 판매 광고한 업체 15곳 적발</t>
+          <t>0.2mm '찔끔비'‥논바닥도 농심도 "쩍쩍 갈라져"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.munhwa.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>“37도 넘는데 밭일하면 안돼요”…드론 띄워 ‘농민 지키기’</t>
+          <t>﻿[AI로 읽는 경제] ﻿② 밭 전체에 농약 뿌리던 시대 끝난다…AI 농업의...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.knnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>유럽 폭염에 남해 시금치 농가 비상</t>
+          <t>'바이킹 후예' 노르웨이, 농수산물 '수확 후 관리공학' 최고인 이유</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.insight.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>폭염 여파로 채소값 급등... 오이 59%·애호박 47% '껑충'</t>
+          <t>고창군, 농작물재해보험 ‘가을배추’ 신규 가입</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.mhns.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>[박근종 칼럼] 소비자물가 석달 만에 2%대 복귀, '히트플레이션' 충격 최...</t>
+          <t>“밖은 42℃, 안은 29℃"…가락시장, 농산물 신선도 유지 ‘안간힘’</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>' 당근 플레이션' 오나?...폭염·가뭄에 제주 당근 비상</t>
+          <t>국산 주황색 미니단호박 제농 '황금미니단호박', 뛰어난 식미와 높은 수...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08월06일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.lecturernews.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>예천군, '젤리킹' 여왕벌 보급 확대…양봉 경쟁력 강화</t>
+          <t>경기도농업기술원, 꿀벌 질병 대응·봉군 관리 기술 전수 '양봉농가 대...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -692,12 +692,12 @@
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>국립종자원 충남지원, 김장용 종자·묘 불법유통 단속 나서</t>
+          <t>고랭지 배추 작황 호조...저장 배추 방출이 시세하락 '주범'</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.sedaily.com</t>
+          <t>www.etoday.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>폭염에 병해충 비상…경기농기원 “수확기 선제 방제해야”</t>
+          <t>CPTPP 문턱서 커지는 '후쿠시마 수산물' 개방 압력 [수출과 식량주권 사...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08월05일</t>
+          <t>08월10일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>'불가마' 대한민국···가락시장 농산물 관리도 비상</t>
+          <t>우장춘 박사 67주기, 후손 방한…추모에서 한일 원예 산업 교류로</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월09일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.jndn.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>영양서 '고추 품종평가회' 개최…우량 품종 한자리 비교</t>
+          <t>폭염에 시금치· 열무 ·상추 출하량 '뚝'…채소값 급등</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월09일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>주간농사정보</t>
+          <t>김장 채소 파종기, 재배 안정성·복합 내병성 챙기세요</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월07일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,47 +822,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>동오시드, 안정성 갖춘 김장채소 품종 '눈길'</t>
+          <t>NH농우바이오, 8월 추천 품종</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08월04일</t>
+          <t>08월07일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>www.kado.net</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr" s="1">
-        <is>
-          <t>정선 고랭지 풋고추 '제값 받기' 나섰다</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>08월03일</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -898,7 +871,6 @@
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-18 18:14
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>폭염·고수온에 밥상물가 비상…정부, 농축수산 물 수급 총력 대응</t>
+          <t>남부지방 폭우 피해신고 2500건 넘어…사망 1명·부상 4명 추가 없어</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월18일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>kjmbc.co.kr</t>
+          <t>www.namdonews.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>장성호 저수율 27%... 말라가는 농작물에 농민들 마음도 '쩍쩍'</t>
+          <t>보성 무농약 참다래, 8월 친환경농산물 선정</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월18일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.m-i.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>영광군, 콩 개화기 병해충 증가 우려…노린재·나방류 예찰 강화 당부</t>
+          <t>해남·진도 배추밭 400㏊ 줄인다… 작목 전환에 18억원 지원</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월18일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>아시아 15개국 종자 전문가 서울 집결…품종보호 협력 논의</t>
+          <t>기능성 강화한 상추 신품종 '고진미'·'노을쌈' 개발</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월18일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.inews365.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>아시아 종묘 , 청송 고추 농가 80여명에 품종 경쟁력 소개</t>
+          <t>배추 키우고 AI로 판다…옥천 농업인 교육 10개 과정 운영</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월17일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.betanews.net</t>
+          <t>www.kbsm.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>전남광주 저탄소 농산물 인증면적 7810㏊…전국 36%</t>
+          <t>예천군, ‘젤리킹’ 여왕벌 325마리 보급…물량 1년 새 3.6배 늘어</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월17일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.seongjuro.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>토종 '풀·꽃·나무'를 우리곁에… 전국 확산 팔걷은 농식품부</t>
+          <t>2026 하반기 종자 ·묘 유통조사 실시</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월14일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 기온 31℃ 이상일 때, 과실에 직사광선 노출 예상될 때 미...</t>
+          <t>품종보호, 지속가능한 종자산업 뒷받침…아시아·태평양 지역 권리보호...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월14일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.ajunews.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>폭염·고수온에 수산 물 수급 안정 총력</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.imaeil.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>폭염 견딘 안반데기 배추밭…농촌진흥청장 직접 찾아 점검</t>
+          <t>폭염·고수온에 밥상물가 비상…정부, 농축수산 물 수급 총력 대응</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.mhns.co.kr</t>
+          <t>kjmbc.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>경북도, 폭염으로 인한 고추 응애 발생 주의</t>
+          <t>장성호 저수율 27%... 말라가는 농작물에 농민들 마음도 '쩍쩍'</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.abcn.kr</t>
+          <t>www.newsmaker.or.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>폭염 시대, 30년 뒤에도 여름에 수박을 먹을 수 있을까?</t>
+          <t>영광군, 콩 개화기 병해충 증가 우려…노린재·나방류 예찰 강화 당부</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월13일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,12 +417,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>마라탕 유행에 ‘녹두’ 인기…기계수확 품종 ‘채흔’ 주목</t>
+          <t>아시아 종묘 , 청송 고추 농가 80여명에 품종 경쟁력 소개</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -432,7 +432,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.getnews.co.kr</t>
+          <t>www.betanews.net</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>폭염에 시금치가 '시金치'로... 8월 채소류 가격 급등에 '히트플레이션...</t>
+          <t>전남광주 저탄소 농산물 인증면적 7810㏊…전국 36%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tjmbc.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>[리포트]잎채소 물러지고 고추는 탄저병⋯번지는 농작물 피해</t>
+          <t>토종 '풀·꽃·나무'를 우리곁에… 전국 확산 팔걷은 농식품부</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>0.2mm '찔끔비'‥논바닥도 농심도 "쩍쩍 갈라져"</t>
+          <t>농사포인트 - 기온 31℃ 이상일 때, 과실에 직사광선 노출 예상될 때 미...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>﻿[AI로 읽는 경제] ﻿② 밭 전체에 농약 뿌리던 시대 끝난다…AI 농업의...</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.news1.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>'바이킹 후예' 노르웨이, 농수산물 '수확 후 관리공학' 최고인 이유</t>
+          <t>폭염 견딘 안반데기 배추밭…농촌진흥청장 직접 찾아 점검</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월11일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.mhns.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>고창군, 농작물재해보험 ‘가을배추’ 신규 가입</t>
+          <t>경북도, 폭염으로 인한 고추 응애 발생 주의</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.abcn.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>“밖은 42℃, 안은 29℃"…가락시장, 농산물 신선도 유지 ‘안간힘’</t>
+          <t>폭염 시대, 30년 뒤에도 여름에 수박을 먹을 수 있을까?</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>국산 주황색 미니단호박 제농 '황금미니단호박', 뛰어난 식미와 높은 수...</t>
+          <t>마라탕 유행에 ‘녹두’ 인기…기계수확 품종 ‘채흔’ 주목</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월12일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.lecturernews.com</t>
+          <t>www.getnews.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>경기도농업기술원, 꿀벌 질병 대응·봉군 관리 기술 전수 '양봉농가 대...</t>
+          <t>폭염에 시금치가 '시金치'로... 8월 채소류 가격 급등에 '히트플레이션...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08월10일</t>
+          <t>08월11일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>고랭지 배추 작황 호조...저장 배추 방출이 시세하락 '주범'</t>
+          <t>고창군, 농작물재해보험 ‘가을배추’ 신규 가입</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.etoday.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>CPTPP 문턱서 커지는 '후쿠시마 수산물' 개방 압력 [수출과 식량주권 사...</t>
+          <t>“밖은 42℃, 안은 29℃"…가락시장, 농산물 신선도 유지 ‘안간힘’</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -728,114 +728,6 @@
         </is>
       </c>
       <c r="E25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>sjbnews.com</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr" s="1">
-        <is>
-          <t>우장춘 박사 67주기, 후손 방한…추모에서 한일 원예 산업 교류로</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>08월09일</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>www.jndn.com</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr" s="1">
-        <is>
-          <t>폭염에 시금치· 열무 ·상추 출하량 '뚝'…채소값 급등</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>08월09일</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>www.agrinet.co.kr</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr" s="1">
-        <is>
-          <t>김장 채소 파종기, 재배 안정성·복합 내병성 챙기세요</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>08월07일</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>www.farmnmarket.com</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr" s="1">
-        <is>
-          <t>NH농우바이오, 8월 추천 품종</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>08월07일</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -867,10 +759,6 @@
     <hyperlink ref="C23" r:id="rId22"/>
     <hyperlink ref="C24" r:id="rId23"/>
     <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
-    <hyperlink ref="C27" r:id="rId26"/>
-    <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>